<commit_message>
added some dataanalysis to be removed at the end
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4E7FB2-1CAC-4FA4-91DD-590DC3CE59E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B36FFC-F06F-4FD0-9CAE-5B4BD3B9BA46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
     <sheet name="Parameters" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -858,7 +858,7 @@
   <dimension ref="A1:R49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="1" max="1" width="55.88671875" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" customWidth="1"/>

</xml_diff>

<commit_message>
Implementing dataanalysis of xarray containing mapped variables
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B36FFC-F06F-4FD0-9CAE-5B4BD3B9BA46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7EFCA8-115B-465F-B417-9FB7AD3D37A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -859,7 +859,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.88671875" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.21875" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="13.77734375" customWidth="1"/>
     <col min="6" max="6" width="17.109375" customWidth="1"/>

</xml_diff>

<commit_message>
assign transport activities according to the decision tree
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD434366-C89D-4D33-A3BE-D509CC2B5F6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8414FC-1405-4F9C-8A66-41FC458B3A88}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
-    <sheet name="ship" sheetId="3" r:id="rId2"/>
-    <sheet name="Parameters" sheetId="2" r:id="rId3"/>
+    <sheet name="hydrogen-transport (2)" sheetId="4" r:id="rId2"/>
+    <sheet name="ship" sheetId="3" r:id="rId3"/>
+    <sheet name="Parameters" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="169">
   <si>
     <t>Database</t>
   </si>
@@ -472,33 +473,6 @@
     <t>C. Wulf et al. / Journal of Cleaner Production 199 (2018) 431-443</t>
   </si>
   <si>
-    <t>Car db</t>
-  </si>
-  <si>
-    <t>ecoinvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transport, gaseous hydrogen, lorry </t>
-  </si>
-  <si>
-    <t>market for hydrogen</t>
-  </si>
-  <si>
-    <t>hydrogen, gaseous</t>
-  </si>
-  <si>
-    <t>market for electricity</t>
-  </si>
-  <si>
-    <t>transport, gaseous hydrogen, lorry, market average propulsion system</t>
-  </si>
-  <si>
-    <t>transport, liquid hydrogen, lorry, market average propulsion system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transport, liquid hydrogen, lorry </t>
-  </si>
-  <si>
     <t>LCI for gaseous hydrogen transport for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Lorry is market average. Boil-off losses are 0.5 % and 0.5 % during compression (Reuß et al. 2019)</t>
   </si>
   <si>
@@ -508,9 +482,6 @@
     <t>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</t>
   </si>
   <si>
-    <t>kWh</t>
-  </si>
-  <si>
     <t>electricity, medium voltage</t>
   </si>
   <si>
@@ -539,6 +510,45 @@
   </si>
   <si>
     <t>air</t>
+  </si>
+  <si>
+    <t>market for hydrogen, gaseous, low pressure</t>
+  </si>
+  <si>
+    <t>hydrogen, gaseous, low pressure</t>
+  </si>
+  <si>
+    <t>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry, market average propulsion system</t>
+  </si>
+  <si>
+    <t>this dataset is used as a proxy</t>
+  </si>
+  <si>
+    <t>market for electricity, medium voltage</t>
+  </si>
+  <si>
+    <t>LCI for hydrogen transport as liquid ammonia for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Market average. Boil-off losses are 3 % and 1.65 % during liquefaction (Reuß et al. 2019)</t>
+  </si>
+  <si>
+    <t>LCI for liquid hydrogen transport for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Ship is market average. Boil-off losses are 3 % and 1.65 % during liquefaction (Reuß et al. 2019)</t>
+  </si>
+  <si>
+    <t>kilowatt hour</t>
+  </si>
+  <si>
+    <t>RER</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry , market average propulsion system</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, liquid, lorry, market average propulsion system</t>
+  </si>
+  <si>
+    <t>DE</t>
   </si>
 </sst>
 </file>
@@ -943,663 +953,821 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="3" max="3" width="33.21875" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
     <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="12" max="12" width="13.21875" customWidth="1"/>
-    <col min="13" max="13" width="43.88671875" customWidth="1"/>
-    <col min="14" max="14" width="13.33203125" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B1" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="str">
+        <f>B6</f>
+        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+      </c>
+      <c r="B12">
+        <f>B5</f>
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" t="str">
+        <f>A12</f>
+        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" t="s">
+        <v>151</v>
+      </c>
+      <c r="I13" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14">
+        <f>1*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>157</v>
+      </c>
+      <c r="I15" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" t="s">
+        <v>155</v>
+      </c>
+      <c r="F16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>141</v>
       </c>
-      <c r="B6">
+      <c r="B20">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="str">
+        <f>B21</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+      <c r="B27">
+        <f>B20</f>
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="str">
+        <f>A27</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28">
+        <v>1000</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" t="s">
+        <v>140</v>
+      </c>
+      <c r="I28" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B29">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="C29" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" t="s">
+        <v>157</v>
+      </c>
+      <c r="I29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>161</v>
+      </c>
+      <c r="B30">
+        <f>1000*6.78</f>
+        <v>6780</v>
+      </c>
+      <c r="C30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D30" t="s">
+        <v>164</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>146</v>
+      </c>
+      <c r="I30" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31">
+        <v>0.6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>168</v>
+      </c>
+      <c r="D31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" t="s">
+        <v>146</v>
+      </c>
+      <c r="I31" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="str">
-        <f>B7</f>
-        <v xml:space="preserve">transport, gaseous hydrogen, lorry </v>
-      </c>
-      <c r="B13">
-        <f>B6</f>
-        <v>1</v>
-      </c>
-      <c r="C13" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D13" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>160</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>144</v>
-      </c>
-      <c r="D14" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" t="s">
-        <v>18</v>
-      </c>
-      <c r="I14" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15">
-        <v>1200</v>
-      </c>
-      <c r="C15" t="s">
-        <v>144</v>
-      </c>
-      <c r="D15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="B32">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="D32" t="s">
         <v>26</v>
-      </c>
-      <c r="G15" t="s">
-        <v>18</v>
-      </c>
-      <c r="I15" t="s">
-        <v>140</v>
-      </c>
-      <c r="J15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B16">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C16" t="s">
-        <v>144</v>
-      </c>
-      <c r="D16" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I16" t="s">
-        <v>147</v>
-      </c>
-      <c r="J16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>162</v>
-      </c>
-      <c r="B17">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" t="s">
-        <v>165</v>
-      </c>
-      <c r="G17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" t="s">
-        <v>23</v>
-      </c>
-      <c r="G27" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" t="s">
-        <v>15</v>
-      </c>
-      <c r="J27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" t="str">
-        <f>B22</f>
-        <v xml:space="preserve">transport, liquid hydrogen, lorry </v>
-      </c>
-      <c r="B28">
-        <f>B21</f>
-        <v>1</v>
-      </c>
-      <c r="C28" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D28" t="s">
-        <v>8</v>
-      </c>
-      <c r="E28" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>140</v>
-      </c>
-      <c r="B29">
-        <v>4300</v>
-      </c>
-      <c r="C29" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" t="s">
-        <v>8</v>
-      </c>
-      <c r="E29" t="s">
-        <v>26</v>
-      </c>
-      <c r="G29" t="s">
-        <v>18</v>
-      </c>
-      <c r="I29" t="s">
-        <v>140</v>
-      </c>
-      <c r="J29" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B30">
-        <v>1.6250000000000001E-2</v>
-      </c>
-      <c r="C30" t="s">
-        <v>144</v>
-      </c>
-      <c r="D30" t="s">
-        <v>8</v>
-      </c>
-      <c r="E30" t="s">
-        <v>26</v>
-      </c>
-      <c r="G30" t="s">
-        <v>18</v>
-      </c>
-      <c r="I30" t="s">
-        <v>147</v>
-      </c>
-      <c r="J30" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>148</v>
-      </c>
-      <c r="B31">
-        <v>6.78</v>
-      </c>
-      <c r="C31" t="s">
-        <v>144</v>
-      </c>
-      <c r="D31" t="s">
-        <v>8</v>
-      </c>
-      <c r="E31" t="s">
-        <v>155</v>
-      </c>
-      <c r="G31" t="s">
-        <v>18</v>
-      </c>
-      <c r="I31" t="s">
-        <v>156</v>
-      </c>
-      <c r="J31" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>148</v>
-      </c>
-      <c r="B32">
-        <v>0.6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" t="s">
-        <v>8</v>
       </c>
       <c r="E32" t="s">
         <v>155</v>
       </c>
-      <c r="G32" t="s">
-        <v>18</v>
-      </c>
-      <c r="I32" t="s">
-        <v>156</v>
-      </c>
-      <c r="J32" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>162</v>
-      </c>
-      <c r="B33">
-        <v>1.6250000000000001E-2</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="F32" t="s">
         <v>27</v>
       </c>
-      <c r="E33" t="s">
-        <v>26</v>
-      </c>
-      <c r="F33" t="s">
-        <v>165</v>
-      </c>
-      <c r="G33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+    </row>
+    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B34" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>141</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>6</v>
+      </c>
+      <c r="B40" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
         <v>7</v>
       </c>
-      <c r="B36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="D42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
         <v>15</v>
-      </c>
-      <c r="B38" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="H42" t="s">
         <v>20</v>
       </c>
       <c r="I42" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="str">
+        <f>B37</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B43">
+        <f>B36</f>
+        <v>1</v>
+      </c>
+      <c r="C43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" t="s">
+        <v>17</v>
+      </c>
+      <c r="G43" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44">
+        <f>1000*1</f>
+        <v>1000</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>26</v>
+      </c>
+      <c r="F44" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B45">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>153</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>141</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>15</v>
       </c>
-      <c r="J42" t="s">
+      <c r="B51" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>14</v>
+      </c>
+      <c r="B52" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="B54" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
         <v>11</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B56" t="s">
         <v>12</v>
       </c>
-      <c r="C43" t="s">
-        <v>13</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C56" t="s">
         <v>7</v>
       </c>
-      <c r="E43" t="s">
+      <c r="D56" t="s">
         <v>14</v>
       </c>
-      <c r="F43" t="s">
+      <c r="E56" t="s">
         <v>23</v>
       </c>
-      <c r="G43" t="s">
+      <c r="F56" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>B38</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
-      </c>
-      <c r="B44">
-        <f>B37</f>
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="str">
+        <f>B51</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B57">
+        <f>B50</f>
         <v>1</v>
       </c>
-      <c r="C44" t="str">
-        <f>B2</f>
-        <v>hydrogen-transport</v>
-      </c>
-      <c r="D44" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" t="s">
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
         <v>16</v>
       </c>
-      <c r="G44" t="s">
+      <c r="F57" t="s">
         <v>17</v>
       </c>
-      <c r="I44" t="s">
+      <c r="G57" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>26</v>
+      </c>
+      <c r="F58" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B59">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>165</v>
+      </c>
+      <c r="D59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>153</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>16</v>
+      </c>
+      <c r="F60" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>140</v>
-      </c>
-      <c r="B45">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>143</v>
-      </c>
-      <c r="D45" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" t="s">
-        <v>26</v>
-      </c>
-      <c r="G45" t="s">
-        <v>18</v>
-      </c>
-      <c r="I45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B46">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C46" t="s">
-        <v>144</v>
-      </c>
-      <c r="D46" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" t="s">
-        <v>26</v>
-      </c>
-      <c r="G46" t="s">
-        <v>18</v>
-      </c>
-      <c r="I46" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>163</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>144</v>
-      </c>
-      <c r="D47" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" t="s">
-        <v>18</v>
-      </c>
-      <c r="I47" t="s">
-        <v>164</v>
-      </c>
+    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+    </row>
+    <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1"/>
+    </row>
+    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
+    </row>
+    <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+    </row>
+    <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+      <c r="G75" s="4"/>
+    </row>
+    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
+    </row>
+    <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1608,392 +1776,1179 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFCFE87B-D030-4AA0-99E6-3DBA7D6E9B67}">
+  <dimension ref="A1:I81"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="82.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="13.77734375" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" customWidth="1"/>
+    <col min="11" max="11" width="13.21875" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="str">
+        <f>B7</f>
+        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
+      </c>
+      <c r="B13">
+        <f>B6</f>
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" t="str">
+        <f>A13</f>
+        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" t="s">
+        <v>151</v>
+      </c>
+      <c r="I14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15">
+        <f>1*1000</f>
+        <v>1000</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
+        <v>157</v>
+      </c>
+      <c r="I16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17">
+        <f>1000*0.005</f>
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+      <c r="I27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f>B22</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+      <c r="B28">
+        <f>B21</f>
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>16</v>
+      </c>
+      <c r="F28" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" t="str">
+        <f>A28</f>
+        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>140</v>
+      </c>
+      <c r="B29">
+        <v>1000</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" t="s">
+        <v>140</v>
+      </c>
+      <c r="I29" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B30">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>157</v>
+      </c>
+      <c r="I30" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31">
+        <f>1000*6.78</f>
+        <v>6780</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
+        <v>164</v>
+      </c>
+      <c r="F31" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" t="s">
+        <v>146</v>
+      </c>
+      <c r="I31" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>161</v>
+      </c>
+      <c r="B32">
+        <v>0.6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33">
+        <f>1000*0.01625</f>
+        <v>16.25</v>
+      </c>
+      <c r="D33" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>141</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" t="s">
+        <v>15</v>
+      </c>
+      <c r="H43" t="s">
+        <v>20</v>
+      </c>
+      <c r="I43" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="str">
+        <f>B38</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B44">
+        <f>B37</f>
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>16</v>
+      </c>
+      <c r="F44" t="s">
+        <v>17</v>
+      </c>
+      <c r="G44" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>140</v>
+      </c>
+      <c r="B45">
+        <f>1000*1</f>
+        <v>1000</v>
+      </c>
+      <c r="C45" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>26</v>
+      </c>
+      <c r="F46" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>141</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>14</v>
+      </c>
+      <c r="B53" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>6</v>
+      </c>
+      <c r="B55" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>11</v>
+      </c>
+      <c r="B57" t="s">
+        <v>12</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" t="s">
+        <v>14</v>
+      </c>
+      <c r="E57" t="s">
+        <v>23</v>
+      </c>
+      <c r="F57" t="s">
+        <v>9</v>
+      </c>
+      <c r="G57" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" t="s">
+        <v>20</v>
+      </c>
+      <c r="I57" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
+        <f>B52</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B58">
+        <f>B51</f>
+        <v>1</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>16</v>
+      </c>
+      <c r="F58" t="s">
+        <v>17</v>
+      </c>
+      <c r="G58" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B60">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C60" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" t="s">
+        <v>26</v>
+      </c>
+      <c r="F60" t="s">
+        <v>18</v>
+      </c>
+      <c r="G60" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>153</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+    </row>
+    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
+    </row>
+    <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="4"/>
+    </row>
+    <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A75" s="4"/>
+    </row>
+    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="G76" s="4"/>
+    </row>
+    <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="4"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="4"/>
+    </row>
+    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF05BD3-82B5-4829-9975-BAE4BAEB41CD}">
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.21875" customWidth="1"/>
+    <col min="8" max="8" width="26.33203125" customWidth="1"/>
+    <col min="15" max="15" width="27.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="3"/>
-    </row>
     <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="8" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>126</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14">
-        <v>2.0000000000000001E-4</v>
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B15">
-        <v>0.03</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B16">
-        <v>2.8500000000000001E-2</v>
+        <v>0.03</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B17">
-        <v>1.5E-3</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B18">
-        <v>1.6999999999999999E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B19">
-        <v>1E-4</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B20">
-        <v>0.95</v>
+        <v>1E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B21">
-        <v>0.05</v>
+        <v>0.95</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B22">
-        <v>0.24912000000000001</v>
-      </c>
-      <c r="C22" t="s">
-        <v>61</v>
+        <v>0.05</v>
       </c>
       <c r="D22" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B23">
-        <v>4.7999999999999998E-6</v>
+        <v>0.24912000000000001</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B24">
-        <v>1.36E-5</v>
+        <v>4.7999999999999998E-6</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25">
+        <v>1.36E-5</v>
+      </c>
+      <c r="C25" t="s">
+        <v>67</v>
+      </c>
+      <c r="D25" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>69</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <v>1000</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+    <row r="28" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" t="s">
-        <v>23</v>
-      </c>
-      <c r="G28" t="s">
-        <v>9</v>
-      </c>
-      <c r="H28" t="s">
-        <v>37</v>
-      </c>
-      <c r="I28" t="s">
-        <v>20</v>
-      </c>
-      <c r="J28" t="s">
-        <v>21</v>
-      </c>
-      <c r="K28" t="s">
-        <v>70</v>
-      </c>
-      <c r="L28" t="s">
-        <v>71</v>
-      </c>
-      <c r="M28" t="s">
-        <v>72</v>
-      </c>
-      <c r="N28" t="s">
-        <v>6</v>
-      </c>
-      <c r="O28" t="s">
-        <v>73</v>
-      </c>
-      <c r="P28" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R28" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29">
-        <v>2.8499999999999998E-6</v>
+        <v>11</v>
+      </c>
+      <c r="B29" t="s">
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="G29" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="H29" t="s">
-        <v>77</v>
-      </c>
-      <c r="I29">
-        <v>2</v>
-      </c>
-      <c r="J29">
-        <v>-13.74250176111102</v>
-      </c>
-      <c r="K29">
-        <v>0.34942810419312298</v>
+        <v>37</v>
+      </c>
+      <c r="I29" t="s">
+        <v>20</v>
+      </c>
+      <c r="J29" t="s">
+        <v>21</v>
+      </c>
+      <c r="K29" t="s">
+        <v>70</v>
       </c>
       <c r="L29" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="M29" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="N29" t="s">
-        <v>132</v>
-      </c>
-      <c r="O29">
-        <v>2.8540000000000002E-3</v>
+        <v>6</v>
+      </c>
+      <c r="O29" t="s">
+        <v>73</v>
       </c>
       <c r="P29" t="s">
-        <v>80</v>
-      </c>
-      <c r="R29">
-        <v>0.2</v>
+        <v>74</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>15</v>
+      </c>
+      <c r="R29" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="B30">
-        <v>3.7367999999999999E-4</v>
+        <v>2.8499999999999998E-6</v>
       </c>
       <c r="C30" t="s">
         <v>25</v>
@@ -2008,42 +2963,42 @@
         <v>27</v>
       </c>
       <c r="H30" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I30">
         <v>2</v>
       </c>
       <c r="J30">
-        <v>-4.781436711539472</v>
+        <v>-13.74250176111102</v>
       </c>
       <c r="K30">
-        <v>0.2046948949045872</v>
+        <v>0.34942810419312298</v>
       </c>
       <c r="L30" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="M30" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="N30" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O30">
-        <v>1.2659999999999999E-4</v>
+        <v>2.8540000000000002E-3</v>
       </c>
       <c r="P30" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="R30">
-        <v>2.4494897427831779E-2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>3.7367999999999999E-4</v>
       </c>
       <c r="C31" t="s">
         <v>25</v>
@@ -2057,34 +3012,43 @@
       <c r="G31" t="s">
         <v>27</v>
       </c>
+      <c r="H31" t="s">
+        <v>82</v>
+      </c>
       <c r="I31">
         <v>2</v>
       </c>
       <c r="J31">
-        <v>-11.84434628152367</v>
+        <v>-4.781436711539472</v>
       </c>
       <c r="K31">
-        <v>0.83144452611103292</v>
+        <v>0.2046948949045872</v>
       </c>
       <c r="L31" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="M31" t="s">
-        <v>88</v>
+        <v>84</v>
+      </c>
+      <c r="N31" t="s">
+        <v>133</v>
+      </c>
+      <c r="O31">
+        <v>1.2659999999999999E-4</v>
       </c>
       <c r="P31" t="s">
         <v>85</v>
       </c>
       <c r="R31">
-        <v>0.80622577482985502</v>
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="B32">
-        <v>2.0400000000000001E-8</v>
+        <v>0</v>
       </c>
       <c r="C32" t="s">
         <v>25</v>
@@ -2098,35 +3062,26 @@
       <c r="G32" t="s">
         <v>27</v>
       </c>
-      <c r="H32" t="s">
-        <v>89</v>
-      </c>
       <c r="I32">
         <v>2</v>
       </c>
       <c r="J32">
-        <v>-14.664736275474411</v>
+        <v>-11.84434628152367</v>
       </c>
       <c r="K32">
-        <v>0.2851315485876651</v>
+        <v>0.83144452611103292</v>
       </c>
       <c r="L32" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="M32" t="s">
-        <v>91</v>
-      </c>
-      <c r="N32" t="s">
-        <v>133</v>
-      </c>
-      <c r="O32">
-        <v>4.27746E-7</v>
+        <v>88</v>
       </c>
       <c r="P32" t="s">
         <v>85</v>
       </c>
       <c r="R32">
-        <v>0.2</v>
+        <v>0.80622577482985502</v>
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.3">
@@ -2134,7 +3089,7 @@
         <v>28</v>
       </c>
       <c r="B33">
-        <v>5.6999999999999996E-6</v>
+        <v>2.0400000000000001E-8</v>
       </c>
       <c r="C33" t="s">
         <v>25</v>
@@ -2149,21 +3104,42 @@
         <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>92</v>
+        <v>89</v>
+      </c>
+      <c r="I33">
+        <v>2</v>
+      </c>
+      <c r="J33">
+        <v>-14.664736275474411</v>
+      </c>
+      <c r="K33">
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="L33" t="s">
+        <v>90</v>
+      </c>
+      <c r="M33" t="s">
+        <v>91</v>
       </c>
       <c r="N33" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O33">
-        <v>5.7000000000000002E-3</v>
+        <v>4.27746E-7</v>
+      </c>
+      <c r="P33" t="s">
+        <v>85</v>
+      </c>
+      <c r="R33">
+        <v>0.2</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="B34">
-        <v>7.2E-9</v>
+        <v>5.6999999999999996E-6</v>
       </c>
       <c r="C34" t="s">
         <v>25</v>
@@ -2178,42 +3154,21 @@
         <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>94</v>
-      </c>
-      <c r="I34">
-        <v>2</v>
-      </c>
-      <c r="J34">
-        <v>-15.751988332064601</v>
-      </c>
-      <c r="K34">
-        <v>0.2851315485876651</v>
-      </c>
-      <c r="L34" t="s">
-        <v>95</v>
-      </c>
-      <c r="M34" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="N34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O34">
-        <v>1E-8</v>
-      </c>
-      <c r="P34" t="s">
-        <v>85</v>
-      </c>
-      <c r="R34">
-        <v>0.2</v>
+        <v>5.7000000000000002E-3</v>
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>7.2E-9</v>
       </c>
       <c r="C35" t="s">
         <v>25</v>
@@ -2227,13 +3182,43 @@
       <c r="G35" t="s">
         <v>27</v>
       </c>
+      <c r="H35" t="s">
+        <v>94</v>
+      </c>
+      <c r="I35">
+        <v>2</v>
+      </c>
+      <c r="J35">
+        <v>-15.751988332064601</v>
+      </c>
+      <c r="K35">
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="L35" t="s">
+        <v>95</v>
+      </c>
+      <c r="M35" t="s">
+        <v>96</v>
+      </c>
+      <c r="N35" t="s">
+        <v>133</v>
+      </c>
+      <c r="O35">
+        <v>1E-8</v>
+      </c>
+      <c r="P35" t="s">
+        <v>85</v>
+      </c>
+      <c r="R35">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B36">
-        <v>4.8449999999999992E-5</v>
+        <v>0</v>
       </c>
       <c r="C36" t="s">
         <v>25</v>
@@ -2247,40 +3232,13 @@
       <c r="G36" t="s">
         <v>27</v>
       </c>
-      <c r="H36" t="s">
-        <v>97</v>
-      </c>
-      <c r="I36">
-        <v>2</v>
-      </c>
-      <c r="J36">
-        <v>-8.5295340272510369</v>
-      </c>
-      <c r="K36">
-        <v>0.2851315485876651</v>
-      </c>
-      <c r="M36" t="s">
-        <v>98</v>
-      </c>
-      <c r="N36" t="s">
-        <v>134</v>
-      </c>
-      <c r="O36">
-        <v>4.8512E-2</v>
-      </c>
-      <c r="P36" t="s">
-        <v>85</v>
-      </c>
-      <c r="R36">
-        <v>0.2</v>
-      </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>4.8449999999999992E-5</v>
       </c>
       <c r="C37" t="s">
         <v>25</v>
@@ -2294,25 +3252,37 @@
       <c r="G37" t="s">
         <v>27</v>
       </c>
+      <c r="H37" t="s">
+        <v>97</v>
+      </c>
       <c r="I37">
         <v>2</v>
       </c>
       <c r="J37">
-        <v>-12.26645129759965</v>
+        <v>-8.5295340272510369</v>
       </c>
       <c r="K37">
-        <v>0.58420886675914119</v>
+        <v>0.2851315485876651</v>
+      </c>
+      <c r="M37" t="s">
+        <v>98</v>
+      </c>
+      <c r="N37" t="s">
+        <v>134</v>
+      </c>
+      <c r="O37">
+        <v>4.8512E-2</v>
       </c>
       <c r="P37" t="s">
         <v>85</v>
       </c>
       <c r="R37">
-        <v>0.54772255750516607</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -2333,21 +3303,21 @@
         <v>2</v>
       </c>
       <c r="J38">
-        <v>-11.90977529142279</v>
+        <v>-12.26645129759965</v>
       </c>
       <c r="K38">
-        <v>0.40162171256046397</v>
+        <v>0.58420886675914119</v>
       </c>
       <c r="P38" t="s">
         <v>85</v>
       </c>
       <c r="R38">
-        <v>0.34641016151377552</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -2368,21 +3338,21 @@
         <v>2</v>
       </c>
       <c r="J39">
-        <v>-12.132918842737</v>
+        <v>-11.90977529142279</v>
       </c>
       <c r="K39">
-        <v>0.58420886675914119</v>
+        <v>0.40162171256046397</v>
       </c>
       <c r="P39" t="s">
         <v>85</v>
       </c>
       <c r="R39">
-        <v>0.54772255750516607</v>
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -2403,82 +3373,88 @@
         <v>2</v>
       </c>
       <c r="J40">
-        <v>-9.0081753390471704</v>
+        <v>-12.132918842737</v>
       </c>
       <c r="K40">
-        <v>0.2046948949045872</v>
-      </c>
-      <c r="L40" t="s">
-        <v>102</v>
-      </c>
-      <c r="M40" t="s">
-        <v>103</v>
+        <v>0.58420886675914119</v>
       </c>
       <c r="P40" t="s">
         <v>85</v>
       </c>
       <c r="R40">
-        <v>2.4494897427831779E-2</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>101</v>
       </c>
       <c r="B41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
-      </c>
-      <c r="D41" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E41" t="s">
-        <v>16</v>
+        <v>26</v>
+      </c>
+      <c r="F41" t="s">
+        <v>76</v>
       </c>
       <c r="G41" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q41" t="s">
-        <v>19</v>
+        <v>27</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="J41">
+        <v>-9.0081753390471704</v>
+      </c>
+      <c r="K41">
+        <v>0.2046948949045872</v>
+      </c>
+      <c r="L41" t="s">
+        <v>102</v>
+      </c>
+      <c r="M41" t="s">
+        <v>103</v>
+      </c>
+      <c r="P41" t="s">
+        <v>85</v>
+      </c>
+      <c r="R41">
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>139</v>
+        <v>34</v>
       </c>
       <c r="B42">
-        <v>2.8500000000000001E-2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>22</v>
+        <v>125</v>
       </c>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>8</v>
       </c>
       <c r="E42" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G42" t="s">
-        <v>18</v>
-      </c>
-      <c r="H42" t="s">
-        <v>44</v>
-      </c>
-      <c r="O42">
-        <v>5.4999999999999997E-3</v>
+        <v>17</v>
       </c>
       <c r="Q42" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
       <c r="B43">
-        <v>-1.2999999999999999E-5</v>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
@@ -2492,40 +3468,28 @@
       <c r="G43" t="s">
         <v>18</v>
       </c>
-      <c r="I43">
-        <v>2</v>
-      </c>
-      <c r="J43">
-        <v>-11.61787681268815</v>
-      </c>
-      <c r="K43">
-        <v>0.21142374511865969</v>
-      </c>
-      <c r="N43" t="s">
-        <v>107</v>
-      </c>
-      <c r="P43" t="s">
-        <v>108</v>
+      <c r="H43" t="s">
+        <v>44</v>
+      </c>
+      <c r="O43">
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="Q43" t="s">
-        <v>109</v>
-      </c>
-      <c r="R43">
-        <v>2.4494897427831779E-2</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B44">
-        <v>1.5E-3</v>
+        <v>-1.2999999999999999E-5</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E44" t="s">
         <v>26</v>
@@ -2533,63 +3497,63 @@
       <c r="G44" t="s">
         <v>18</v>
       </c>
-      <c r="H44" t="s">
-        <v>47</v>
-      </c>
-      <c r="O44">
-        <v>1.2659999999999999E-4</v>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
+        <v>-11.61787681268815</v>
+      </c>
+      <c r="K44">
+        <v>0.21142374511865969</v>
+      </c>
+      <c r="N44" t="s">
+        <v>107</v>
+      </c>
+      <c r="P44" t="s">
+        <v>108</v>
       </c>
       <c r="Q44" t="s">
-        <v>112</v>
+        <v>109</v>
+      </c>
+      <c r="R44">
+        <v>2.4494897427831779E-2</v>
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B45">
-        <v>1.0593999999999999E-11</v>
+        <v>1.5E-3</v>
       </c>
       <c r="C45" t="s">
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>8</v>
+        <v>111</v>
       </c>
       <c r="E45" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G45" t="s">
         <v>18</v>
       </c>
-      <c r="I45">
-        <v>2</v>
-      </c>
-      <c r="J45">
-        <v>-25.270733312806211</v>
-      </c>
-      <c r="K45">
-        <v>0.46540305112880392</v>
-      </c>
-      <c r="N45" t="s">
-        <v>114</v>
-      </c>
-      <c r="P45" t="s">
-        <v>115</v>
+      <c r="H45" t="s">
+        <v>47</v>
+      </c>
+      <c r="O45">
+        <v>1.2659999999999999E-4</v>
       </c>
       <c r="Q45" t="s">
-        <v>116</v>
-      </c>
-      <c r="R45">
-        <v>0.34641016151377552</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>32</v>
+        <v>113</v>
       </c>
       <c r="B46">
-        <v>1.3798099999999999E-16</v>
+        <v>1.0593999999999999E-11</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
@@ -2607,30 +3571,30 @@
         <v>2</v>
       </c>
       <c r="J46">
-        <v>-36.519415679373957</v>
+        <v>-25.270733312806211</v>
       </c>
       <c r="K46">
-        <v>0.58702640485756685</v>
+        <v>0.46540305112880392</v>
       </c>
       <c r="N46" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="P46" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="Q46" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="R46">
-        <v>0.54772255750516607</v>
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="B47">
-        <v>1.0593999999999999E-11</v>
+        <v>1.3798099999999999E-16</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
@@ -2648,50 +3612,68 @@
         <v>2</v>
       </c>
       <c r="J47">
-        <v>-25.270733312806211</v>
+        <v>-36.519415679373957</v>
       </c>
       <c r="K47">
-        <v>0.46540305112880392</v>
+        <v>0.58702640485756685</v>
       </c>
       <c r="N47" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="P47" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="Q47" t="s">
-        <v>120</v>
+        <v>33</v>
       </c>
       <c r="R47">
-        <v>0.34641016151377552</v>
+        <v>0.54772255750516607</v>
       </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B48">
-        <v>0</v>
+        <v>1.0593999999999999E-11</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>8</v>
       </c>
       <c r="E48" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G48" t="s">
         <v>18</v>
       </c>
+      <c r="I48">
+        <v>2</v>
+      </c>
+      <c r="J48">
+        <v>-25.270733312806211</v>
+      </c>
+      <c r="K48">
+        <v>0.46540305112880392</v>
+      </c>
+      <c r="N48" t="s">
+        <v>114</v>
+      </c>
+      <c r="P48" t="s">
+        <v>115</v>
+      </c>
       <c r="Q48" t="s">
-        <v>122</v>
+        <v>120</v>
+      </c>
+      <c r="R48">
+        <v>0.34641016151377552</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -2709,6 +3691,29 @@
         <v>18</v>
       </c>
       <c r="Q49" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>123</v>
+      </c>
+      <c r="B50">
+        <v>0</v>
+      </c>
+      <c r="C50" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" t="s">
+        <v>104</v>
+      </c>
+      <c r="E50" t="s">
+        <v>26</v>
+      </c>
+      <c r="G50" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q50" t="s">
         <v>124</v>
       </c>
     </row>
@@ -2717,7 +3722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EFFFC2-89D0-45E5-B7FA-4B2E66075D0E}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
commenting for better understanding
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8414FC-1405-4F9C-8A66-41FC458B3A88}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE1B97-7C35-432D-8D53-B8814D8B19BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="174">
   <si>
     <t>Database</t>
   </si>
@@ -549,6 +549,21 @@
   </si>
   <si>
     <t>DE</t>
+  </si>
+  <si>
+    <t>market for transport, freight, lorry</t>
+  </si>
+  <si>
+    <t>transport, freight, lorry</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, gaseous, lorry, unspecified</t>
+  </si>
+  <si>
+    <t>transport, hydrogen, liquid, lorry, unspecified</t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
   </si>
 </sst>
 </file>
@@ -953,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
@@ -982,7 +997,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1006,7 +1021,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1067,7 +1082,7 @@
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <f>B6</f>
-        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+        <v>transport, hydrogen, gaseous, lorry, unspecified</v>
       </c>
       <c r="B12">
         <f>B5</f>
@@ -1084,7 +1099,7 @@
       </c>
       <c r="G12" t="str">
         <f>A12</f>
-        <v>transport, hydrogen, gaseous, lorry, market average propulsion system</v>
+        <v>transport, hydrogen, gaseous, lorry, unspecified</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1115,8 +1130,8 @@
         <v>140</v>
       </c>
       <c r="B14">
-        <f>1*1000</f>
-        <v>1000</v>
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
@@ -1158,203 +1173,197 @@
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16">
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17">
         <f>1000*0.005</f>
         <v>5</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D17" t="s">
         <v>26</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E17" t="s">
         <v>155</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F17" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" t="s">
-        <v>8</v>
+      <c r="B19" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>141</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="s">
-        <v>167</v>
+        <v>141</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>16</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>6</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>11</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B27" t="s">
         <v>12</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C27" t="s">
         <v>7</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D27" t="s">
         <v>14</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E27" t="s">
         <v>23</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F27" t="s">
         <v>9</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G27" t="s">
         <v>15</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H27" t="s">
         <v>20</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I27" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" t="str">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" t="str">
+        <f>B22</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      </c>
+      <c r="B28">
         <f>B21</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-      <c r="B27">
-        <f>B20</f>
         <v>1</v>
       </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
         <v>16</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F28" t="s">
         <v>17</v>
       </c>
-      <c r="G27" t="str">
-        <f>A27</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="G28" t="str">
+        <f>A28</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>140</v>
       </c>
-      <c r="B28">
-        <v>1000</v>
-      </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="B29">
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
         <v>26</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F29" t="s">
         <v>18</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>140</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I29" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
+    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>165</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D30" t="s">
         <v>26</v>
-      </c>
-      <c r="F29" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" t="s">
-        <v>157</v>
-      </c>
-      <c r="I29" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>161</v>
-      </c>
-      <c r="B30">
-        <f>1000*6.78</f>
-        <v>6780</v>
-      </c>
-      <c r="C30" t="s">
-        <v>168</v>
-      </c>
-      <c r="D30" t="s">
-        <v>164</v>
       </c>
       <c r="F30" t="s">
         <v>18</v>
       </c>
       <c r="G30" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="I30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -1362,7 +1371,8 @@
         <v>161</v>
       </c>
       <c r="B31">
-        <v>0.6</v>
+        <f>1000*6.78</f>
+        <v>6780</v>
       </c>
       <c r="C31" t="s">
         <v>168</v>
@@ -1377,166 +1387,170 @@
         <v>146</v>
       </c>
       <c r="I31" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="B32">
+        <f>1000*0.6</f>
+        <v>600</v>
+      </c>
+      <c r="C32" t="s">
+        <v>168</v>
+      </c>
+      <c r="D32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F32" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" t="s">
+        <v>146</v>
+      </c>
+      <c r="I32" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>173</v>
+      </c>
+      <c r="B33">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>26</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E33" t="s">
         <v>155</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F33" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>141</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>15</v>
-      </c>
-      <c r="B37" t="s">
-        <v>145</v>
+        <v>141</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>16</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
         <v>6</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>11</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>12</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>7</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D43" t="s">
         <v>14</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E43" t="s">
         <v>23</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F43" t="s">
         <v>9</v>
       </c>
-      <c r="G42" t="s">
+      <c r="G43" t="s">
         <v>15</v>
       </c>
-      <c r="H42" t="s">
+      <c r="H43" t="s">
         <v>20</v>
       </c>
-      <c r="I42" t="s">
+      <c r="I43" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" t="str">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A44" t="str">
+        <f>B38</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B44">
         <f>B37</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
-      </c>
-      <c r="B43">
-        <f>B36</f>
         <v>1</v>
       </c>
-      <c r="C43" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
         <v>16</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F44" t="s">
         <v>17</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G44" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>140</v>
       </c>
-      <c r="B44">
-        <f>1000*1</f>
-        <v>1000</v>
-      </c>
-      <c r="C44" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" t="s">
-        <v>26</v>
-      </c>
-      <c r="F44" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>156</v>
-      </c>
       <c r="B45">
-        <v>5.0000000000000001E-3</v>
+        <f>1000*1/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C45" t="s">
-        <v>165</v>
+        <v>8</v>
       </c>
       <c r="D45" t="s">
         <v>26</v>
@@ -1545,167 +1559,167 @@
         <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>153</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="B46">
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="D46" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F46" t="s">
         <v>18</v>
       </c>
       <c r="G46" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B47">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>16</v>
+      </c>
+      <c r="F47" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>7</v>
-      </c>
-      <c r="B49" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>141</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>15</v>
-      </c>
-      <c r="B51" t="s">
-        <v>158</v>
+        <v>141</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
-        <v>16</v>
+        <v>158</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="B53" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
         <v>6</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>11</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>12</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>7</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D57" t="s">
         <v>14</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E57" t="s">
         <v>23</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F57" t="s">
         <v>9</v>
       </c>
-      <c r="G56" t="s">
+      <c r="G57" t="s">
         <v>15</v>
       </c>
-      <c r="H56" t="s">
+      <c r="H57" t="s">
         <v>20</v>
       </c>
-      <c r="I56" t="s">
+      <c r="I57" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" t="str">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" t="str">
+        <f>B52</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B58">
         <f>B51</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
-      </c>
-      <c r="B57">
-        <f>B50</f>
         <v>1</v>
       </c>
-      <c r="C57" t="s">
-        <v>8</v>
-      </c>
-      <c r="D57" t="s">
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
         <v>16</v>
       </c>
-      <c r="F57" t="s">
+      <c r="F58" t="s">
         <v>17</v>
       </c>
-      <c r="G57" t="s">
+      <c r="G58" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
         <v>140</v>
       </c>
-      <c r="B58">
+      <c r="B59">
         <v>0</v>
       </c>
-      <c r="C58" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" t="s">
-        <v>26</v>
-      </c>
-      <c r="F58" t="s">
-        <v>18</v>
-      </c>
-      <c r="G58" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B59">
-        <v>5.0000000000000001E-3</v>
-      </c>
       <c r="C59" t="s">
-        <v>165</v>
+        <v>8</v>
       </c>
       <c r="D59" t="s">
         <v>26</v>
@@ -1714,38 +1728,55 @@
         <v>18</v>
       </c>
       <c r="G59" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>153</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>156</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C60" t="s">
-        <v>8</v>
+        <v>165</v>
       </c>
       <c r="D60" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F60" t="s">
         <v>18</v>
       </c>
       <c r="G60" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>153</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1"/>
-    </row>
-    <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" s="1"/>
-    </row>
-    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="4"/>
+    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+    </row>
+    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
     </row>
     <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
@@ -1755,10 +1786,10 @@
     </row>
     <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
-      <c r="G75" s="4"/>
-    </row>
-    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A77" s="4"/>
+    </row>
+    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A76" s="4"/>
+      <c r="G76" s="4"/>
     </row>
     <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
@@ -1768,6 +1799,9 @@
     </row>
     <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
+    </row>
+    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A81" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changed h2 transport names. added search for hydrogen consumers in test_premise
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE1B97-7C35-432D-8D53-B8814D8B19BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47834992-4E3F-4A46-99FC-1AC8250CAD41}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
-    <sheet name="hydrogen-transport (2)" sheetId="4" r:id="rId2"/>
-    <sheet name="ship" sheetId="3" r:id="rId3"/>
-    <sheet name="Parameters" sheetId="2" r:id="rId4"/>
+    <sheet name="ship" sheetId="3" r:id="rId2"/>
+    <sheet name="Parameters" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="169">
   <si>
     <t>Database</t>
   </si>
@@ -491,18 +490,6 @@
     <t>electricity needed for liquefaction, Stoltenberg et al</t>
   </si>
   <si>
-    <t>compensation for losses</t>
-  </si>
-  <si>
-    <t>market for transport, freight, lorry with refrigeration machine, diesel, freezing, fleet average</t>
-  </si>
-  <si>
-    <t>transport, freight, lorry with refrigeration machine, diesel, freezing, fleet average</t>
-  </si>
-  <si>
-    <t>hydrogen</t>
-  </si>
-  <si>
     <t>market for transport, freight, sea, tanker for liquefied natural gas, heavy fuel oil</t>
   </si>
   <si>
@@ -521,12 +508,6 @@
     <t>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</t>
   </si>
   <si>
-    <t>transport, hydrogen, gaseous, lorry, market average propulsion system</t>
-  </si>
-  <si>
-    <t>this dataset is used as a proxy</t>
-  </si>
-  <si>
     <t>market for electricity, medium voltage</t>
   </si>
   <si>
@@ -542,12 +523,6 @@
     <t>RER</t>
   </si>
   <si>
-    <t>transport, hydrogen, gaseous, lorry , market average propulsion system</t>
-  </si>
-  <si>
-    <t>transport, hydrogen, liquid, lorry, market average propulsion system</t>
-  </si>
-  <si>
     <t>DE</t>
   </si>
   <si>
@@ -564,6 +539,15 @@
   </si>
   <si>
     <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>this dataset is used as a proxy, so the lorry used uses the propulsion system chosen by the IAM scenario</t>
+  </si>
+  <si>
+    <t>boil-off losses to the atmosphere</t>
+  </si>
+  <si>
+    <t>compensation for boil-off losses</t>
   </si>
 </sst>
 </file>
@@ -968,7 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
@@ -997,7 +981,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1021,7 +1005,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1104,37 +1088,38 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
       </c>
       <c r="G13" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="I13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>140</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="B14">
-        <f>1*1000/540000</f>
-        <v>1.8518518518518519E-3</v>
+        <f>1000*0.005</f>
+        <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>159</v>
       </c>
       <c r="D14" t="s">
         <v>26</v>
@@ -1143,665 +1128,630 @@
         <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="I14" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>156</v>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>165</v>
       </c>
       <c r="B15">
         <f>1000*0.005</f>
         <v>5</v>
       </c>
-      <c r="C15" t="s">
-        <v>165</v>
-      </c>
       <c r="D15" t="s">
         <v>26</v>
       </c>
+      <c r="E15" t="s">
+        <v>151</v>
+      </c>
       <c r="F15" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" t="s">
-        <v>157</v>
+        <v>27</v>
       </c>
       <c r="I15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C16" t="s">
-        <v>165</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>173</v>
-      </c>
-      <c r="B17">
-        <f>1000*0.005</f>
-        <v>5</v>
-      </c>
-      <c r="D17" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>172</v>
+      <c r="B17" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>172</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>126</v>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" t="s">
         <v>6</v>
       </c>
-      <c r="B25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>10</v>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="str">
+        <f>B20</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      </c>
+      <c r="B26">
+        <f>B19</f>
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" t="str">
+        <f>A26</f>
+        <v>transport, hydrogen, liquid, lorry, unspecified</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
+        <v>140</v>
+      </c>
+      <c r="B27">
+        <f>1*1000/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C27" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F27" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="I27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" t="str">
-        <f>B22</f>
-        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="B28">
-        <f>B21</f>
-        <v>1</v>
+        <f>1000*0.01625</f>
+        <v>16.25</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>159</v>
       </c>
       <c r="D28" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F28" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" t="str">
-        <f>A28</f>
-        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+        <v>18</v>
+      </c>
+      <c r="G28" t="s">
+        <v>153</v>
+      </c>
+      <c r="I28" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="B29">
-        <f>1*1000/540000</f>
-        <v>1.8518518518518519E-3</v>
+        <f>1000*6.78</f>
+        <v>6780</v>
       </c>
       <c r="C29" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>158</v>
       </c>
       <c r="F29" t="s">
         <v>18</v>
       </c>
       <c r="G29" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="I29" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>156</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>155</v>
       </c>
       <c r="B30">
+        <f>1000*0.6</f>
+        <v>600</v>
+      </c>
+      <c r="C30" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" t="s">
+        <v>158</v>
+      </c>
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>146</v>
+      </c>
+      <c r="I30" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>165</v>
+      </c>
+      <c r="B31">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="C30" t="s">
-        <v>165</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="D31" t="s">
         <v>26</v>
       </c>
-      <c r="F30" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" t="s">
-        <v>157</v>
-      </c>
-      <c r="I30" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>161</v>
-      </c>
-      <c r="B31">
-        <f>1000*6.78</f>
-        <v>6780</v>
-      </c>
-      <c r="C31" t="s">
-        <v>168</v>
-      </c>
-      <c r="D31" t="s">
-        <v>164</v>
+      <c r="E31" t="s">
+        <v>151</v>
       </c>
       <c r="F31" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" t="s">
-        <v>146</v>
+        <v>27</v>
       </c>
       <c r="I31" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>161</v>
-      </c>
-      <c r="B32">
-        <f>1000*0.6</f>
-        <v>600</v>
-      </c>
-      <c r="C32" t="s">
-        <v>168</v>
-      </c>
-      <c r="D32" t="s">
-        <v>164</v>
-      </c>
-      <c r="F32" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>173</v>
-      </c>
-      <c r="B33">
-        <f>1000*0.01625</f>
-        <v>16.25</v>
-      </c>
-      <c r="D33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" t="s">
-        <v>155</v>
-      </c>
-      <c r="F33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>8</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="B37" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>126</v>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>20</v>
+      </c>
+      <c r="I41" t="s">
         <v>6</v>
       </c>
-      <c r="B41" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>10</v>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="str">
+        <f>B36</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B42">
+        <f>B35</f>
+        <v>1</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" t="s">
+        <v>17</v>
+      </c>
+      <c r="G42" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" t="s">
-        <v>12</v>
+        <v>140</v>
+      </c>
+      <c r="B43">
+        <f>1000*1/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C43" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D43" t="s">
-        <v>14</v>
-      </c>
-      <c r="E43" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F43" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G43" t="s">
-        <v>15</v>
-      </c>
-      <c r="H43" t="s">
-        <v>20</v>
-      </c>
-      <c r="I43" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>B38</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="B44">
-        <f>B37</f>
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C44" t="s">
-        <v>8</v>
+        <v>159</v>
       </c>
       <c r="D44" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G44" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="B45">
-        <f>1000*1/540000</f>
-        <v>1.8518518518518519E-3</v>
+        <v>1</v>
       </c>
       <c r="C45" t="s">
         <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F45" t="s">
         <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B46">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C46" t="s">
-        <v>165</v>
-      </c>
-      <c r="D46" t="s">
-        <v>26</v>
-      </c>
-      <c r="F46" t="s">
-        <v>18</v>
-      </c>
-      <c r="G46" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>153</v>
-      </c>
-      <c r="B47">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>141</v>
+      </c>
+      <c r="B49">
         <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" t="s">
-        <v>16</v>
-      </c>
-      <c r="F47" t="s">
-        <v>18</v>
-      </c>
-      <c r="G47" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
-        <v>8</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>141</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="B51" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>15</v>
-      </c>
-      <c r="B52" t="s">
-        <v>158</v>
+        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B53" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>126</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
+        <v>11</v>
+      </c>
+      <c r="B55" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" t="s">
+        <v>14</v>
+      </c>
+      <c r="E55" t="s">
+        <v>23</v>
+      </c>
+      <c r="F55" t="s">
+        <v>9</v>
+      </c>
+      <c r="G55" t="s">
+        <v>15</v>
+      </c>
+      <c r="H55" t="s">
+        <v>20</v>
+      </c>
+      <c r="I55" t="s">
         <v>6</v>
       </c>
-      <c r="B55" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
-        <v>10</v>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" t="str">
+        <f>B50</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B56">
+        <f>B49</f>
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" t="s">
+        <v>16</v>
+      </c>
+      <c r="F56" t="s">
+        <v>17</v>
+      </c>
+      <c r="G56" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" t="s">
-        <v>12</v>
+        <v>140</v>
+      </c>
+      <c r="B57">
+        <v>0</v>
       </c>
       <c r="C57" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D57" t="s">
-        <v>14</v>
-      </c>
-      <c r="E57" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F57" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G57" t="s">
-        <v>15</v>
-      </c>
-      <c r="H57" t="s">
-        <v>20</v>
-      </c>
-      <c r="I57" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" t="str">
-        <f>B52</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="B58">
-        <f>B51</f>
-        <v>1</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C58" t="s">
-        <v>8</v>
+        <v>159</v>
       </c>
       <c r="D58" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G58" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="B59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F59" t="s">
         <v>18</v>
       </c>
       <c r="G59" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B60">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C60" t="s">
-        <v>165</v>
-      </c>
-      <c r="D60" t="s">
-        <v>26</v>
-      </c>
-      <c r="F60" t="s">
-        <v>18</v>
-      </c>
-      <c r="G60" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>153</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" t="s">
-        <v>16</v>
-      </c>
-      <c r="F61" t="s">
-        <v>18</v>
-      </c>
-      <c r="G61" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-    </row>
-    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="1"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+    </row>
+    <row r="68" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A68" s="1"/>
+    </row>
+    <row r="71" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A71" s="4"/>
+    </row>
+    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
     </row>
     <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
     </row>
     <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
-    </row>
-    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="4"/>
+      <c r="G74" s="4"/>
     </row>
     <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
-      <c r="G76" s="4"/>
+    </row>
+    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
     </row>
     <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
     </row>
     <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
-    </row>
-    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="4"/>
-    </row>
-    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A81" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1810,835 +1760,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFCFE87B-D030-4AA0-99E6-3DBA7D6E9B67}">
-  <dimension ref="A1:I81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="85.44140625" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.21875" customWidth="1"/>
-    <col min="12" max="12" width="43.88671875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" t="str">
-        <f>B7</f>
-        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
-      </c>
-      <c r="B13">
-        <f>B6</f>
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" t="str">
-        <f>A13</f>
-        <v>transport, hydrogen, gaseous, lorry , market average propulsion system</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>150</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" t="s">
-        <v>151</v>
-      </c>
-      <c r="I14" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15">
-        <f>1*1000</f>
-        <v>1000</v>
-      </c>
-      <c r="C15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" t="s">
-        <v>140</v>
-      </c>
-      <c r="I15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B16">
-        <f>1000*0.005</f>
-        <v>5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" t="s">
-        <v>157</v>
-      </c>
-      <c r="I16" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B17">
-        <f>1000*0.005</f>
-        <v>5</v>
-      </c>
-      <c r="D17" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" t="str">
-        <f>B22</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-      <c r="B28">
-        <f>B21</f>
-        <v>1</v>
-      </c>
-      <c r="C28" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" t="s">
-        <v>16</v>
-      </c>
-      <c r="F28" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" t="str">
-        <f>A28</f>
-        <v>transport, hydrogen, liquid, lorry, market average propulsion system</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>140</v>
-      </c>
-      <c r="B29">
-        <v>1000</v>
-      </c>
-      <c r="C29" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" t="s">
-        <v>26</v>
-      </c>
-      <c r="F29" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" t="s">
-        <v>140</v>
-      </c>
-      <c r="I29" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B30">
-        <f>1000*0.01625</f>
-        <v>16.25</v>
-      </c>
-      <c r="C30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" t="s">
-        <v>26</v>
-      </c>
-      <c r="F30" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" t="s">
-        <v>157</v>
-      </c>
-      <c r="I30" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>161</v>
-      </c>
-      <c r="B31">
-        <f>1000*6.78</f>
-        <v>6780</v>
-      </c>
-      <c r="C31" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" t="s">
-        <v>164</v>
-      </c>
-      <c r="F31" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" t="s">
-        <v>146</v>
-      </c>
-      <c r="I31" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>161</v>
-      </c>
-      <c r="B32">
-        <v>0.6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" t="s">
-        <v>164</v>
-      </c>
-      <c r="F32" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33">
-        <f>1000*0.01625</f>
-        <v>16.25</v>
-      </c>
-      <c r="D33" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" t="s">
-        <v>155</v>
-      </c>
-      <c r="F33" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" t="s">
-        <v>14</v>
-      </c>
-      <c r="E43" t="s">
-        <v>23</v>
-      </c>
-      <c r="F43" t="s">
-        <v>9</v>
-      </c>
-      <c r="G43" t="s">
-        <v>15</v>
-      </c>
-      <c r="H43" t="s">
-        <v>20</v>
-      </c>
-      <c r="I43" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>B38</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
-      </c>
-      <c r="B44">
-        <f>B37</f>
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" t="s">
-        <v>16</v>
-      </c>
-      <c r="F44" t="s">
-        <v>17</v>
-      </c>
-      <c r="G44" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>140</v>
-      </c>
-      <c r="B45">
-        <f>1000*1</f>
-        <v>1000</v>
-      </c>
-      <c r="C45" t="s">
-        <v>8</v>
-      </c>
-      <c r="D45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F45" t="s">
-        <v>18</v>
-      </c>
-      <c r="G45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B46">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C46" t="s">
-        <v>8</v>
-      </c>
-      <c r="D46" t="s">
-        <v>26</v>
-      </c>
-      <c r="F46" t="s">
-        <v>18</v>
-      </c>
-      <c r="G46" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>153</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" t="s">
-        <v>16</v>
-      </c>
-      <c r="F47" t="s">
-        <v>18</v>
-      </c>
-      <c r="G47" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>7</v>
-      </c>
-      <c r="B50" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>141</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>15</v>
-      </c>
-      <c r="B52" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>14</v>
-      </c>
-      <c r="B53" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>6</v>
-      </c>
-      <c r="B55" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" t="s">
-        <v>12</v>
-      </c>
-      <c r="C57" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" t="s">
-        <v>14</v>
-      </c>
-      <c r="E57" t="s">
-        <v>23</v>
-      </c>
-      <c r="F57" t="s">
-        <v>9</v>
-      </c>
-      <c r="G57" t="s">
-        <v>15</v>
-      </c>
-      <c r="H57" t="s">
-        <v>20</v>
-      </c>
-      <c r="I57" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" t="str">
-        <f>B52</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
-      </c>
-      <c r="B58">
-        <f>B51</f>
-        <v>1</v>
-      </c>
-      <c r="C58" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" t="s">
-        <v>16</v>
-      </c>
-      <c r="F58" t="s">
-        <v>17</v>
-      </c>
-      <c r="G58" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>140</v>
-      </c>
-      <c r="B59">
-        <v>0</v>
-      </c>
-      <c r="C59" t="s">
-        <v>8</v>
-      </c>
-      <c r="D59" t="s">
-        <v>26</v>
-      </c>
-      <c r="F59" t="s">
-        <v>18</v>
-      </c>
-      <c r="G59" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="B60">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C60" t="s">
-        <v>8</v>
-      </c>
-      <c r="D60" t="s">
-        <v>26</v>
-      </c>
-      <c r="F60" t="s">
-        <v>18</v>
-      </c>
-      <c r="G60" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>153</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" t="s">
-        <v>16</v>
-      </c>
-      <c r="F61" t="s">
-        <v>18</v>
-      </c>
-      <c r="G61" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-    </row>
-    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="1"/>
-    </row>
-    <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="4"/>
-    </row>
-    <row r="74" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A74" s="4"/>
-    </row>
-    <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="4"/>
-    </row>
-    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A76" s="4"/>
-      <c r="G76" s="4"/>
-    </row>
-    <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="4"/>
-    </row>
-    <row r="79" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="4"/>
-    </row>
-    <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="4"/>
-    </row>
-    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A81" s="4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF05BD3-82B5-4829-9975-BAE4BAEB41CD}">
   <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3756,9 +2877,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EFFFC2-89D0-45E5-B7FA-4B2E66075D0E}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.44140625" customWidth="1"/>
@@ -3940,6 +3061,29 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>159</v>
+      </c>
+      <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" t="s">
+        <v>162</v>
+      </c>
+      <c r="I18" t="s">
+        <v>166</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
tried to fix issue during transport transformation, didn't work so far
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D2B0F93-51E5-4662-9B5F-6A7A027D09D7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6FDD85-B1F6-4435-869C-A3C85E096D7A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="169">
   <si>
     <t>Database</t>
   </si>
@@ -1081,9 +1081,8 @@
       <c r="F12" t="s">
         <v>17</v>
       </c>
-      <c r="G12" t="str">
-        <f>A12</f>
-        <v>transport, hydrogen, gaseous, lorry, unspecified</v>
+      <c r="G12" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -1283,9 +1282,8 @@
       <c r="F27" t="s">
         <v>17</v>
       </c>
-      <c r="G27" t="str">
-        <f>A27</f>
-        <v>transport, hydrogen, liquid, lorry, unspecified</v>
+      <c r="G27" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
resolved doubling of ref-product in hydrogen transport. Added validation of matched activities to base and hydrogen.py.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6FDD85-B1F6-4435-869C-A3C85E096D7A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{311ACBD1-3D42-4228-849E-1360DB7DB079}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="167">
   <si>
     <t>Database</t>
   </si>
@@ -484,12 +484,6 @@
     <t>electricity, medium voltage</t>
   </si>
   <si>
-    <t>electricity needed for evaporation</t>
-  </si>
-  <si>
-    <t>electricity needed for liquefaction, Stoltenberg et al</t>
-  </si>
-  <si>
     <t>market for transport, freight, sea, tanker for liquefied natural gas, heavy fuel oil</t>
   </si>
   <si>
@@ -508,9 +502,6 @@
     <t>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</t>
   </si>
   <si>
-    <t>market for electricity, medium voltage</t>
-  </si>
-  <si>
     <t>LCI for hydrogen transport as liquid ammonia for 1 tkm. Storage tank taken from the hydrogen-distribution dataset. Market average. Boil-off losses are 3 % and 1.65 % during liquefaction (Reuß et al. 2019)</t>
   </si>
   <si>
@@ -523,31 +514,34 @@
     <t>RER</t>
   </si>
   <si>
-    <t>DE</t>
-  </si>
-  <si>
     <t>transport, hydrogen, gaseous, lorry, unspecified</t>
   </si>
   <si>
+    <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>this dataset is used as a proxy, so the lorry used uses the propulsion system chosen by the IAM scenario</t>
+  </si>
+  <si>
+    <t>boil-off losses to the atmosphere</t>
+  </si>
+  <si>
+    <t>compensation for boil-off losses</t>
+  </si>
+  <si>
+    <t>transport, freight, lorry, diesel, unspecified</t>
+  </si>
+  <si>
+    <t>market for transport, freight, lorry, unspecified</t>
+  </si>
+  <si>
     <t>transport, hydrogen, liquid, lorry, unspecified</t>
   </si>
   <si>
-    <t>Hydrogen</t>
-  </si>
-  <si>
-    <t>this dataset is used as a proxy, so the lorry used uses the propulsion system chosen by the IAM scenario</t>
-  </si>
-  <si>
-    <t>boil-off losses to the atmosphere</t>
-  </si>
-  <si>
-    <t>compensation for boil-off losses</t>
-  </si>
-  <si>
-    <t>transport, freight, lorry, diesel, unspecified</t>
-  </si>
-  <si>
-    <t>market for transport, freight, lorry, unspecified</t>
+    <t>electricity needed for liquefaction, Stoltenberg et al; electricity needed for evaporation</t>
+  </si>
+  <si>
+    <t>market group for electricity, medium voltage</t>
   </si>
 </sst>
 </file>
@@ -952,7 +946,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
@@ -981,7 +975,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1005,7 +999,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1082,18 +1076,18 @@
         <v>17</v>
       </c>
       <c r="G12" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
@@ -1102,10 +1096,10 @@
         <v>18</v>
       </c>
       <c r="G13" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="I13" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -1134,14 +1128,14 @@
     </row>
     <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B15">
         <f>1000*0.005</f>
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D15" t="s">
         <v>26</v>
@@ -1150,15 +1144,15 @@
         <v>18</v>
       </c>
       <c r="G15" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I15" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B16">
         <f>1000*0.005</f>
@@ -1168,13 +1162,13 @@
         <v>26</v>
       </c>
       <c r="E16" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F16" t="s">
         <v>27</v>
       </c>
       <c r="I16" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
@@ -1182,7 +1176,7 @@
         <v>2</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
@@ -1206,7 +1200,7 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -1283,18 +1277,18 @@
         <v>17</v>
       </c>
       <c r="G27" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
@@ -1303,10 +1297,10 @@
         <v>18</v>
       </c>
       <c r="G28" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="I28" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -1335,14 +1329,14 @@
     </row>
     <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B30">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
       <c r="C30" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D30" t="s">
         <v>26</v>
@@ -1351,25 +1345,25 @@
         <v>18</v>
       </c>
       <c r="G30" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I30" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>166</v>
+      </c>
+      <c r="B31">
+        <f>1000*(6.78+0.6)</f>
+        <v>7380</v>
+      </c>
+      <c r="C31" t="s">
+        <v>156</v>
+      </c>
+      <c r="D31" t="s">
         <v>155</v>
-      </c>
-      <c r="B31">
-        <f>1000*6.78</f>
-        <v>6780</v>
-      </c>
-      <c r="C31" t="s">
-        <v>160</v>
-      </c>
-      <c r="D31" t="s">
-        <v>158</v>
       </c>
       <c r="F31" t="s">
         <v>18</v>
@@ -1378,173 +1372,169 @@
         <v>146</v>
       </c>
       <c r="I31" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B32">
-        <f>1000*0.6</f>
-        <v>600</v>
-      </c>
-      <c r="C32" t="s">
-        <v>160</v>
-      </c>
-      <c r="D32" t="s">
-        <v>158</v>
-      </c>
-      <c r="F32" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>163</v>
-      </c>
-      <c r="B33">
         <f>1000*0.01625</f>
         <v>16.25</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D32" t="s">
         <v>26</v>
       </c>
-      <c r="E33" t="s">
-        <v>151</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="E32" t="s">
+        <v>149</v>
+      </c>
+      <c r="F32" t="s">
         <v>27</v>
       </c>
-      <c r="I33" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+      <c r="I32" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>8</v>
+        <v>141</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>141</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s">
-        <v>145</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
         <v>6</v>
       </c>
-      <c r="B41" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="B40" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
     </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" t="s">
+        <v>23</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>20</v>
+      </c>
+      <c r="I42" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" t="s">
-        <v>12</v>
+      <c r="A43" t="str">
+        <f>B37</f>
+        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      </c>
+      <c r="B43">
+        <f>B36</f>
+        <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D43" t="s">
-        <v>14</v>
-      </c>
-      <c r="E43" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F43" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G43" t="s">
-        <v>15</v>
-      </c>
-      <c r="H43" t="s">
-        <v>20</v>
-      </c>
-      <c r="I43" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" t="str">
-        <f>B38</f>
-        <v>transport, freight, sea, tanker for liquefied hydrogen, heavy fuel oil</v>
+      <c r="A44" t="s">
+        <v>140</v>
       </c>
       <c r="B44">
-        <f>B37</f>
-        <v>1</v>
+        <f>1000*1/540000</f>
+        <v>1.8518518518518519E-3</v>
       </c>
       <c r="C44" t="s">
         <v>8</v>
       </c>
       <c r="D44" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G44" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
         <v>140</v>
       </c>
+    </row>
+    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="B45">
-        <f>1000*1/540000</f>
-        <v>1.8518518518518519E-3</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C45" t="s">
-        <v>8</v>
+        <v>156</v>
       </c>
       <c r="D45" t="s">
         <v>26</v>
@@ -1553,167 +1543,167 @@
         <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>147</v>
       </c>
       <c r="B46">
-        <v>5.0000000000000001E-3</v>
+        <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>159</v>
+        <v>8</v>
       </c>
       <c r="D46" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F46" t="s">
         <v>18</v>
       </c>
       <c r="G46" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>149</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
-      </c>
-      <c r="C47" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" t="s">
         <v>8</v>
-      </c>
-      <c r="D47" t="s">
-        <v>16</v>
-      </c>
-      <c r="F47" t="s">
-        <v>18</v>
-      </c>
-      <c r="G47" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>7</v>
-      </c>
-      <c r="B50" t="s">
-        <v>8</v>
+        <v>141</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>141</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="B51" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B52" t="s">
-        <v>154</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>14</v>
-      </c>
-      <c r="B53" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
         <v>6</v>
       </c>
-      <c r="B55" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+      <c r="B54" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
         <v>10</v>
       </c>
     </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>11</v>
+      </c>
+      <c r="B56" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" t="s">
+        <v>14</v>
+      </c>
+      <c r="E56" t="s">
+        <v>23</v>
+      </c>
+      <c r="F56" t="s">
+        <v>9</v>
+      </c>
+      <c r="G56" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" t="s">
+        <v>20</v>
+      </c>
+      <c r="I56" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" t="s">
-        <v>12</v>
+      <c r="A57" t="str">
+        <f>B51</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      </c>
+      <c r="B57">
+        <f>B50</f>
+        <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D57" t="s">
-        <v>14</v>
-      </c>
-      <c r="E57" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F57" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G57" t="s">
-        <v>15</v>
-      </c>
-      <c r="H57" t="s">
-        <v>20</v>
-      </c>
-      <c r="I57" t="s">
-        <v>6</v>
+        <v>152</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" t="str">
-        <f>B52</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, heavy fuel oil</v>
+      <c r="A58" t="s">
+        <v>140</v>
       </c>
       <c r="B58">
-        <f>B51</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C58" t="s">
         <v>8</v>
       </c>
       <c r="D58" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G58" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
         <v>140</v>
       </c>
+    </row>
+    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
+        <v>150</v>
+      </c>
       <c r="B59">
-        <v>0</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C59" t="s">
-        <v>8</v>
+        <v>156</v>
       </c>
       <c r="D59" t="s">
         <v>26</v>
@@ -1722,55 +1712,38 @@
         <v>18</v>
       </c>
       <c r="G59" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>147</v>
       </c>
       <c r="B60">
-        <v>5.0000000000000001E-3</v>
+        <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>159</v>
+        <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F60" t="s">
         <v>18</v>
       </c>
       <c r="G60" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>149</v>
-      </c>
-      <c r="B61">
-        <v>1</v>
-      </c>
-      <c r="C61" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" t="s">
-        <v>16</v>
-      </c>
-      <c r="F61" t="s">
-        <v>18</v>
-      </c>
-      <c r="G61" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-    </row>
-    <row r="70" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="1"/>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+    </row>
+    <row r="69" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A69" s="1"/>
+    </row>
+    <row r="72" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A72" s="4"/>
     </row>
     <row r="73" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
@@ -1780,10 +1753,10 @@
     </row>
     <row r="75" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
-    </row>
-    <row r="76" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A76" s="4"/>
-      <c r="G76" s="4"/>
+      <c r="G75" s="4"/>
+    </row>
+    <row r="77" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4"/>
     </row>
     <row r="78" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
@@ -1793,9 +1766,6 @@
     </row>
     <row r="80" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
-    </row>
-    <row r="81" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A81" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
skip sector if hydrogen final energy use in that sector is zero validated that tests work fixed lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3F1925-0864-4927-A61B-FB5386ECD6F5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9CE762F-1924-4B06-9DE6-7DBB6433CE37}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
-    <sheet name="parameters" sheetId="5" r:id="rId2"/>
+    <sheet name="unused activities" sheetId="6" r:id="rId2"/>
+    <sheet name="parameters" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="144">
   <si>
     <t>Database</t>
   </si>
@@ -450,6 +451,9 @@
   </si>
   <si>
     <t>This dataset represents transporting 1 ton of liquid ammonia for 1 km using 95 % ammonia and 5 % marine gas oil (mgo) as fuel in a dual-fuel engine. Boil off gas (0.25% per day) are assumed to be reliquified, raising fuel consumption. The final product is hydrogen, gaseous, low pressure, which the electricity is needed for. Make-up hydrogen for losses is taken from the general market for hydrogen. The tanker chosen here is a 50,000 cbm vessel taken from IMO 2018, as a typical ship that size. The dataset is based on the transport, freight, sea, tanker for liquefied natural gas, heavy fuel oil dataset from ecoinvent v3. Auxiliary processes have therefore not been adapted.</t>
+  </si>
+  <si>
+    <t>RoW</t>
   </si>
 </sst>
 </file>
@@ -1700,8 +1704,8 @@
         <f>parameters!D5/1000</f>
         <v>5.0618999999999994E-3</v>
       </c>
-      <c r="C60" s="6" t="s">
-        <v>73</v>
+      <c r="C60" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>21</v>
@@ -1724,8 +1728,8 @@
       <c r="B61" s="5">
         <v>-1.2999999999999999E-5</v>
       </c>
-      <c r="C61" s="6" t="s">
-        <v>73</v>
+      <c r="C61" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>21</v>
@@ -1749,8 +1753,8 @@
         <f>parameters!D7/1000</f>
         <v>1.147E-4</v>
       </c>
-      <c r="C62" s="6" t="s">
-        <v>73</v>
+      <c r="C62" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>21</v>
@@ -1845,8 +1849,8 @@
       <c r="B66" s="5">
         <v>0</v>
       </c>
-      <c r="C66" s="6" t="s">
-        <v>73</v>
+      <c r="C66" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>21</v>
@@ -1868,8 +1872,8 @@
         <f>(parameters!D10*parameters!D6/1000)*parameters!D9</f>
         <v>1.4850480349344979E-4</v>
       </c>
-      <c r="C67" s="6" t="s">
-        <v>73</v>
+      <c r="C67" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>21</v>
@@ -1886,293 +1890,278 @@
       </c>
     </row>
     <row r="68" spans="1:8">
-      <c r="A68" s="5" t="s">
+      <c r="A68" t="s">
+        <v>83</v>
+      </c>
+      <c r="B68">
+        <v>3.0859999999999999</v>
+      </c>
+      <c r="C68" t="s">
+        <v>73</v>
+      </c>
+      <c r="D68" t="s">
+        <v>72</v>
+      </c>
+      <c r="F68" t="s">
+        <v>17</v>
+      </c>
+      <c r="G68" t="s">
+        <v>139</v>
+      </c>
+      <c r="H68" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B68" s="5">
+      <c r="B69" s="5">
         <f>((parameters!D15*parameters!D6/1000)*parameters!D9)+((parameters!D16*parameters!D6/1000)*(1-parameters!D9))</f>
         <v>4.7617641921397384E-4</v>
       </c>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E68" s="5" t="s">
+      <c r="C69" s="5"/>
+      <c r="D69" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F68" s="5" t="s">
+      <c r="F69" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G68" s="6" t="s">
+      <c r="G69" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H68" s="5"/>
-    </row>
-    <row r="69" spans="1:8">
-      <c r="A69" s="5" t="s">
+      <c r="H69" s="5"/>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B69" s="5">
+      <c r="B70" s="5">
         <f>(parameters!D22/1000)*parameters!D8</f>
         <v>3.4876800000000001E-4</v>
       </c>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E69" s="5" t="s">
+      <c r="C70" s="5"/>
+      <c r="D70" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E70" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F70" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G69" s="6" t="s">
+      <c r="G70" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H69" s="5"/>
-    </row>
-    <row r="70" spans="1:8">
-      <c r="A70" s="5" t="s">
+      <c r="H70" s="5"/>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B71" s="5">
         <f>(parameters!D24/1000)*parameters!D8</f>
         <v>2.8000000000000002E-7</v>
       </c>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E70" s="5" t="s">
+      <c r="C71" s="5"/>
+      <c r="D71" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E71" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F71" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G70" s="6" t="s">
+      <c r="G71" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="H70" s="5"/>
-    </row>
-    <row r="71" spans="1:8">
-      <c r="A71" s="5" t="s">
+      <c r="H71" s="5"/>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B71" s="5">
+      <c r="B72" s="5">
         <f>((parameters!D6*parameters!D12/1000)*parameters!D9)+((parameters!D6*parameters!D13/1000)*(1-parameters!D9))+((parameters!D8/1000)*parameters!D23)</f>
         <v>1.2346794829694324E-4</v>
       </c>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E71" s="5" t="s">
+      <c r="C72" s="5"/>
+      <c r="D72" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E72" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F72" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G71" s="6" t="s">
+      <c r="G72" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="H71" s="5"/>
-    </row>
-    <row r="72" spans="1:8">
-      <c r="A72" s="5" t="s">
+      <c r="H72" s="5"/>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B72" s="5">
+      <c r="B73" s="5">
         <f>(parameters!D8/1000)*parameters!D25</f>
         <v>1.4E-8</v>
       </c>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E72" s="5" t="s">
+      <c r="C73" s="5"/>
+      <c r="D73" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E73" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="F73" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G72" s="5" t="s">
+      <c r="G73" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H72" s="5"/>
-    </row>
-    <row r="73" spans="1:8">
-      <c r="A73" s="5" t="s">
+      <c r="H73" s="5"/>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B73" s="5">
+      <c r="B74" s="5">
         <f>parameters!D32*parameters!D8/1000</f>
         <v>1.4000000000000001E-7</v>
       </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E73" s="5" t="s">
+      <c r="C74" s="5"/>
+      <c r="D74" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F74" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G73" s="5" t="s">
+      <c r="G74" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H73" s="5"/>
-    </row>
-    <row r="74" spans="1:8">
-      <c r="A74" s="5" t="s">
+      <c r="H74" s="5"/>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B74" s="5">
+      <c r="B75" s="5">
         <f>((parameters!D6*parameters!D17/1000)*parameters!D9)+((parameters!D6*parameters!D18/1000)*(1-parameters!D9))+((parameters!D8/1000*parameters!D27)*(parameters!D9))+((parameters!D8/1000)*parameters!D28)*(1-parameters!D9)</f>
         <v>1.5558654148471616E-3</v>
       </c>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E74" s="5" t="s">
+      <c r="C75" s="5"/>
+      <c r="D75" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F75" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G74" s="6" t="s">
+      <c r="G75" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="H74" s="5"/>
-    </row>
-    <row r="75" spans="1:8">
-      <c r="A75" s="5" t="s">
+      <c r="H75" s="5"/>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B75" s="5">
+      <c r="B76" s="5">
         <f>parameters!D8*parameters!D30/1000</f>
         <v>4.3399999999999998E-8</v>
       </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E75" s="5" t="s">
+      <c r="C76" s="5"/>
+      <c r="D76" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E76" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F76" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G75" s="5" t="s">
+      <c r="G76" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H75" s="5"/>
-    </row>
-    <row r="76" spans="1:8">
-      <c r="A76" s="5" t="s">
+      <c r="H76" s="5"/>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B76" s="5">
+      <c r="B77" s="5">
         <f>parameters!D31*parameters!D8/1000</f>
         <v>4.2000000000000004E-9</v>
       </c>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E76" s="5" t="s">
+      <c r="C77" s="5"/>
+      <c r="D77" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F76" s="5" t="s">
+      <c r="F77" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G76" s="5" t="s">
+      <c r="G77" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H76" s="5"/>
-    </row>
-    <row r="77" spans="1:8">
-      <c r="A77" s="5" t="s">
+      <c r="H77" s="5"/>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B77" s="5">
+      <c r="B78" s="5">
         <f>parameters!D8*parameters!D29/1000</f>
         <v>1.2599999999999999E-7</v>
       </c>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E77" s="5" t="s">
+      <c r="C78" s="5"/>
+      <c r="D78" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F77" s="5" t="s">
+      <c r="F78" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G77" s="5" t="s">
+      <c r="G78" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H77" s="5"/>
-    </row>
-    <row r="78" spans="1:8">
-      <c r="A78" t="s">
-        <v>83</v>
-      </c>
-      <c r="B78">
-        <v>3.0859999999999999</v>
-      </c>
-      <c r="C78" t="s">
-        <v>73</v>
-      </c>
-      <c r="D78" t="s">
-        <v>72</v>
-      </c>
-      <c r="F78" t="s">
-        <v>17</v>
-      </c>
-      <c r="G78" t="s">
-        <v>139</v>
-      </c>
-      <c r="H78" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" ht="15.6">
-      <c r="A79" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B79">
-        <v>200.74</v>
-      </c>
-      <c r="C79" t="s">
-        <v>8</v>
-      </c>
-      <c r="D79" t="s">
-        <v>21</v>
-      </c>
-      <c r="F79" t="s">
-        <v>17</v>
-      </c>
-      <c r="G79" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8">
-      <c r="A80" s="5"/>
-      <c r="B80" s="5"/>
+      <c r="H78" s="5"/>
+    </row>
+    <row r="80" spans="1:8" ht="15.6">
+      <c r="A80" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>133</v>
+      </c>
       <c r="C80" s="5"/>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
+      <c r="G80" s="5"/>
       <c r="H80" s="5"/>
     </row>
-    <row r="81" spans="1:8" ht="15.6">
-      <c r="A81" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>133</v>
+    <row r="81" spans="1:8">
+      <c r="A81" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="C81" s="5"/>
       <c r="D81" s="5"/>
@@ -2183,10 +2172,10 @@
     </row>
     <row r="82" spans="1:8">
       <c r="A82" s="5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="C82" s="5"/>
       <c r="D82" s="5"/>
@@ -2197,10 +2186,10 @@
     </row>
     <row r="83" spans="1:8">
       <c r="A83" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5"/>
@@ -2209,12 +2198,12 @@
       <c r="G83" s="5"/>
       <c r="H83" s="5"/>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" ht="21" customHeight="1">
       <c r="A84" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>55</v>
+        <v>6</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="C84" s="5"/>
       <c r="D84" s="5"/>
@@ -2223,12 +2212,12 @@
       <c r="G84" s="5"/>
       <c r="H84" s="5"/>
     </row>
-    <row r="85" spans="1:8" ht="21" customHeight="1">
+    <row r="85" spans="1:8">
       <c r="A85" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B85" s="11" t="s">
-        <v>141</v>
+        <v>53</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="C85" s="5"/>
       <c r="D85" s="5"/>
@@ -2239,10 +2228,10 @@
     </row>
     <row r="86" spans="1:8">
       <c r="A86" s="5" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C86" s="5"/>
       <c r="D86" s="5"/>
@@ -2253,10 +2242,10 @@
     </row>
     <row r="87" spans="1:8">
       <c r="A87" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="B87" s="12" t="s">
+        <v>133</v>
       </c>
       <c r="C87" s="5"/>
       <c r="D87" s="5"/>
@@ -2267,10 +2256,10 @@
     </row>
     <row r="88" spans="1:8">
       <c r="A88" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B88" s="12" t="s">
-        <v>133</v>
+        <v>13</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="C88" s="5"/>
       <c r="D88" s="5"/>
@@ -2279,13 +2268,11 @@
       <c r="G88" s="5"/>
       <c r="H88" s="5"/>
     </row>
-    <row r="89" spans="1:8">
-      <c r="A89" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>15</v>
-      </c>
+    <row r="89" spans="1:8" ht="15.6">
+      <c r="A89" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B89" s="5"/>
       <c r="C89" s="5"/>
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
@@ -2293,77 +2280,89 @@
       <c r="G89" s="5"/>
       <c r="H89" s="5"/>
     </row>
-    <row r="90" spans="1:8" ht="15.6">
-      <c r="A90" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B90" s="5"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="5"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-      <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
+    <row r="90" spans="1:8">
+      <c r="A90" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="91" spans="1:8">
-      <c r="A91" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>12</v>
+      <c r="A91" s="6" t="str">
+        <f>B87</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, mgo</v>
+      </c>
+      <c r="B91" s="5">
+        <v>1</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D91" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>19</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E91" s="5"/>
       <c r="F91" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G91" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H91" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="G91" s="5"/>
+      <c r="H91" s="5" t="str">
+        <f>A91</f>
+        <v>transport, freight, sea, tanker for liquefied ammonia, mgo</v>
       </c>
     </row>
     <row r="92" spans="1:8">
-      <c r="A92" s="6" t="str">
-        <f>B88</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, mgo</v>
+      <c r="A92" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="B92" s="5">
-        <v>1</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>73</v>
       </c>
       <c r="D92" s="5" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E92" s="5"/>
       <c r="F92" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="G92" s="5"/>
-      <c r="H92" s="5" t="str">
-        <f>A92</f>
-        <v>transport, freight, sea, tanker for liquefied ammonia, mgo</v>
+        <v>17</v>
+      </c>
+      <c r="G92" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H92" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" s="5" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B93" s="5">
-        <v>0</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>73</v>
+        <v>-1.2999999999999999E-5</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>21</v>
@@ -2372,22 +2371,23 @@
       <c r="F93" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G93" s="6" t="s">
-        <v>85</v>
+      <c r="G93" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="H93" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" s="5" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B94" s="5">
-        <v>-1.2999999999999999E-5</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>73</v>
+        <f>(parameters!C7+parameters!C5)/1000</f>
+        <v>2.3197999999999999E-3</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>21</v>
@@ -2396,44 +2396,43 @@
       <c r="F94" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G94" s="5" t="s">
-        <v>38</v>
+      <c r="G94" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="H94" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B95" s="5">
-        <f>(parameters!C7+parameters!C5)/1000</f>
-        <v>2.3197999999999999E-3</v>
-      </c>
-      <c r="C95" s="6" t="s">
-        <v>73</v>
+        <v>1.0593999999999999E-11</v>
+      </c>
+      <c r="C95" s="5" t="s">
+        <v>8</v>
       </c>
       <c r="D95" s="5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E95" s="5"/>
       <c r="F95" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G95" s="6" t="s">
-        <v>86</v>
+      <c r="G95" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="H95" s="5" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" s="5" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B96" s="5">
-        <v>1.0593999999999999E-11</v>
+        <v>1.3798099999999999E-16</v>
       </c>
       <c r="C96" s="5" t="s">
         <v>8</v>
@@ -2446,18 +2445,18 @@
         <v>17</v>
       </c>
       <c r="G96" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H96" s="5" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" s="5" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="B97" s="5">
-        <v>1.3798099999999999E-16</v>
+        <v>1.0593999999999999E-11</v>
       </c>
       <c r="C97" s="5" t="s">
         <v>8</v>
@@ -2470,45 +2469,44 @@
         <v>17</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="H97" s="5" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B98" s="5">
-        <v>1.0593999999999999E-11</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>8</v>
+        <v>0</v>
+      </c>
+      <c r="C98" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D98" s="5" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E98" s="5"/>
       <c r="F98" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G98" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="G98" s="5"/>
       <c r="H98" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B99" s="5">
-        <v>0</v>
-      </c>
-      <c r="C99" s="6" t="s">
-        <v>73</v>
+        <f>(parameters!C10*parameters!C6/1000)*parameters!C9</f>
+        <v>6.4616593886462886E-6</v>
+      </c>
+      <c r="C99" s="12" t="s">
+        <v>143</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>21</v>
@@ -2517,34 +2515,34 @@
       <c r="F99" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G99" s="5"/>
+      <c r="G99" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="H99" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="100" spans="1:8">
-      <c r="A100" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B100" s="5">
-        <f>(parameters!C10*parameters!C6/1000)*parameters!C9</f>
-        <v>6.4616593886462886E-6</v>
-      </c>
-      <c r="C100" s="6" t="s">
+      <c r="A100" t="s">
+        <v>83</v>
+      </c>
+      <c r="B100">
+        <v>3.0859999999999999</v>
+      </c>
+      <c r="C100" t="s">
         <v>73</v>
       </c>
-      <c r="D100" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E100" s="5"/>
-      <c r="F100" s="5" t="s">
+      <c r="D100" t="s">
+        <v>72</v>
+      </c>
+      <c r="F100" t="s">
         <v>17</v>
       </c>
-      <c r="G100" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="H100" s="5" t="s">
-        <v>51</v>
+      <c r="G100" t="s">
+        <v>139</v>
+      </c>
+      <c r="H100" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -2784,6 +2782,41 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.6">
+      <c r="A3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3">
+        <v>200.74</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>

</xml_diff>

<commit_message>
fixed reference product in lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE685954-1C7C-498E-A374-C54D4866C558}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE06584-B89C-421D-8CE6-DEE9C06D7B80}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="173">
   <si>
     <t>Database</t>
   </si>
@@ -523,6 +523,24 @@
   </si>
   <si>
     <t>Air</t>
+  </si>
+  <si>
+    <t>steel, chromium steel 18/8</t>
+  </si>
+  <si>
+    <t>reinforcing steel</t>
+  </si>
+  <si>
+    <t>concrete, normal</t>
+  </si>
+  <si>
+    <t>copper, cathode</t>
+  </si>
+  <si>
+    <t>aluminium alloy, AlMg3</t>
+  </si>
+  <si>
+    <t>electricity, low voltage</t>
   </si>
 </sst>
 </file>
@@ -2899,7 +2917,7 @@
         <v>17</v>
       </c>
       <c r="G107" s="15" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="H107" s="15"/>
       <c r="I107" s="15"/>
@@ -3153,7 +3171,7 @@
         <v>17</v>
       </c>
       <c r="G119" s="15" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="H119" s="15"/>
       <c r="I119" s="15"/>
@@ -3179,7 +3197,7 @@
         <v>17</v>
       </c>
       <c r="G120" s="15" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="H120" s="15"/>
       <c r="I120" s="15"/>
@@ -3205,7 +3223,7 @@
         <v>17</v>
       </c>
       <c r="G121" s="15" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="H121" s="15"/>
       <c r="I121" s="15"/>
@@ -3231,7 +3249,7 @@
         <v>17</v>
       </c>
       <c r="G122" s="15" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
@@ -3257,7 +3275,7 @@
         <v>17</v>
       </c>
       <c r="G123" s="15" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="H123" s="15"/>
       <c r="I123" s="15"/>
@@ -3517,7 +3535,7 @@
         <v>17</v>
       </c>
       <c r="G135" s="15" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="H135" s="15" t="s">
         <v>159</v>

</xml_diff>

<commit_message>
small typo fix in lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE06584-B89C-421D-8CE6-DEE9C06D7B80}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED34EB59-29C9-4D95-8AC7-C87CEC8AB83B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -486,9 +486,6 @@
     <t>market for reinforcing steel</t>
   </si>
   <si>
-    <t>market group for concrete, normal</t>
-  </si>
-  <si>
     <t>cubic meter</t>
   </si>
   <si>
@@ -531,9 +528,6 @@
     <t>reinforcing steel</t>
   </si>
   <si>
-    <t>concrete, normal</t>
-  </si>
-  <si>
     <t>copper, cathode</t>
   </si>
   <si>
@@ -541,6 +535,12 @@
   </si>
   <si>
     <t>electricity, low voltage</t>
+  </si>
+  <si>
+    <t>market group for concrete, normal strength</t>
+  </si>
+  <si>
+    <t>concrete, normal strengh</t>
   </si>
 </sst>
 </file>
@@ -2917,7 +2917,7 @@
         <v>17</v>
       </c>
       <c r="G107" s="15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H107" s="15"/>
       <c r="I107" s="15"/>
@@ -3171,7 +3171,7 @@
         <v>17</v>
       </c>
       <c r="G119" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H119" s="15"/>
       <c r="I119" s="15"/>
@@ -3197,7 +3197,7 @@
         <v>17</v>
       </c>
       <c r="G120" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H120" s="15"/>
       <c r="I120" s="15"/>
@@ -3207,7 +3207,7 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="15" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="B121" s="17">
         <v>20300</v>
@@ -3216,14 +3216,14 @@
         <v>8</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E121" s="15"/>
       <c r="F121" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G121" s="15" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H121" s="15"/>
       <c r="I121" s="15"/>
@@ -3233,7 +3233,7 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B122" s="17">
         <v>150000</v>
@@ -3249,7 +3249,7 @@
         <v>17</v>
       </c>
       <c r="G122" s="15" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
@@ -3259,7 +3259,7 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B123" s="17">
         <v>140000</v>
@@ -3275,7 +3275,7 @@
         <v>17</v>
       </c>
       <c r="G123" s="15" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H123" s="15"/>
       <c r="I123" s="15"/>
@@ -3302,7 +3302,7 @@
         <v>2</v>
       </c>
       <c r="B125" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
@@ -3374,7 +3374,7 @@
         <v>14</v>
       </c>
       <c r="B129" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -3510,7 +3510,7 @@
         <v>146</v>
       </c>
       <c r="H134" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I134" s="15"/>
       <c r="J134" s="15"/>
@@ -3535,10 +3535,10 @@
         <v>17</v>
       </c>
       <c r="G135" s="15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H135" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I135" s="15"/>
       <c r="J135" s="15"/>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="G136" s="15"/>
       <c r="H136" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I136" s="15"/>
       <c r="J136" s="15"/>
@@ -3573,24 +3573,24 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B137" s="12">
         <v>3.8000000000000002E-4</v>
       </c>
       <c r="C137" s="15"/>
       <c r="D137" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E137" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F137" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G137" s="15"/>
       <c r="H137" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I137" s="15"/>
       <c r="J137" s="15"/>
@@ -3599,24 +3599,24 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B138" s="15">
         <v>9.4600000000000004E-2</v>
       </c>
       <c r="C138" s="15"/>
       <c r="D138" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E138" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F138" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G138" s="15"/>
       <c r="H138" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I138" s="15"/>
       <c r="J138" s="15"/>
@@ -3625,24 +3625,24 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B139" s="15">
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="C139" s="15"/>
       <c r="D139" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E139" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F139" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G139" s="15"/>
       <c r="H139" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I139" s="15"/>
       <c r="J139" s="15"/>

</xml_diff>

<commit_message>
added HB process and NH3 cracking to the transport lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2237D9D-3783-40A2-A110-17FBBF280CC0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92ACD2AE-E7A2-4130-BB8B-182BC46EB2C9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="207">
   <si>
     <t>Database</t>
   </si>
@@ -444,12 +444,6 @@
     <t>liquid hydrogen production</t>
   </si>
   <si>
-    <t>Extracted from Wei et al. (2025) Supporting Information, Table S21. Functional unit: 1 kg.</t>
-  </si>
-  <si>
-    <t>Wei et al. 2025 Supporting Information, Table S21; Data source: Al Ghafri, et al.17 and Wulf and Zapp.18</t>
-  </si>
-  <si>
     <t>loc</t>
   </si>
   <si>
@@ -471,12 +465,6 @@
     <t>market group for electricity, low voltage</t>
   </si>
   <si>
-    <t>Extracted from Wei et al. (2025) Supporting Information, Table S22. Functional unit: 1 unit.</t>
-  </si>
-  <si>
-    <t>Wei et al. 2025 Supporting Information, Table S22; Data source: Al Ghafri, et al.17</t>
-  </si>
-  <si>
     <t>Production exchange added to match lci-ships workbook format. Original data in Table S22.</t>
   </si>
   <si>
@@ -501,9 +489,6 @@
     <t>As in ecoinvent dataset for hydrogen compression, from low to medium pressure</t>
   </si>
   <si>
-    <t>Used as a proxy for now.</t>
-  </si>
-  <si>
     <t>air::unspecified</t>
   </si>
   <si>
@@ -541,6 +526,123 @@
   </si>
   <si>
     <t>concrete, normal strength</t>
+  </si>
+  <si>
+    <t>ammonia cracking</t>
+  </si>
+  <si>
+    <t>market for liquid storage tank, chemicals, organics</t>
+  </si>
+  <si>
+    <t>liquid storage tank, chemicals, organics</t>
+  </si>
+  <si>
+    <t>Used as a proxy for compressor</t>
+  </si>
+  <si>
+    <t>market for chemical factory, organics</t>
+  </si>
+  <si>
+    <t>chemical factory, organics</t>
+  </si>
+  <si>
+    <t>Used as the ammonia cracker facility, lifetime 50a, 28 t of NH3 cracked per day, 300d per year</t>
+  </si>
+  <si>
+    <t>Used as proxy for liquid ammonia storage at the facility before cracking,  lifetime 50a, 28 t of NH3 cracked per day, 300d per year</t>
+  </si>
+  <si>
+    <t>Size of cracker and storage taken from https://www.thyssenkrupp-uhde.com/en/ammonia-cracking</t>
+  </si>
+  <si>
+    <t>liquid ammonia production</t>
+  </si>
+  <si>
+    <t>ammonia production, liquid</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>Production exchange added to match lci-ships workbook format. Original data in Table S28.</t>
+  </si>
+  <si>
+    <t>market for hydrogen, gaseous, 25-30 bar</t>
+  </si>
+  <si>
+    <t>nitrogen, gaseous, from cryogenic distillation, without compression</t>
+  </si>
+  <si>
+    <t>ammonia synthesis catalyst</t>
+  </si>
+  <si>
+    <t>treatment of inert waste, inert material landfill</t>
+  </si>
+  <si>
+    <t>Production exchange added to match lci-ships workbook format. Original data in Table S29.</t>
+  </si>
+  <si>
+    <t>market for air separation facility</t>
+  </si>
+  <si>
+    <t>Extracted from Wei et al. (2025) Supporting Information, Table S30. Functional unit: 1 kg.</t>
+  </si>
+  <si>
+    <t>Production exchange added to match lci-ships workbook format. Original data in Table S30.</t>
+  </si>
+  <si>
+    <t>market for magnetite</t>
+  </si>
+  <si>
+    <t>market for lime</t>
+  </si>
+  <si>
+    <t>market for zeolite, powder</t>
+  </si>
+  <si>
+    <t>This activity is for ammonia conversion from hydrogen. It is an aiding activity specifically, thus there is no hydrogen itself within this activity.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S28; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S21; Data source: Al Ghafri, et al.17 and Wulf and Zapp.18, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S22; Data source: Al Ghafri, et al.17, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>Compression of 1 kg hydrogen to 250 bar for transport in lorry</t>
+  </si>
+  <si>
+    <t>Liqeufaction of 1 kg hydrogen for transport in lorry</t>
+  </si>
+  <si>
+    <t>Building a hydrogen liquefaction plant</t>
+  </si>
+  <si>
+    <t>nitrogen production via air separation</t>
+  </si>
+  <si>
+    <t>magnetite</t>
+  </si>
+  <si>
+    <t>lime</t>
+  </si>
+  <si>
+    <t>zeolite, powder</t>
+  </si>
+  <si>
+    <t>air separation facility</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S29; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S30; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671</t>
+  </si>
+  <si>
+    <t>compensation for losses: Haber-Bosch process, Shipping and cracking (pressure swing adsorption)</t>
   </si>
 </sst>
 </file>
@@ -624,7 +726,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -647,6 +749,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Prozent 2" xfId="3" xr:uid="{36DC7AD1-E470-45B6-8861-287273FFBF17}"/>
@@ -988,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:L203"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="82.7109375" customWidth="1"/>
@@ -2704,7 +2807,7 @@
         <v>6</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>140</v>
+        <v>197</v>
       </c>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -2722,7 +2825,7 @@
         <v>53</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>141</v>
+        <v>194</v>
       </c>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -2834,13 +2937,13 @@
         <v>18</v>
       </c>
       <c r="J104" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K104" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L104" s="15" t="s">
         <v>142</v>
-      </c>
-      <c r="K104" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="L104" s="15" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="105" spans="1:12">
@@ -2864,62 +2967,60 @@
         <v>139</v>
       </c>
       <c r="H105" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I105" s="15"/>
       <c r="J105" s="15"/>
       <c r="K105" s="15"/>
       <c r="L105" s="15"/>
     </row>
-    <row r="106" spans="1:12">
-      <c r="A106" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B106" s="17">
-        <v>3.4299999999999999E-9</v>
-      </c>
-      <c r="C106" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D106" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E106" s="15"/>
-      <c r="F106" s="15" t="s">
+    <row r="106" spans="1:12" ht="15.75">
+      <c r="A106" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B106">
+        <f>B109</f>
+        <v>1.6199999999999999E-2</v>
+      </c>
+      <c r="C106" t="s">
+        <v>69</v>
+      </c>
+      <c r="D106" t="s">
+        <v>21</v>
+      </c>
+      <c r="F106" t="s">
         <v>17</v>
       </c>
-      <c r="G106" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="H106" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="I106" s="15"/>
-      <c r="J106" s="15"/>
-      <c r="K106" s="15"/>
-      <c r="L106" s="15"/>
+      <c r="G106" t="s">
+        <v>67</v>
+      </c>
+      <c r="H106" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="107" spans="1:12">
       <c r="A107" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B107" s="16">
-        <v>10.5</v>
+        <v>144</v>
+      </c>
+      <c r="B107" s="17">
+        <v>3.4299999999999999E-9</v>
       </c>
       <c r="C107" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D107" s="15" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="E107" s="15"/>
       <c r="F107" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G107" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="H107" s="15"/>
+        <v>144</v>
+      </c>
+      <c r="H107" s="15" t="s">
+        <v>145</v>
+      </c>
       <c r="I107" s="15"/>
       <c r="J107" s="15"/>
       <c r="K107" s="15"/>
@@ -2927,22 +3028,24 @@
     </row>
     <row r="108" spans="1:12">
       <c r="A108" s="15" t="s">
-        <v>71</v>
+        <v>146</v>
       </c>
       <c r="B108" s="16">
-        <v>1.6199999999999999E-2</v>
-      </c>
-      <c r="C108" s="15"/>
+        <v>10.5</v>
+      </c>
+      <c r="C108" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="D108" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E108" s="12" t="s">
-        <v>30</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="E108" s="15"/>
       <c r="F108" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G108" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="G108" s="15" t="s">
+        <v>165</v>
+      </c>
       <c r="H108" s="15"/>
       <c r="I108" s="15"/>
       <c r="J108" s="15"/>
@@ -2950,12 +3053,22 @@
       <c r="L108" s="15"/>
     </row>
     <row r="109" spans="1:12">
-      <c r="A109" s="15"/>
-      <c r="B109" s="15"/>
+      <c r="A109" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B109" s="16">
+        <v>1.6199999999999999E-2</v>
+      </c>
       <c r="C109" s="15"/>
-      <c r="D109" s="15"/>
-      <c r="E109" s="15"/>
-      <c r="F109" s="15"/>
+      <c r="D109" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E109" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F109" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G109" s="15"/>
       <c r="H109" s="15"/>
       <c r="I109" s="15"/>
@@ -2964,12 +3077,8 @@
       <c r="L109" s="15"/>
     </row>
     <row r="110" spans="1:12">
-      <c r="A110" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B110" s="13" t="s">
-        <v>146</v>
-      </c>
+      <c r="A110" s="15"/>
+      <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="15"/>
       <c r="E110" s="15"/>
@@ -2983,10 +3092,10 @@
     </row>
     <row r="111" spans="1:12">
       <c r="A111" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B111" s="15" t="s">
-        <v>149</v>
+        <v>2</v>
+      </c>
+      <c r="B111" s="13" t="s">
+        <v>144</v>
       </c>
       <c r="C111" s="15"/>
       <c r="D111" s="15"/>
@@ -3001,10 +3110,10 @@
     </row>
     <row r="112" spans="1:12">
       <c r="A112" s="15" t="s">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3019,10 +3128,10 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" s="15" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>8</v>
+        <v>195</v>
       </c>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3037,10 +3146,10 @@
     </row>
     <row r="114" spans="1:12">
       <c r="A114" s="15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B114" s="15" t="s">
-        <v>146</v>
+        <v>8</v>
       </c>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -3055,10 +3164,10 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B115" s="15" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -3073,9 +3182,11 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B116" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B116" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
       <c r="E116" s="15"/>
@@ -3089,76 +3200,64 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B117" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C117" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D117" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E117" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F117" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G117" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H117" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I117" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J117" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="K117" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="L117" s="15" t="s">
-        <v>144</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B117" s="15"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="15"/>
+      <c r="E117" s="15"/>
+      <c r="F117" s="15"/>
+      <c r="G117" s="15"/>
+      <c r="H117" s="15"/>
+      <c r="I117" s="15"/>
+      <c r="J117" s="15"/>
+      <c r="K117" s="15"/>
+      <c r="L117" s="15"/>
     </row>
     <row r="118" spans="1:12">
       <c r="A118" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B118" s="16">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="B118" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D118" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E118" s="15"/>
+      <c r="E118" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F118" s="15" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G118" s="15" t="s">
-        <v>146</v>
+        <v>14</v>
       </c>
       <c r="H118" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="I118" s="15"/>
-      <c r="J118" s="15"/>
-      <c r="K118" s="15"/>
-      <c r="L118" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="I118" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J118" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K118" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L118" s="15" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="119" spans="1:12">
       <c r="A119" s="15" t="s">
-        <v>152</v>
-      </c>
-      <c r="B119" s="17">
-        <v>595000</v>
+        <v>144</v>
+      </c>
+      <c r="B119" s="16">
+        <v>1</v>
       </c>
       <c r="C119" s="15" t="s">
         <v>8</v>
@@ -3168,12 +3267,14 @@
       </c>
       <c r="E119" s="15"/>
       <c r="F119" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G119" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="H119" s="15"/>
+        <v>144</v>
+      </c>
+      <c r="H119" s="15" t="s">
+        <v>147</v>
+      </c>
       <c r="I119" s="15"/>
       <c r="J119" s="15"/>
       <c r="K119" s="15"/>
@@ -3181,10 +3282,10 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="15" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B120" s="17">
-        <v>380000</v>
+        <v>595000</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>8</v>
@@ -3197,7 +3298,7 @@
         <v>17</v>
       </c>
       <c r="G120" s="15" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="H120" s="15"/>
       <c r="I120" s="15"/>
@@ -3207,23 +3308,23 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="15" t="s">
-        <v>171</v>
+        <v>149</v>
       </c>
       <c r="B121" s="17">
-        <v>20300</v>
+        <v>380000</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D121" s="15" t="s">
-        <v>154</v>
+        <v>21</v>
       </c>
       <c r="E121" s="15"/>
       <c r="F121" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G121" s="15" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="H121" s="15"/>
       <c r="I121" s="15"/>
@@ -3233,23 +3334,23 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="15" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B122" s="17">
-        <v>150000</v>
+        <v>20300</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>21</v>
+        <v>150</v>
       </c>
       <c r="E122" s="15"/>
       <c r="F122" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G122" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
@@ -3259,10 +3360,10 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="15" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B123" s="17">
-        <v>140000</v>
+        <v>150000</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>8</v>
@@ -3275,7 +3376,7 @@
         <v>17</v>
       </c>
       <c r="G123" s="15" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="H123" s="15"/>
       <c r="I123" s="15"/>
@@ -3284,13 +3385,25 @@
       <c r="L123" s="15"/>
     </row>
     <row r="124" spans="1:12">
-      <c r="A124" s="15"/>
-      <c r="B124" s="12"/>
-      <c r="C124" s="15"/>
-      <c r="D124" s="15"/>
+      <c r="A124" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B124" s="17">
+        <v>140000</v>
+      </c>
+      <c r="C124" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D124" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="E124" s="15"/>
-      <c r="F124" s="15"/>
-      <c r="G124" s="15"/>
+      <c r="F124" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G124" s="15" t="s">
+        <v>164</v>
+      </c>
       <c r="H124" s="15"/>
       <c r="I124" s="15"/>
       <c r="J124" s="15"/>
@@ -3298,12 +3411,8 @@
       <c r="L124" s="15"/>
     </row>
     <row r="125" spans="1:12">
-      <c r="A125" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B125" s="13" t="s">
-        <v>157</v>
-      </c>
+      <c r="A125" s="15"/>
+      <c r="B125" s="12"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
       <c r="E125" s="15"/>
@@ -3317,10 +3426,10 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B126" s="15" t="s">
-        <v>140</v>
+        <v>2</v>
+      </c>
+      <c r="B126" s="13" t="s">
+        <v>153</v>
       </c>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -3335,10 +3444,10 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="15" t="s">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="B127" s="15" t="s">
-        <v>141</v>
+        <v>196</v>
       </c>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3353,10 +3462,10 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" s="15" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>8</v>
+        <v>194</v>
       </c>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3371,10 +3480,10 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" s="15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B129" s="15" t="s">
-        <v>157</v>
+        <v>8</v>
       </c>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -3389,10 +3498,10 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B130" s="15" t="s">
-        <v>21</v>
+        <v>153</v>
       </c>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -3407,9 +3516,11 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B131" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B131" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
       <c r="E131" s="15"/>
@@ -3423,148 +3534,134 @@
     </row>
     <row r="132" spans="1:12">
       <c r="A132" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="15"/>
+      <c r="E132" s="15"/>
+      <c r="F132" s="15"/>
+      <c r="G132" s="15"/>
+      <c r="H132" s="15"/>
+      <c r="I132" s="15"/>
+      <c r="J132" s="15"/>
+      <c r="K132" s="15"/>
+      <c r="L132" s="15"/>
+    </row>
+    <row r="133" spans="1:12">
+      <c r="A133" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B132" s="15" t="s">
+      <c r="B133" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C132" s="15" t="s">
+      <c r="C133" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D132" s="15" t="s">
+      <c r="D133" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E132" s="15" t="s">
+      <c r="E133" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F132" s="15" t="s">
+      <c r="F133" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G132" s="15" t="s">
+      <c r="G133" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="H132" s="15" t="s">
+      <c r="H133" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I132" s="15" t="s">
+      <c r="I133" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="J132" s="15" t="s">
+      <c r="J133" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K133" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L133" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="K132" s="15" t="s">
-        <v>143</v>
-      </c>
-      <c r="L132" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="133" spans="1:12">
-      <c r="A133" s="15" t="str">
-        <f>B129</f>
+    </row>
+    <row r="134" spans="1:12">
+      <c r="A134" s="15" t="str">
+        <f>B130</f>
         <v>gaseous hydrogen production</v>
       </c>
-      <c r="B133" s="16">
+      <c r="B134" s="16">
         <v>1</v>
       </c>
-      <c r="C133" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D133" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E133" s="15"/>
-      <c r="F133" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G133" s="15" t="str">
-        <f>B129</f>
-        <v>gaseous hydrogen production</v>
-      </c>
-      <c r="H133" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="I133" s="15"/>
-      <c r="J133" s="15"/>
-      <c r="K133" s="15"/>
-      <c r="L133" s="15"/>
-    </row>
-    <row r="134" spans="1:12">
-      <c r="A134" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B134" s="17">
-        <v>3.4299999999999999E-9</v>
-      </c>
       <c r="C134" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D134" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E134" s="15"/>
       <c r="F134" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G134" s="15" t="s">
-        <v>146</v>
+        <v>16</v>
+      </c>
+      <c r="G134" s="15" t="str">
+        <f>B130</f>
+        <v>gaseous hydrogen production</v>
       </c>
       <c r="H134" s="15" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="I134" s="15"/>
       <c r="J134" s="15"/>
       <c r="K134" s="15"/>
       <c r="L134" s="15"/>
     </row>
-    <row r="135" spans="1:12">
-      <c r="A135" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B135" s="16">
-        <v>1.25</v>
-      </c>
-      <c r="C135" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D135" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E135" s="15"/>
-      <c r="F135" s="15" t="s">
+    <row r="135" spans="1:12" ht="15.75">
+      <c r="A135" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B135">
+        <f>B138</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C135" t="s">
+        <v>8</v>
+      </c>
+      <c r="D135" t="s">
+        <v>21</v>
+      </c>
+      <c r="F135" t="s">
         <v>17</v>
       </c>
-      <c r="G135" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="H135" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="I135" s="15"/>
-      <c r="J135" s="15"/>
-      <c r="K135" s="15"/>
-      <c r="L135" s="15"/>
+      <c r="G135" t="s">
+        <v>67</v>
+      </c>
+      <c r="H135" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="136" spans="1:12">
       <c r="A136" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B136" s="16">
-        <v>1.6199999999999999E-2</v>
-      </c>
-      <c r="C136" s="15"/>
+        <v>144</v>
+      </c>
+      <c r="B136" s="17">
+        <v>3.4299999999999999E-9</v>
+      </c>
+      <c r="C136" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="D136" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E136" s="12" t="s">
-        <v>30</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E136" s="15"/>
       <c r="F136" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G136" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="G136" s="15" t="s">
+        <v>144</v>
+      </c>
       <c r="H136" s="15" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="I136" s="15"/>
       <c r="J136" s="15"/>
@@ -3573,24 +3670,26 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B137" s="16">
+        <v>1.25</v>
+      </c>
+      <c r="C137" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D137" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E137" s="15"/>
+      <c r="F137" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G137" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="B137" s="12">
-        <v>3.8000000000000002E-4</v>
-      </c>
-      <c r="C137" s="15"/>
-      <c r="D137" s="15" t="s">
+      <c r="H137" s="15" t="s">
         <v>154</v>
-      </c>
-      <c r="E137" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="F137" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G137" s="15"/>
-      <c r="H137" s="15" t="s">
-        <v>158</v>
       </c>
       <c r="I137" s="15"/>
       <c r="J137" s="15"/>
@@ -3599,24 +3698,24 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="B138" s="15">
-        <v>9.4600000000000004E-2</v>
+        <v>71</v>
+      </c>
+      <c r="B138" s="16">
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C138" s="15"/>
       <c r="D138" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="E138" s="15" t="s">
-        <v>161</v>
+        <v>21</v>
+      </c>
+      <c r="E138" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F138" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G138" s="15"/>
       <c r="H138" s="15" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I138" s="15"/>
       <c r="J138" s="15"/>
@@ -3625,24 +3724,24 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="B139" s="15">
-        <v>9.5000000000000001E-2</v>
+        <v>160</v>
+      </c>
+      <c r="B139" s="12">
+        <v>3.8000000000000002E-4</v>
       </c>
       <c r="C139" s="15"/>
       <c r="D139" s="15" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E139" s="15" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="F139" s="15" t="s">
         <v>22</v>
       </c>
       <c r="G139" s="15"/>
       <c r="H139" s="15" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I139" s="15"/>
       <c r="J139" s="15"/>
@@ -3650,28 +3749,52 @@
       <c r="L139" s="15"/>
     </row>
     <row r="140" spans="1:12">
-      <c r="A140" s="15"/>
-      <c r="B140" s="15"/>
+      <c r="A140" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="B140" s="15">
+        <v>9.4600000000000004E-2</v>
+      </c>
       <c r="C140" s="15"/>
-      <c r="D140" s="15"/>
-      <c r="E140" s="15"/>
-      <c r="F140" s="15"/>
+      <c r="D140" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E140" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="F140" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G140" s="15"/>
-      <c r="H140" s="15"/>
+      <c r="H140" s="15" t="s">
+        <v>154</v>
+      </c>
       <c r="I140" s="15"/>
       <c r="J140" s="15"/>
       <c r="K140" s="15"/>
       <c r="L140" s="15"/>
     </row>
     <row r="141" spans="1:12">
-      <c r="A141" s="15"/>
-      <c r="B141" s="15"/>
+      <c r="A141" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B141" s="15">
+        <v>9.5000000000000001E-2</v>
+      </c>
       <c r="C141" s="15"/>
-      <c r="D141" s="15"/>
-      <c r="E141" s="15"/>
-      <c r="F141" s="15"/>
+      <c r="D141" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="E141" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F141" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G141" s="15"/>
-      <c r="H141" s="15"/>
+      <c r="H141" s="15" t="s">
+        <v>154</v>
+      </c>
       <c r="I141" s="15"/>
       <c r="J141" s="15"/>
       <c r="K141" s="15"/>
@@ -3692,8 +3815,12 @@
       <c r="L142" s="15"/>
     </row>
     <row r="143" spans="1:12">
-      <c r="A143" s="15"/>
-      <c r="B143" s="15"/>
+      <c r="A143" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143" s="13" t="s">
+        <v>168</v>
+      </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
       <c r="E143" s="15"/>
@@ -3705,110 +3832,974 @@
       <c r="K143" s="15"/>
       <c r="L143" s="15"/>
     </row>
-    <row r="144" spans="1:12" ht="15.75">
-      <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
-      <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
-      <c r="F144" s="2"/>
-      <c r="G144" s="2"/>
-      <c r="H144" s="2"/>
-      <c r="I144" s="2"/>
-      <c r="J144" s="2"/>
-      <c r="K144" s="2"/>
-      <c r="L144" s="2"/>
-    </row>
-    <row r="145" spans="1:11" ht="15.75">
-      <c r="A145" s="2"/>
-      <c r="B145" s="2"/>
-      <c r="C145" s="2"/>
-      <c r="D145" s="2"/>
-      <c r="E145" s="2"/>
-      <c r="F145" s="2"/>
-      <c r="G145" s="2"/>
-      <c r="H145" s="2"/>
-      <c r="I145" s="2"/>
-      <c r="J145" s="2"/>
-      <c r="K145" s="2"/>
-    </row>
-    <row r="146" spans="1:11" ht="15.75">
-      <c r="A146" s="2"/>
-      <c r="B146" s="2"/>
-      <c r="C146" s="2"/>
-      <c r="D146" s="2"/>
-      <c r="E146" s="2"/>
-      <c r="F146" s="2"/>
-      <c r="G146" s="2"/>
-      <c r="H146" s="2"/>
-      <c r="I146" s="2"/>
-      <c r="J146" s="2"/>
-      <c r="K146" s="2"/>
-    </row>
-    <row r="147" spans="1:11" ht="15.75">
-      <c r="A147" s="2"/>
-      <c r="B147" s="2"/>
-      <c r="C147" s="2"/>
-      <c r="D147" s="2"/>
-      <c r="E147" s="2"/>
-      <c r="F147" s="2"/>
-      <c r="G147" s="2"/>
-      <c r="H147" s="2"/>
-      <c r="I147" s="2"/>
-      <c r="J147" s="2"/>
-      <c r="K147" s="2"/>
-    </row>
-    <row r="148" spans="1:11" ht="15.75">
-      <c r="A148" s="2"/>
-      <c r="B148" s="2"/>
-      <c r="C148" s="2"/>
-      <c r="D148" s="2"/>
-      <c r="E148" s="2"/>
-      <c r="F148" s="2"/>
-      <c r="G148" s="2"/>
-      <c r="H148" s="2"/>
-      <c r="I148" s="2"/>
-      <c r="J148" s="2"/>
-      <c r="K148" s="2"/>
-    </row>
-    <row r="149" spans="1:11" ht="15.75">
-      <c r="A149" s="2"/>
-      <c r="B149" s="2"/>
-      <c r="C149" s="2"/>
-      <c r="D149" s="2"/>
-      <c r="E149" s="2"/>
-      <c r="F149" s="2"/>
-      <c r="G149" s="2"/>
-      <c r="H149" s="2"/>
-      <c r="I149" s="2"/>
-      <c r="J149" s="2"/>
-      <c r="K149" s="2"/>
-    </row>
-    <row r="150" spans="1:11" ht="15.75">
-      <c r="A150" s="2"/>
-      <c r="B150" s="2"/>
-      <c r="C150" s="2"/>
-      <c r="D150" s="2"/>
-      <c r="E150" s="2"/>
-      <c r="F150" s="2"/>
-      <c r="G150" s="2"/>
-      <c r="H150" s="2"/>
-      <c r="I150" s="2"/>
-      <c r="J150" s="2"/>
-      <c r="K150" s="2"/>
-    </row>
-    <row r="151" spans="1:11" ht="15.75">
-      <c r="A151" s="2"/>
-      <c r="B151" s="2"/>
-      <c r="C151" s="2"/>
-      <c r="D151" s="2"/>
-      <c r="E151" s="2"/>
-      <c r="F151" s="2"/>
-      <c r="G151" s="2"/>
-      <c r="H151" s="2"/>
-      <c r="I151" s="2"/>
-      <c r="J151" s="2"/>
-      <c r="K151" s="2"/>
+    <row r="144" spans="1:12">
+      <c r="A144" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B144" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="C144" s="15"/>
+      <c r="D144" s="15"/>
+      <c r="E144" s="15"/>
+      <c r="F144" s="15"/>
+      <c r="G144" s="15"/>
+      <c r="H144" s="15"/>
+      <c r="I144" s="15"/>
+      <c r="J144" s="15"/>
+      <c r="K144" s="15"/>
+      <c r="L144" s="15"/>
+    </row>
+    <row r="145" spans="1:12">
+      <c r="A145" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B145" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="C145" s="15"/>
+      <c r="D145" s="15"/>
+      <c r="E145" s="15"/>
+      <c r="F145" s="15"/>
+      <c r="G145" s="15"/>
+      <c r="H145" s="15"/>
+      <c r="I145" s="15"/>
+      <c r="J145" s="15"/>
+      <c r="K145" s="15"/>
+      <c r="L145" s="15"/>
+    </row>
+    <row r="146" spans="1:12">
+      <c r="A146" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B146" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="15"/>
+      <c r="F146" s="15"/>
+      <c r="G146" s="15"/>
+      <c r="H146" s="15"/>
+      <c r="I146" s="15"/>
+      <c r="J146" s="15"/>
+      <c r="K146" s="15"/>
+      <c r="L146" s="15"/>
+    </row>
+    <row r="147" spans="1:12">
+      <c r="A147" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B147" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="C147" s="15"/>
+      <c r="D147" s="15"/>
+      <c r="E147" s="15"/>
+      <c r="F147" s="15"/>
+      <c r="G147" s="15"/>
+      <c r="H147" s="15"/>
+      <c r="I147" s="15"/>
+      <c r="J147" s="15"/>
+      <c r="K147" s="15"/>
+      <c r="L147" s="15"/>
+    </row>
+    <row r="148" spans="1:12">
+      <c r="A148" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B148" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C148" s="15"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="15"/>
+      <c r="F148" s="15"/>
+      <c r="G148" s="15"/>
+      <c r="H148" s="15"/>
+      <c r="I148" s="15"/>
+      <c r="J148" s="15"/>
+      <c r="K148" s="15"/>
+      <c r="L148" s="15"/>
+    </row>
+    <row r="149" spans="1:12">
+      <c r="A149" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15"/>
+      <c r="F149" s="15"/>
+      <c r="G149" s="15"/>
+      <c r="H149" s="15"/>
+      <c r="I149" s="15"/>
+      <c r="J149" s="15"/>
+      <c r="K149" s="15"/>
+      <c r="L149" s="15"/>
+    </row>
+    <row r="150" spans="1:12">
+      <c r="A150" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B150" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C150" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D150" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E150" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F150" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G150" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H150" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I150" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J150" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K150" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L150" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12">
+      <c r="A151" s="15" t="str">
+        <f>B147</f>
+        <v>ammonia cracking</v>
+      </c>
+      <c r="B151" s="16">
+        <v>1</v>
+      </c>
+      <c r="C151" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D151" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E151" s="15"/>
+      <c r="F151" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G151" s="15" t="str">
+        <f>B147</f>
+        <v>ammonia cracking</v>
+      </c>
+      <c r="H151" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="I151" s="15"/>
+      <c r="J151" s="15"/>
+      <c r="K151" s="15"/>
+      <c r="L151" s="15"/>
+    </row>
+    <row r="152" spans="1:12" ht="15.75">
+      <c r="A152" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B152">
+        <v>0.35</v>
+      </c>
+      <c r="C152" t="s">
+        <v>8</v>
+      </c>
+      <c r="D152" t="s">
+        <v>21</v>
+      </c>
+      <c r="F152" t="s">
+        <v>17</v>
+      </c>
+      <c r="G152" t="s">
+        <v>67</v>
+      </c>
+      <c r="H152" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12">
+      <c r="A153" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B153" s="17">
+        <f>1/(28*300*50)</f>
+        <v>2.3809523809523808E-6</v>
+      </c>
+      <c r="C153" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D153" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E153" s="15"/>
+      <c r="F153" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G153" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="H153" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="I153" s="15"/>
+      <c r="J153" s="15"/>
+      <c r="K153" s="15"/>
+      <c r="L153" s="15"/>
+    </row>
+    <row r="154" spans="1:12">
+      <c r="A154" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="B154" s="17">
+        <f>1/(28*300*50)</f>
+        <v>2.3809523809523808E-6</v>
+      </c>
+      <c r="C154" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D154" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E154" s="15"/>
+      <c r="F154" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G154" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="H154" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="I154" s="15"/>
+      <c r="J154" s="15"/>
+      <c r="K154" s="15"/>
+      <c r="L154" s="15"/>
+    </row>
+    <row r="155" spans="1:12">
+      <c r="A155" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B155" s="16">
+        <v>0.6</v>
+      </c>
+      <c r="C155" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D155" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E155" s="15"/>
+      <c r="F155" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G155" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="H155" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="I155" s="15"/>
+      <c r="J155" s="15"/>
+      <c r="K155" s="15"/>
+      <c r="L155" s="15"/>
+    </row>
+    <row r="157" spans="1:12">
+      <c r="A157" t="s">
+        <v>2</v>
+      </c>
+      <c r="B157" s="13" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12">
+      <c r="A158" t="s">
+        <v>6</v>
+      </c>
+      <c r="B158" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="159" spans="1:12">
+      <c r="A159" t="s">
+        <v>53</v>
+      </c>
+      <c r="B159" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12">
+      <c r="A160" t="s">
+        <v>7</v>
+      </c>
+      <c r="B160" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12">
+      <c r="A161" t="s">
+        <v>14</v>
+      </c>
+      <c r="B161" t="str">
+        <f>B157</f>
+        <v>liquid ammonia production</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12">
+      <c r="A162" t="s">
+        <v>13</v>
+      </c>
+      <c r="B162" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12">
+      <c r="A163" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12">
+      <c r="A164" t="s">
+        <v>11</v>
+      </c>
+      <c r="B164" t="s">
+        <v>12</v>
+      </c>
+      <c r="C164" t="s">
+        <v>7</v>
+      </c>
+      <c r="D164" t="s">
+        <v>13</v>
+      </c>
+      <c r="E164" t="s">
+        <v>19</v>
+      </c>
+      <c r="F164" t="s">
+        <v>9</v>
+      </c>
+      <c r="G164" t="s">
+        <v>14</v>
+      </c>
+      <c r="H164" t="s">
+        <v>6</v>
+      </c>
+      <c r="I164" t="s">
+        <v>18</v>
+      </c>
+      <c r="J164" t="s">
+        <v>140</v>
+      </c>
+      <c r="K164" t="s">
+        <v>141</v>
+      </c>
+      <c r="L164" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12">
+      <c r="A165" t="str">
+        <f>B161</f>
+        <v>liquid ammonia production</v>
+      </c>
+      <c r="B165" s="18">
+        <v>1</v>
+      </c>
+      <c r="C165" t="s">
+        <v>8</v>
+      </c>
+      <c r="D165" t="s">
+        <v>13</v>
+      </c>
+      <c r="F165" t="s">
+        <v>16</v>
+      </c>
+      <c r="G165" t="s">
+        <v>178</v>
+      </c>
+      <c r="H165" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12">
+      <c r="A166" t="s">
+        <v>182</v>
+      </c>
+      <c r="B166" s="18">
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="C166" t="s">
+        <v>8</v>
+      </c>
+      <c r="D166" t="s">
+        <v>21</v>
+      </c>
+      <c r="F166" t="s">
+        <v>17</v>
+      </c>
+      <c r="G166" t="s">
+        <v>182</v>
+      </c>
+      <c r="H166" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12">
+      <c r="A167" t="s">
+        <v>183</v>
+      </c>
+      <c r="B167" s="18">
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C167" t="s">
+        <v>8</v>
+      </c>
+      <c r="D167" t="s">
+        <v>21</v>
+      </c>
+      <c r="F167" t="s">
+        <v>17</v>
+      </c>
+      <c r="G167" t="s">
+        <v>183</v>
+      </c>
+      <c r="H167" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12">
+      <c r="A168" t="s">
+        <v>172</v>
+      </c>
+      <c r="B168" s="18">
+        <v>3.29E-10</v>
+      </c>
+      <c r="C168" t="s">
+        <v>8</v>
+      </c>
+      <c r="D168" t="s">
+        <v>13</v>
+      </c>
+      <c r="F168" t="s">
+        <v>17</v>
+      </c>
+      <c r="G168" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12">
+      <c r="A169" t="s">
+        <v>146</v>
+      </c>
+      <c r="B169" s="18">
+        <v>1.44</v>
+      </c>
+      <c r="C169" t="s">
+        <v>8</v>
+      </c>
+      <c r="D169" t="s">
+        <v>68</v>
+      </c>
+      <c r="F169" t="s">
+        <v>17</v>
+      </c>
+      <c r="G169" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12">
+      <c r="A170" t="s">
+        <v>184</v>
+      </c>
+      <c r="B170" s="18">
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C170" t="s">
+        <v>8</v>
+      </c>
+      <c r="D170" t="s">
+        <v>21</v>
+      </c>
+      <c r="F170" t="s">
+        <v>17</v>
+      </c>
+      <c r="G170" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12">
+      <c r="A171" t="s">
+        <v>158</v>
+      </c>
+      <c r="B171" s="18">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="D171" t="s">
+        <v>150</v>
+      </c>
+      <c r="E171" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F171" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="172" spans="1:12">
+      <c r="A172" t="s">
+        <v>71</v>
+      </c>
+      <c r="B172" s="18">
+        <v>7.67E-4</v>
+      </c>
+      <c r="D172" t="s">
+        <v>21</v>
+      </c>
+      <c r="E172" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F172" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12">
+      <c r="A173" t="s">
+        <v>20</v>
+      </c>
+      <c r="B173" s="18">
+        <v>1.6299999999999999E-3</v>
+      </c>
+      <c r="D173" t="s">
+        <v>21</v>
+      </c>
+      <c r="E173" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F173" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12">
+      <c r="A174" t="s">
+        <v>25</v>
+      </c>
+      <c r="B174" s="18">
+        <v>1E-3</v>
+      </c>
+      <c r="D174" t="s">
+        <v>21</v>
+      </c>
+      <c r="E174" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F174" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12">
+      <c r="A175" t="s">
+        <v>157</v>
+      </c>
+      <c r="B175" s="18">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="D175" t="s">
+        <v>150</v>
+      </c>
+      <c r="E175" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F175" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12">
+      <c r="A176" t="s">
+        <v>157</v>
+      </c>
+      <c r="B176" s="18">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="D176" t="s">
+        <v>150</v>
+      </c>
+      <c r="E176" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="F176" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12">
+      <c r="A178" t="s">
+        <v>2</v>
+      </c>
+      <c r="B178" s="13" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12">
+      <c r="A179" t="s">
+        <v>6</v>
+      </c>
+      <c r="B179" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12">
+      <c r="A180" t="s">
+        <v>53</v>
+      </c>
+      <c r="B180" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12">
+      <c r="A181" t="s">
+        <v>7</v>
+      </c>
+      <c r="B181" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12">
+      <c r="A182" t="s">
+        <v>14</v>
+      </c>
+      <c r="B182" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12">
+      <c r="A183" t="s">
+        <v>13</v>
+      </c>
+      <c r="B183" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12">
+      <c r="A184" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12">
+      <c r="A185" t="s">
+        <v>11</v>
+      </c>
+      <c r="B185" t="s">
+        <v>12</v>
+      </c>
+      <c r="C185" t="s">
+        <v>7</v>
+      </c>
+      <c r="D185" t="s">
+        <v>13</v>
+      </c>
+      <c r="E185" t="s">
+        <v>19</v>
+      </c>
+      <c r="F185" t="s">
+        <v>9</v>
+      </c>
+      <c r="G185" t="s">
+        <v>14</v>
+      </c>
+      <c r="H185" t="s">
+        <v>6</v>
+      </c>
+      <c r="I185" t="s">
+        <v>18</v>
+      </c>
+      <c r="J185" t="s">
+        <v>140</v>
+      </c>
+      <c r="K185" t="s">
+        <v>141</v>
+      </c>
+      <c r="L185" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="186" spans="1:12">
+      <c r="A186" t="s">
+        <v>182</v>
+      </c>
+      <c r="B186" s="18">
+        <v>1</v>
+      </c>
+      <c r="C186" t="s">
+        <v>8</v>
+      </c>
+      <c r="D186" t="s">
+        <v>179</v>
+      </c>
+      <c r="F186" t="s">
+        <v>16</v>
+      </c>
+      <c r="G186" t="s">
+        <v>182</v>
+      </c>
+      <c r="H186" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187" spans="1:12">
+      <c r="A187" t="s">
+        <v>186</v>
+      </c>
+      <c r="B187" s="18">
+        <v>4.4300000000000002E-10</v>
+      </c>
+      <c r="C187" t="s">
+        <v>8</v>
+      </c>
+      <c r="D187" t="s">
+        <v>13</v>
+      </c>
+      <c r="F187" t="s">
+        <v>17</v>
+      </c>
+      <c r="G187" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="188" spans="1:12">
+      <c r="A188" t="s">
+        <v>158</v>
+      </c>
+      <c r="B188" s="18">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D188" t="s">
+        <v>150</v>
+      </c>
+      <c r="E188" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="F188" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12">
+      <c r="A189" t="s">
+        <v>157</v>
+      </c>
+      <c r="B189" s="18">
+        <v>2.4499999999999999E-3</v>
+      </c>
+      <c r="D189" t="s">
+        <v>150</v>
+      </c>
+      <c r="E189" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="F189" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12">
+      <c r="A191" t="s">
+        <v>2</v>
+      </c>
+      <c r="B191" s="13" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12">
+      <c r="A192" t="s">
+        <v>6</v>
+      </c>
+      <c r="B192" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12">
+      <c r="A193" t="s">
+        <v>53</v>
+      </c>
+      <c r="B193" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12">
+      <c r="A194" t="s">
+        <v>7</v>
+      </c>
+      <c r="B194" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12">
+      <c r="A195" t="s">
+        <v>14</v>
+      </c>
+      <c r="B195" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12">
+      <c r="A196" t="s">
+        <v>13</v>
+      </c>
+      <c r="B196" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12">
+      <c r="A197" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12">
+      <c r="A198" t="s">
+        <v>11</v>
+      </c>
+      <c r="B198" t="s">
+        <v>12</v>
+      </c>
+      <c r="C198" t="s">
+        <v>7</v>
+      </c>
+      <c r="D198" t="s">
+        <v>13</v>
+      </c>
+      <c r="E198" t="s">
+        <v>19</v>
+      </c>
+      <c r="F198" t="s">
+        <v>9</v>
+      </c>
+      <c r="G198" t="s">
+        <v>14</v>
+      </c>
+      <c r="H198" t="s">
+        <v>6</v>
+      </c>
+      <c r="I198" t="s">
+        <v>18</v>
+      </c>
+      <c r="J198" t="s">
+        <v>140</v>
+      </c>
+      <c r="K198" t="s">
+        <v>141</v>
+      </c>
+      <c r="L198" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="199" spans="1:12">
+      <c r="A199" t="s">
+        <v>183</v>
+      </c>
+      <c r="B199" s="18">
+        <v>1</v>
+      </c>
+      <c r="C199" t="s">
+        <v>8</v>
+      </c>
+      <c r="D199" t="s">
+        <v>179</v>
+      </c>
+      <c r="F199" t="s">
+        <v>16</v>
+      </c>
+      <c r="G199" t="s">
+        <v>183</v>
+      </c>
+      <c r="H199" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12">
+      <c r="A200" t="s">
+        <v>189</v>
+      </c>
+      <c r="B200" s="18">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="C200" t="s">
+        <v>8</v>
+      </c>
+      <c r="D200" t="s">
+        <v>21</v>
+      </c>
+      <c r="F200" t="s">
+        <v>17</v>
+      </c>
+      <c r="G200" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="201" spans="1:12">
+      <c r="A201" t="s">
+        <v>190</v>
+      </c>
+      <c r="B201" s="18">
+        <v>0.03</v>
+      </c>
+      <c r="C201" t="s">
+        <v>8</v>
+      </c>
+      <c r="D201" t="s">
+        <v>21</v>
+      </c>
+      <c r="F201" t="s">
+        <v>17</v>
+      </c>
+      <c r="G201" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12">
+      <c r="A202" t="s">
+        <v>191</v>
+      </c>
+      <c r="B202" s="18">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="C202" t="s">
+        <v>8</v>
+      </c>
+      <c r="D202" t="s">
+        <v>21</v>
+      </c>
+      <c r="F202" t="s">
+        <v>17</v>
+      </c>
+      <c r="G202" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12">
+      <c r="A203" t="s">
+        <v>146</v>
+      </c>
+      <c r="B203" s="18">
+        <v>1.78</v>
+      </c>
+      <c r="C203" t="s">
+        <v>8</v>
+      </c>
+      <c r="D203" t="s">
+        <v>68</v>
+      </c>
+      <c r="F203" t="s">
+        <v>17</v>
+      </c>
+      <c r="G203" t="s">
+        <v>165</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3818,7 +4809,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -3895,6 +4886,26 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="18">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>181</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fixed unlinked exchanges in lci
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F9404C-D1DC-4A93-9DD7-F5AB1E74CF42}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FECC368-3476-44E1-804A-C45BE22211B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="208">
   <si>
     <t>Database</t>
   </si>
@@ -594,9 +594,6 @@
     <t>market for magnetite</t>
   </si>
   <si>
-    <t>market for lime</t>
-  </si>
-  <si>
     <t>market for zeolite, powder</t>
   </si>
   <si>
@@ -627,9 +624,6 @@
     <t>magnetite</t>
   </si>
   <si>
-    <t>lime</t>
-  </si>
-  <si>
     <t>zeolite, powder</t>
   </si>
   <si>
@@ -643,6 +637,15 @@
   </si>
   <si>
     <t>compensation for losses: Haber-Bosch process, Shipping and cracking (pressure swing adsorption)</t>
+  </si>
+  <si>
+    <t>inert waste, for final disposal</t>
+  </si>
+  <si>
+    <t>hydraulic lime</t>
+  </si>
+  <si>
+    <t>market for hydraulic lime</t>
   </si>
 </sst>
 </file>
@@ -2807,7 +2810,7 @@
         <v>6</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -2825,7 +2828,7 @@
         <v>53</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -3113,7 +3116,7 @@
         <v>6</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3131,7 +3134,7 @@
         <v>53</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3185,7 +3188,7 @@
         <v>13</v>
       </c>
       <c r="B116" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -3263,7 +3266,7 @@
         <v>8</v>
       </c>
       <c r="D119" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E119" s="15"/>
       <c r="F119" s="15" t="s">
@@ -3447,7 +3450,7 @@
         <v>6</v>
       </c>
       <c r="B127" s="15" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3465,7 +3468,7 @@
         <v>53</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3855,7 +3858,7 @@
         <v>53</v>
       </c>
       <c r="B145" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
@@ -4014,7 +4017,7 @@
         <v>0.35</v>
       </c>
       <c r="C152" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D152" t="s">
         <v>21</v>
@@ -4026,7 +4029,7 @@
         <v>67</v>
       </c>
       <c r="H152" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="153" spans="1:12">
@@ -4128,7 +4131,7 @@
         <v>6</v>
       </c>
       <c r="B158" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="159" spans="1:12">
@@ -4136,7 +4139,7 @@
         <v>53</v>
       </c>
       <c r="B159" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="160" spans="1:12">
@@ -4334,7 +4337,7 @@
         <v>17</v>
       </c>
       <c r="G170" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -4452,7 +4455,7 @@
         <v>6</v>
       </c>
       <c r="B179" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="180" spans="1:12">
@@ -4460,7 +4463,7 @@
         <v>53</v>
       </c>
       <c r="B180" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="181" spans="1:12">
@@ -4570,7 +4573,7 @@
         <v>17</v>
       </c>
       <c r="G187" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="188" spans="1:12">
@@ -4628,7 +4631,7 @@
         <v>53</v>
       </c>
       <c r="B193" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="194" spans="1:12">
@@ -4738,12 +4741,12 @@
         <v>17</v>
       </c>
       <c r="G200" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="B201" s="18">
         <v>0.03</v>
@@ -4758,12 +4761,12 @@
         <v>17</v>
       </c>
       <c r="G201" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B202" s="18">
         <v>5.2499999999999998E-2</v>
@@ -4778,7 +4781,7 @@
         <v>17</v>
       </c>
       <c r="G202" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="203" spans="1:12">

</xml_diff>

<commit_message>
typo in lci fix
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF000F44-251C-4B31-95FB-2BE5AE08E0E0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB1B19D-8DF5-4699-9A20-87151F72AD46}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4222,7 +4222,7 @@
         <v>8</v>
       </c>
       <c r="D165" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F165" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
added regasification of liquid hydrogen dataset to lci and fixed infrastructure problem
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E931148-1FE1-47E0-A487-15341F0E331C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A60CD7E-5B87-40E0-B945-0187B97EB7CA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="214">
   <si>
     <t>Database</t>
   </si>
@@ -465,9 +465,6 @@
     <t>market group for electricity, low voltage</t>
   </si>
   <si>
-    <t>Production exchange added to match lci-ships workbook format. Original data in Table S22.</t>
-  </si>
-  <si>
     <t>market for steel, chromium steel 18/8</t>
   </si>
   <si>
@@ -537,9 +534,6 @@
     <t>liquid storage tank, chemicals, organics</t>
   </si>
   <si>
-    <t>Used as a proxy for compressor</t>
-  </si>
-  <si>
     <t>market for chemical factory, organics</t>
   </si>
   <si>
@@ -646,6 +640,30 @@
   </si>
   <si>
     <t>market for limestone, milled, loose</t>
+  </si>
+  <si>
+    <t>liquid hydrogen regasification</t>
+  </si>
+  <si>
+    <t>regasification of liquid hydrogen to compressed gaseous hydrogen (30 bar)</t>
+  </si>
+  <si>
+    <t>boil of losses of 0.5 % during compression</t>
+  </si>
+  <si>
+    <t>Kolb et al 2022, https://doi.org/10.1016/j.jclepro.2022.133289</t>
+  </si>
+  <si>
+    <t>compressor assembly for transmission hydrogen pipeline</t>
+  </si>
+  <si>
+    <t>compressor, for hydrogen transmission</t>
+  </si>
+  <si>
+    <t>The same compressor type as for pipeline transport is used here.</t>
+  </si>
+  <si>
+    <t>The same compressor type as for pipeline transport is used here. Note, that this might underestimate the actual size of compressor, given the higher pressures required here.</t>
   </si>
 </sst>
 </file>
@@ -1094,7 +1112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L203"/>
+  <dimension ref="A1:L216"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="82.6640625" customWidth="1"/>
@@ -2810,7 +2828,7 @@
         <v>6</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -2828,7 +2846,7 @@
         <v>53</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C99" s="15"/>
       <c r="D99" s="15"/>
@@ -3047,7 +3065,7 @@
         <v>17</v>
       </c>
       <c r="G108" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H108" s="15"/>
       <c r="I108" s="15"/>
@@ -3116,7 +3134,7 @@
         <v>6</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3134,7 +3152,7 @@
         <v>53</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3275,9 +3293,7 @@
       <c r="G119" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="H119" s="15" t="s">
-        <v>147</v>
-      </c>
+      <c r="H119" s="15"/>
       <c r="I119" s="15"/>
       <c r="J119" s="15"/>
       <c r="K119" s="15"/>
@@ -3285,7 +3301,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B120" s="17">
         <v>595000</v>
@@ -3301,7 +3317,7 @@
         <v>17</v>
       </c>
       <c r="G120" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H120" s="15"/>
       <c r="I120" s="15"/>
@@ -3311,7 +3327,7 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B121" s="17">
         <v>380000</v>
@@ -3327,7 +3343,7 @@
         <v>17</v>
       </c>
       <c r="G121" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H121" s="15"/>
       <c r="I121" s="15"/>
@@ -3337,7 +3353,7 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B122" s="17">
         <v>20300</v>
@@ -3346,14 +3362,14 @@
         <v>8</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E122" s="15"/>
       <c r="F122" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G122" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
@@ -3363,7 +3379,7 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B123" s="17">
         <v>150000</v>
@@ -3379,7 +3395,7 @@
         <v>17</v>
       </c>
       <c r="G123" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H123" s="15"/>
       <c r="I123" s="15"/>
@@ -3389,7 +3405,7 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B124" s="17">
         <v>140000</v>
@@ -3405,7 +3421,7 @@
         <v>17</v>
       </c>
       <c r="G124" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H124" s="15"/>
       <c r="I124" s="15"/>
@@ -3415,7 +3431,7 @@
     </row>
     <row r="125" spans="1:12">
       <c r="A125" s="15"/>
-      <c r="B125" s="12"/>
+      <c r="B125" s="17"/>
       <c r="C125" s="15"/>
       <c r="D125" s="15"/>
       <c r="E125" s="15"/>
@@ -3432,7 +3448,7 @@
         <v>2</v>
       </c>
       <c r="B126" s="13" t="s">
-        <v>153</v>
+        <v>206</v>
       </c>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
@@ -3450,7 +3466,7 @@
         <v>6</v>
       </c>
       <c r="B127" s="15" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3468,7 +3484,7 @@
         <v>53</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3503,8 +3519,9 @@
       <c r="A130" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B130" s="15" t="s">
-        <v>153</v>
+      <c r="B130" s="15" t="str">
+        <f>B126</f>
+        <v>liquid hydrogen regasification</v>
       </c>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -3592,7 +3609,7 @@
     <row r="134" spans="1:12">
       <c r="A134" s="15" t="str">
         <f>B130</f>
-        <v>gaseous hydrogen production</v>
+        <v>liquid hydrogen regasification</v>
       </c>
       <c r="B134" s="16">
         <v>1</v>
@@ -3609,43 +3626,44 @@
       </c>
       <c r="G134" s="15" t="str">
         <f>B130</f>
-        <v>gaseous hydrogen production</v>
-      </c>
-      <c r="H134" s="15" t="s">
-        <v>143</v>
-      </c>
+        <v>liquid hydrogen regasification</v>
+      </c>
+      <c r="H134" s="15"/>
       <c r="I134" s="15"/>
       <c r="J134" s="15"/>
       <c r="K134" s="15"/>
       <c r="L134" s="15"/>
     </row>
-    <row r="135" spans="1:12" ht="15.6">
-      <c r="A135" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B135">
-        <f>B138</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C135" t="s">
-        <v>69</v>
-      </c>
-      <c r="D135" t="s">
-        <v>21</v>
-      </c>
-      <c r="F135" t="s">
+    <row r="135" spans="1:12">
+      <c r="A135" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B135" s="16">
+        <f>0.88+0.47</f>
+        <v>1.35</v>
+      </c>
+      <c r="C135" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D135" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E135" s="15"/>
+      <c r="F135" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G135" t="s">
-        <v>67</v>
-      </c>
-      <c r="H135" t="s">
-        <v>74</v>
-      </c>
+      <c r="G135" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H135" s="15"/>
+      <c r="I135" s="15"/>
+      <c r="J135" s="15"/>
+      <c r="K135" s="15"/>
+      <c r="L135" s="15"/>
     </row>
     <row r="136" spans="1:12">
       <c r="A136" s="15" t="s">
-        <v>144</v>
+        <v>210</v>
       </c>
       <c r="B136" s="17">
         <v>3.4299999999999999E-9</v>
@@ -3660,11 +3678,11 @@
       <c r="F136" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G136" s="15" t="s">
-        <v>144</v>
+      <c r="G136" t="s">
+        <v>211</v>
       </c>
       <c r="H136" s="15" t="s">
-        <v>171</v>
+        <v>212</v>
       </c>
       <c r="I136" s="15"/>
       <c r="J136" s="15"/>
@@ -3673,26 +3691,24 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="15" t="s">
-        <v>146</v>
+        <v>71</v>
       </c>
       <c r="B137" s="16">
-        <v>1.25</v>
-      </c>
-      <c r="C137" s="15" t="s">
-        <v>8</v>
-      </c>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C137" s="15"/>
       <c r="D137" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E137" s="15"/>
+        <v>21</v>
+      </c>
+      <c r="E137" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="F137" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G137" s="15" t="s">
-        <v>165</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G137" s="15"/>
       <c r="H137" s="15" t="s">
-        <v>154</v>
+        <v>208</v>
       </c>
       <c r="I137" s="15"/>
       <c r="J137" s="15"/>
@@ -3700,26 +3716,14 @@
       <c r="L137" s="15"/>
     </row>
     <row r="138" spans="1:12">
-      <c r="A138" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B138" s="16">
-        <v>3.0000000000000001E-3</v>
-      </c>
+      <c r="A138" s="15"/>
+      <c r="B138" s="12"/>
       <c r="C138" s="15"/>
-      <c r="D138" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E138" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F138" s="15" t="s">
-        <v>22</v>
-      </c>
+      <c r="D138" s="15"/>
+      <c r="E138" s="15"/>
+      <c r="F138" s="15"/>
       <c r="G138" s="15"/>
-      <c r="H138" s="15" t="s">
-        <v>154</v>
-      </c>
+      <c r="H138" s="15"/>
       <c r="I138" s="15"/>
       <c r="J138" s="15"/>
       <c r="K138" s="15"/>
@@ -3727,25 +3731,17 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="B139" s="12">
-        <v>3.8000000000000002E-4</v>
+        <v>2</v>
+      </c>
+      <c r="B139" s="13" t="s">
+        <v>152</v>
       </c>
       <c r="C139" s="15"/>
-      <c r="D139" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E139" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="F139" s="15" t="s">
-        <v>22</v>
-      </c>
+      <c r="D139" s="15"/>
+      <c r="E139" s="15"/>
+      <c r="F139" s="15"/>
       <c r="G139" s="15"/>
-      <c r="H139" s="15" t="s">
-        <v>154</v>
-      </c>
+      <c r="H139" s="15"/>
       <c r="I139" s="15"/>
       <c r="J139" s="15"/>
       <c r="K139" s="15"/>
@@ -3753,25 +3749,17 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="B140" s="15">
-        <v>9.4600000000000004E-2</v>
+        <v>6</v>
+      </c>
+      <c r="B140" s="15" t="s">
+        <v>192</v>
       </c>
       <c r="C140" s="15"/>
-      <c r="D140" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E140" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="F140" s="15" t="s">
-        <v>22</v>
-      </c>
+      <c r="D140" s="15"/>
+      <c r="E140" s="15"/>
+      <c r="F140" s="15"/>
       <c r="G140" s="15"/>
-      <c r="H140" s="15" t="s">
-        <v>154</v>
-      </c>
+      <c r="H140" s="15"/>
       <c r="I140" s="15"/>
       <c r="J140" s="15"/>
       <c r="K140" s="15"/>
@@ -3779,33 +3767,29 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="B141" s="15">
-        <v>9.5000000000000001E-2</v>
+        <v>53</v>
+      </c>
+      <c r="B141" s="15" t="s">
+        <v>190</v>
       </c>
       <c r="C141" s="15"/>
-      <c r="D141" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E141" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="F141" s="15" t="s">
-        <v>22</v>
-      </c>
+      <c r="D141" s="15"/>
+      <c r="E141" s="15"/>
+      <c r="F141" s="15"/>
       <c r="G141" s="15"/>
-      <c r="H141" s="15" t="s">
-        <v>154</v>
-      </c>
+      <c r="H141" s="15"/>
       <c r="I141" s="15"/>
       <c r="J141" s="15"/>
       <c r="K141" s="15"/>
       <c r="L141" s="15"/>
     </row>
     <row r="142" spans="1:12">
-      <c r="A142" s="15"/>
-      <c r="B142" s="15"/>
+      <c r="A142" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B142" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
       <c r="E142" s="15"/>
@@ -3819,10 +3803,10 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B143" s="13" t="s">
-        <v>168</v>
+        <v>14</v>
+      </c>
+      <c r="B143" s="15" t="s">
+        <v>152</v>
       </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -3837,10 +3821,10 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" s="15" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B144" s="15" t="s">
-        <v>176</v>
+        <v>21</v>
       </c>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -3855,11 +3839,9 @@
     </row>
     <row r="145" spans="1:12">
       <c r="A145" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B145" s="15" t="s">
-        <v>192</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
       <c r="E145" s="15"/>
@@ -3873,35 +3855,67 @@
     </row>
     <row r="146" spans="1:12">
       <c r="A146" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B146" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C146" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B146" s="15" t="s">
+      <c r="D146" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E146" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F146" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G146" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H146" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I146" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J146" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K146" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L146" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12">
+      <c r="A147" s="15" t="str">
+        <f>B143</f>
+        <v>gaseous hydrogen production</v>
+      </c>
+      <c r="B147" s="16">
+        <v>1</v>
+      </c>
+      <c r="C147" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C146" s="15"/>
-      <c r="D146" s="15"/>
-      <c r="E146" s="15"/>
-      <c r="F146" s="15"/>
-      <c r="G146" s="15"/>
-      <c r="H146" s="15"/>
-      <c r="I146" s="15"/>
-      <c r="J146" s="15"/>
-      <c r="K146" s="15"/>
-      <c r="L146" s="15"/>
-    </row>
-    <row r="147" spans="1:12">
-      <c r="A147" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B147" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="C147" s="15"/>
-      <c r="D147" s="15"/>
+      <c r="D147" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="E147" s="15"/>
-      <c r="F147" s="15"/>
-      <c r="G147" s="15"/>
-      <c r="H147" s="15"/>
+      <c r="F147" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G147" s="15" t="str">
+        <f>B143</f>
+        <v>gaseous hydrogen production</v>
+      </c>
+      <c r="H147" s="15" t="s">
+        <v>143</v>
+      </c>
       <c r="I147" s="15"/>
       <c r="J147" s="15"/>
       <c r="K147" s="15"/>
@@ -3909,33 +3923,51 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B148" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C148" s="15"/>
-      <c r="D148" s="15"/>
-      <c r="E148" s="15"/>
-      <c r="F148" s="15"/>
-      <c r="G148" s="15"/>
-      <c r="H148" s="15"/>
-      <c r="I148" s="15"/>
-      <c r="J148" s="15"/>
-      <c r="K148" s="15"/>
-      <c r="L148" s="15"/>
+        <v>66</v>
+      </c>
+      <c r="B148">
+        <f>B151</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C148" t="s">
+        <v>69</v>
+      </c>
+      <c r="D148" t="s">
+        <v>21</v>
+      </c>
+      <c r="F148" t="s">
+        <v>17</v>
+      </c>
+      <c r="G148" t="s">
+        <v>67</v>
+      </c>
+      <c r="H148" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B149" s="15"/>
-      <c r="C149" s="15"/>
-      <c r="D149" s="15"/>
+        <v>210</v>
+      </c>
+      <c r="B149" s="17">
+        <v>3.4299999999999999E-9</v>
+      </c>
+      <c r="C149" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D149" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="E149" s="15"/>
-      <c r="F149" s="15"/>
-      <c r="G149" s="15"/>
-      <c r="H149" s="15"/>
+      <c r="F149" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G149" t="s">
+        <v>211</v>
+      </c>
+      <c r="H149" s="15" t="s">
+        <v>213</v>
+      </c>
       <c r="I149" s="15"/>
       <c r="J149" s="15"/>
       <c r="K149" s="15"/>
@@ -3943,118 +3975,104 @@
     </row>
     <row r="150" spans="1:12">
       <c r="A150" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B150" s="15" t="s">
-        <v>12</v>
+        <v>146</v>
+      </c>
+      <c r="B150" s="16">
+        <v>1.25</v>
       </c>
       <c r="C150" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E150" s="15" t="s">
-        <v>19</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="E150" s="15"/>
       <c r="F150" s="15" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G150" s="15" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="H150" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I150" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J150" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="K150" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="L150" s="15" t="s">
-        <v>142</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="I150" s="15"/>
+      <c r="J150" s="15"/>
+      <c r="K150" s="15"/>
+      <c r="L150" s="15"/>
     </row>
     <row r="151" spans="1:12">
-      <c r="A151" s="15" t="str">
-        <f>B147</f>
-        <v>ammonia cracking</v>
+      <c r="A151" s="15" t="s">
+        <v>71</v>
       </c>
       <c r="B151" s="16">
-        <v>1</v>
-      </c>
-      <c r="C151" s="15" t="s">
-        <v>8</v>
-      </c>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C151" s="15"/>
       <c r="D151" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E151" s="15"/>
+      <c r="E151" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="F151" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G151" s="15" t="str">
-        <f>B147</f>
-        <v>ammonia cracking</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G151" s="15"/>
       <c r="H151" s="15" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="I151" s="15"/>
       <c r="J151" s="15"/>
       <c r="K151" s="15"/>
       <c r="L151" s="15"/>
     </row>
-    <row r="152" spans="1:12" ht="15.6">
-      <c r="A152" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B152">
-        <v>0.35</v>
-      </c>
-      <c r="C152" t="s">
-        <v>69</v>
-      </c>
-      <c r="D152" t="s">
-        <v>21</v>
-      </c>
-      <c r="F152" t="s">
-        <v>17</v>
-      </c>
-      <c r="G152" t="s">
-        <v>67</v>
-      </c>
-      <c r="H152" t="s">
-        <v>203</v>
-      </c>
+    <row r="152" spans="1:12">
+      <c r="A152" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B152" s="12">
+        <v>3.8000000000000002E-4</v>
+      </c>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E152" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="F152" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="G152" s="15"/>
+      <c r="H152" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="I152" s="15"/>
+      <c r="J152" s="15"/>
+      <c r="K152" s="15"/>
+      <c r="L152" s="15"/>
     </row>
     <row r="153" spans="1:12">
       <c r="A153" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="B153" s="17">
-        <f>1/(28*300*50)</f>
-        <v>2.3809523809523808E-6</v>
-      </c>
-      <c r="C153" s="15" t="s">
-        <v>8</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="B153" s="15">
+        <v>9.4600000000000004E-2</v>
+      </c>
+      <c r="C153" s="15"/>
       <c r="D153" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E153" s="15"/>
+        <v>149</v>
+      </c>
+      <c r="E153" s="15" t="s">
+        <v>155</v>
+      </c>
       <c r="F153" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G153" s="15" t="s">
-        <v>170</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G153" s="15"/>
       <c r="H153" s="15" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
       <c r="I153" s="15"/>
       <c r="J153" s="15"/>
@@ -4063,27 +4081,24 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="B154" s="17">
-        <f>1/(28*300*50)</f>
-        <v>2.3809523809523808E-6</v>
-      </c>
-      <c r="C154" s="15" t="s">
-        <v>8</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="B154" s="15">
+        <v>9.5000000000000001E-2</v>
+      </c>
+      <c r="C154" s="15"/>
       <c r="D154" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E154" s="15"/>
+        <v>149</v>
+      </c>
+      <c r="E154" s="15" t="s">
+        <v>158</v>
+      </c>
       <c r="F154" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G154" s="15" t="s">
-        <v>173</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="G154" s="15"/>
       <c r="H154" s="15" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="I154" s="15"/>
       <c r="J154" s="15"/>
@@ -4091,503 +4106,622 @@
       <c r="L154" s="15"/>
     </row>
     <row r="155" spans="1:12">
-      <c r="A155" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B155" s="16">
-        <v>0.6</v>
-      </c>
-      <c r="C155" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D155" s="15" t="s">
-        <v>68</v>
-      </c>
+      <c r="A155" s="15"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="15"/>
       <c r="E155" s="15"/>
-      <c r="F155" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G155" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="H155" s="15" t="s">
-        <v>154</v>
-      </c>
+      <c r="F155" s="15"/>
+      <c r="G155" s="15"/>
+      <c r="H155" s="15"/>
       <c r="I155" s="15"/>
       <c r="J155" s="15"/>
       <c r="K155" s="15"/>
       <c r="L155" s="15"/>
     </row>
+    <row r="156" spans="1:12">
+      <c r="A156" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B156" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C156" s="15"/>
+      <c r="D156" s="15"/>
+      <c r="E156" s="15"/>
+      <c r="F156" s="15"/>
+      <c r="G156" s="15"/>
+      <c r="H156" s="15"/>
+      <c r="I156" s="15"/>
+      <c r="J156" s="15"/>
+      <c r="K156" s="15"/>
+      <c r="L156" s="15"/>
+    </row>
     <row r="157" spans="1:12">
-      <c r="A157" t="s">
-        <v>2</v>
-      </c>
-      <c r="B157" s="13" t="s">
-        <v>177</v>
-      </c>
+      <c r="A157" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B157" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C157" s="15"/>
+      <c r="D157" s="15"/>
+      <c r="E157" s="15"/>
+      <c r="F157" s="15"/>
+      <c r="G157" s="15"/>
+      <c r="H157" s="15"/>
+      <c r="I157" s="15"/>
+      <c r="J157" s="15"/>
+      <c r="K157" s="15"/>
+      <c r="L157" s="15"/>
     </row>
     <row r="158" spans="1:12">
-      <c r="A158" t="s">
+      <c r="A158" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B158" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="C158" s="15"/>
+      <c r="D158" s="15"/>
+      <c r="E158" s="15"/>
+      <c r="F158" s="15"/>
+      <c r="G158" s="15"/>
+      <c r="H158" s="15"/>
+      <c r="I158" s="15"/>
+      <c r="J158" s="15"/>
+      <c r="K158" s="15"/>
+      <c r="L158" s="15"/>
+    </row>
+    <row r="159" spans="1:12">
+      <c r="A159" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B159" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C159" s="15"/>
+      <c r="D159" s="15"/>
+      <c r="E159" s="15"/>
+      <c r="F159" s="15"/>
+      <c r="G159" s="15"/>
+      <c r="H159" s="15"/>
+      <c r="I159" s="15"/>
+      <c r="J159" s="15"/>
+      <c r="K159" s="15"/>
+      <c r="L159" s="15"/>
+    </row>
+    <row r="160" spans="1:12">
+      <c r="A160" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B160" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="C160" s="15"/>
+      <c r="D160" s="15"/>
+      <c r="E160" s="15"/>
+      <c r="F160" s="15"/>
+      <c r="G160" s="15"/>
+      <c r="H160" s="15"/>
+      <c r="I160" s="15"/>
+      <c r="J160" s="15"/>
+      <c r="K160" s="15"/>
+      <c r="L160" s="15"/>
+    </row>
+    <row r="161" spans="1:12">
+      <c r="A161" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B161" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C161" s="15"/>
+      <c r="D161" s="15"/>
+      <c r="E161" s="15"/>
+      <c r="F161" s="15"/>
+      <c r="G161" s="15"/>
+      <c r="H161" s="15"/>
+      <c r="I161" s="15"/>
+      <c r="J161" s="15"/>
+      <c r="K161" s="15"/>
+      <c r="L161" s="15"/>
+    </row>
+    <row r="162" spans="1:12">
+      <c r="A162" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="15"/>
+      <c r="E162" s="15"/>
+      <c r="F162" s="15"/>
+      <c r="G162" s="15"/>
+      <c r="H162" s="15"/>
+      <c r="I162" s="15"/>
+      <c r="J162" s="15"/>
+      <c r="K162" s="15"/>
+      <c r="L162" s="15"/>
+    </row>
+    <row r="163" spans="1:12">
+      <c r="A163" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B163" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C163" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D163" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E163" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F163" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G163" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H163" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B158" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="159" spans="1:12">
-      <c r="A159" t="s">
-        <v>53</v>
-      </c>
-      <c r="B159" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="160" spans="1:12">
-      <c r="A160" t="s">
-        <v>7</v>
-      </c>
-      <c r="B160" t="s">
+      <c r="I163" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J163" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K163" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L163" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12">
+      <c r="A164" s="15" t="str">
+        <f>B160</f>
+        <v>ammonia cracking</v>
+      </c>
+      <c r="B164" s="16">
+        <v>1</v>
+      </c>
+      <c r="C164" s="15" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="161" spans="1:12">
-      <c r="A161" t="s">
-        <v>14</v>
-      </c>
-      <c r="B161" t="str">
-        <f>B157</f>
-        <v>liquid ammonia production</v>
-      </c>
-    </row>
-    <row r="162" spans="1:12">
-      <c r="A162" t="s">
+      <c r="D164" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E164" s="15"/>
+      <c r="F164" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G164" s="15" t="str">
+        <f>B160</f>
+        <v>ammonia cracking</v>
+      </c>
+      <c r="H164" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="I164" s="15"/>
+      <c r="J164" s="15"/>
+      <c r="K164" s="15"/>
+      <c r="L164" s="15"/>
+    </row>
+    <row r="165" spans="1:12" ht="15.6">
+      <c r="A165" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B165">
+        <v>0.35</v>
+      </c>
+      <c r="C165" t="s">
+        <v>69</v>
+      </c>
+      <c r="D165" t="s">
+        <v>21</v>
+      </c>
+      <c r="F165" t="s">
+        <v>17</v>
+      </c>
+      <c r="G165" t="s">
+        <v>67</v>
+      </c>
+      <c r="H165" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12">
+      <c r="A166" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B166" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C166" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D166" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B162" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="163" spans="1:12">
-      <c r="A163" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="164" spans="1:12">
-      <c r="A164" t="s">
-        <v>11</v>
-      </c>
-      <c r="B164" t="s">
-        <v>12</v>
-      </c>
-      <c r="C164" t="s">
-        <v>7</v>
-      </c>
-      <c r="D164" t="s">
+      <c r="E166" s="15"/>
+      <c r="F166" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G166" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="H166" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="I166" s="15"/>
+      <c r="J166" s="15"/>
+      <c r="K166" s="15"/>
+      <c r="L166" s="15"/>
+    </row>
+    <row r="167" spans="1:12">
+      <c r="A167" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B167" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C167" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D167" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E164" t="s">
-        <v>19</v>
-      </c>
-      <c r="F164" t="s">
-        <v>9</v>
-      </c>
-      <c r="G164" t="s">
-        <v>14</v>
-      </c>
-      <c r="H164" t="s">
-        <v>6</v>
-      </c>
-      <c r="I164" t="s">
-        <v>18</v>
-      </c>
-      <c r="J164" t="s">
-        <v>140</v>
-      </c>
-      <c r="K164" t="s">
-        <v>141</v>
-      </c>
-      <c r="L164" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="165" spans="1:12">
-      <c r="A165" t="str">
-        <f>B161</f>
-        <v>liquid ammonia production</v>
-      </c>
-      <c r="B165" s="18">
-        <v>1</v>
-      </c>
-      <c r="C165" t="s">
+      <c r="E167" s="15"/>
+      <c r="F167" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G167" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="H167" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="I167" s="15"/>
+      <c r="J167" s="15"/>
+      <c r="K167" s="15"/>
+      <c r="L167" s="15"/>
+    </row>
+    <row r="168" spans="1:12">
+      <c r="A168" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B168" s="16">
+        <v>0.6</v>
+      </c>
+      <c r="C168" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D165" t="s">
-        <v>21</v>
-      </c>
-      <c r="F165" t="s">
-        <v>16</v>
-      </c>
-      <c r="G165" t="s">
-        <v>178</v>
-      </c>
-      <c r="H165" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="166" spans="1:12">
-      <c r="A166" t="s">
-        <v>181</v>
-      </c>
-      <c r="B166" s="18">
-        <v>0.81499999999999995</v>
-      </c>
-      <c r="C166" t="s">
-        <v>8</v>
-      </c>
-      <c r="D166" t="s">
-        <v>21</v>
-      </c>
-      <c r="F166" t="s">
+      <c r="D168" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E168" s="15"/>
+      <c r="F168" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G166" t="s">
-        <v>181</v>
-      </c>
-      <c r="H166" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="167" spans="1:12">
-      <c r="A167" t="s">
-        <v>182</v>
-      </c>
-      <c r="B167" s="18">
-        <v>5.1499999999999998E-5</v>
-      </c>
-      <c r="C167" t="s">
-        <v>8</v>
-      </c>
-      <c r="D167" t="s">
-        <v>21</v>
-      </c>
-      <c r="F167" t="s">
-        <v>17</v>
-      </c>
-      <c r="G167" t="s">
-        <v>182</v>
-      </c>
-      <c r="H167" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="168" spans="1:12">
-      <c r="A168" t="s">
-        <v>172</v>
-      </c>
-      <c r="B168" s="18">
-        <v>3.29E-10</v>
-      </c>
-      <c r="C168" t="s">
-        <v>8</v>
-      </c>
-      <c r="D168" t="s">
-        <v>13</v>
-      </c>
-      <c r="F168" t="s">
-        <v>17</v>
-      </c>
-      <c r="G168" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="169" spans="1:12">
-      <c r="A169" t="s">
-        <v>146</v>
-      </c>
-      <c r="B169" s="18">
-        <v>1.44</v>
-      </c>
-      <c r="C169" t="s">
-        <v>8</v>
-      </c>
-      <c r="D169" t="s">
-        <v>68</v>
-      </c>
-      <c r="F169" t="s">
-        <v>17</v>
-      </c>
-      <c r="G169" t="s">
-        <v>165</v>
-      </c>
+      <c r="G168" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H168" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="I168" s="15"/>
+      <c r="J168" s="15"/>
+      <c r="K168" s="15"/>
+      <c r="L168" s="15"/>
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>183</v>
-      </c>
-      <c r="B170" s="18">
-        <v>5.1499999999999998E-5</v>
-      </c>
-      <c r="C170" t="s">
-        <v>138</v>
-      </c>
-      <c r="D170" t="s">
-        <v>21</v>
-      </c>
-      <c r="F170" t="s">
-        <v>17</v>
-      </c>
-      <c r="G170" t="s">
-        <v>204</v>
+        <v>2</v>
+      </c>
+      <c r="B170" s="13" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="171" spans="1:12">
       <c r="A171" t="s">
-        <v>158</v>
-      </c>
-      <c r="B171" s="18">
-        <v>0.14899999999999999</v>
-      </c>
-      <c r="D171" t="s">
-        <v>150</v>
-      </c>
-      <c r="E171" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="F171" t="s">
-        <v>22</v>
+        <v>6</v>
+      </c>
+      <c r="B171" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="172" spans="1:12">
       <c r="A172" t="s">
-        <v>71</v>
-      </c>
-      <c r="B172" s="18">
-        <v>7.67E-4</v>
-      </c>
-      <c r="D172" t="s">
-        <v>21</v>
-      </c>
-      <c r="E172" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F172" t="s">
-        <v>22</v>
+        <v>53</v>
+      </c>
+      <c r="B172" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="173" spans="1:12">
       <c r="A173" t="s">
-        <v>20</v>
-      </c>
-      <c r="B173" s="18">
-        <v>1.6299999999999999E-3</v>
-      </c>
-      <c r="D173" t="s">
-        <v>21</v>
-      </c>
-      <c r="E173" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F173" t="s">
-        <v>22</v>
+        <v>7</v>
+      </c>
+      <c r="B173" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>25</v>
-      </c>
-      <c r="B174" s="18">
-        <v>1E-3</v>
-      </c>
-      <c r="D174" t="s">
-        <v>21</v>
-      </c>
-      <c r="E174" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F174" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="B174" t="str">
+        <f>B170</f>
+        <v>liquid ammonia production</v>
       </c>
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>157</v>
-      </c>
-      <c r="B175" s="18">
-        <v>4.7600000000000003E-2</v>
-      </c>
-      <c r="D175" t="s">
-        <v>150</v>
-      </c>
-      <c r="E175" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F175" t="s">
-        <v>22</v>
+        <v>13</v>
+      </c>
+      <c r="B175" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>157</v>
-      </c>
-      <c r="B176" s="18">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="D176" t="s">
-        <v>150</v>
-      </c>
-      <c r="E176" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="F176" t="s">
-        <v>22</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12">
+      <c r="A177" t="s">
+        <v>11</v>
+      </c>
+      <c r="B177" t="s">
+        <v>12</v>
+      </c>
+      <c r="C177" t="s">
+        <v>7</v>
+      </c>
+      <c r="D177" t="s">
+        <v>13</v>
+      </c>
+      <c r="E177" t="s">
+        <v>19</v>
+      </c>
+      <c r="F177" t="s">
+        <v>9</v>
+      </c>
+      <c r="G177" t="s">
+        <v>14</v>
+      </c>
+      <c r="H177" t="s">
+        <v>6</v>
+      </c>
+      <c r="I177" t="s">
+        <v>18</v>
+      </c>
+      <c r="J177" t="s">
+        <v>140</v>
+      </c>
+      <c r="K177" t="s">
+        <v>141</v>
+      </c>
+      <c r="L177" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="178" spans="1:12">
-      <c r="A178" t="s">
-        <v>2</v>
-      </c>
-      <c r="B178" s="13" t="s">
-        <v>181</v>
+      <c r="A178" t="str">
+        <f>B174</f>
+        <v>liquid ammonia production</v>
+      </c>
+      <c r="B178" s="18">
+        <v>1</v>
+      </c>
+      <c r="C178" t="s">
+        <v>8</v>
+      </c>
+      <c r="D178" t="s">
+        <v>21</v>
+      </c>
+      <c r="F178" t="s">
+        <v>16</v>
+      </c>
+      <c r="G178" t="s">
+        <v>176</v>
+      </c>
+      <c r="H178" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="179" spans="1:12">
       <c r="A179" t="s">
-        <v>6</v>
-      </c>
-      <c r="B179" t="s">
-        <v>197</v>
+        <v>179</v>
+      </c>
+      <c r="B179" s="18">
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="C179" t="s">
+        <v>8</v>
+      </c>
+      <c r="D179" t="s">
+        <v>21</v>
+      </c>
+      <c r="F179" t="s">
+        <v>17</v>
+      </c>
+      <c r="G179" t="s">
+        <v>179</v>
+      </c>
+      <c r="H179" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
-        <v>53</v>
-      </c>
-      <c r="B180" t="s">
-        <v>201</v>
+        <v>180</v>
+      </c>
+      <c r="B180" s="18">
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C180" t="s">
+        <v>8</v>
+      </c>
+      <c r="D180" t="s">
+        <v>21</v>
+      </c>
+      <c r="F180" t="s">
+        <v>17</v>
+      </c>
+      <c r="G180" t="s">
+        <v>180</v>
+      </c>
+      <c r="H180" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>7</v>
-      </c>
-      <c r="B181" t="s">
+        <v>170</v>
+      </c>
+      <c r="B181" s="18">
+        <v>3.29E-10</v>
+      </c>
+      <c r="C181" t="s">
         <v>8</v>
+      </c>
+      <c r="D181" t="s">
+        <v>13</v>
+      </c>
+      <c r="F181" t="s">
+        <v>17</v>
+      </c>
+      <c r="G181" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="182" spans="1:12">
       <c r="A182" t="s">
-        <v>14</v>
-      </c>
-      <c r="B182" t="s">
-        <v>181</v>
+        <v>146</v>
+      </c>
+      <c r="B182" s="18">
+        <v>1.44</v>
+      </c>
+      <c r="C182" t="s">
+        <v>8</v>
+      </c>
+      <c r="D182" t="s">
+        <v>68</v>
+      </c>
+      <c r="F182" t="s">
+        <v>17</v>
+      </c>
+      <c r="G182" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="183" spans="1:12">
       <c r="A183" t="s">
-        <v>13</v>
-      </c>
-      <c r="B183" t="s">
-        <v>21</v>
+        <v>181</v>
+      </c>
+      <c r="B183" s="18">
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C183" t="s">
+        <v>138</v>
+      </c>
+      <c r="D183" t="s">
+        <v>21</v>
+      </c>
+      <c r="F183" t="s">
+        <v>17</v>
+      </c>
+      <c r="G183" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>10</v>
+        <v>157</v>
+      </c>
+      <c r="B184" s="18">
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="D184" t="s">
+        <v>149</v>
+      </c>
+      <c r="E184" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="F184" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>11</v>
-      </c>
-      <c r="B185" t="s">
-        <v>12</v>
-      </c>
-      <c r="C185" t="s">
-        <v>7</v>
+        <v>71</v>
+      </c>
+      <c r="B185" s="18">
+        <v>7.67E-4</v>
       </c>
       <c r="D185" t="s">
-        <v>13</v>
-      </c>
-      <c r="E185" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="E185" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F185" t="s">
-        <v>9</v>
-      </c>
-      <c r="G185" t="s">
-        <v>14</v>
-      </c>
-      <c r="H185" t="s">
-        <v>6</v>
-      </c>
-      <c r="I185" t="s">
-        <v>18</v>
-      </c>
-      <c r="J185" t="s">
-        <v>140</v>
-      </c>
-      <c r="K185" t="s">
-        <v>141</v>
-      </c>
-      <c r="L185" t="s">
-        <v>142</v>
+        <v>22</v>
       </c>
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>181</v>
+        <v>20</v>
       </c>
       <c r="B186" s="18">
-        <v>1</v>
-      </c>
-      <c r="C186" t="s">
-        <v>8</v>
+        <v>1.6299999999999999E-3</v>
       </c>
       <c r="D186" t="s">
         <v>21</v>
       </c>
+      <c r="E186" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="F186" t="s">
-        <v>16</v>
-      </c>
-      <c r="G186" t="s">
-        <v>181</v>
-      </c>
-      <c r="H186" t="s">
-        <v>184</v>
+        <v>22</v>
       </c>
     </row>
     <row r="187" spans="1:12">
       <c r="A187" t="s">
-        <v>185</v>
+        <v>25</v>
       </c>
       <c r="B187" s="18">
-        <v>4.4300000000000002E-10</v>
-      </c>
-      <c r="C187" t="s">
-        <v>8</v>
+        <v>1E-3</v>
       </c>
       <c r="D187" t="s">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="E187" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F187" t="s">
-        <v>17</v>
-      </c>
-      <c r="G187" t="s">
-        <v>200</v>
+        <v>22</v>
       </c>
     </row>
     <row r="188" spans="1:12">
       <c r="A188" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B188" s="18">
-        <v>4.0000000000000001E-3</v>
+        <v>4.7600000000000003E-2</v>
       </c>
       <c r="D188" t="s">
-        <v>150</v>
-      </c>
-      <c r="E188" s="15" t="s">
-        <v>159</v>
+        <v>149</v>
+      </c>
+      <c r="E188" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F188" t="s">
         <v>22</v>
@@ -4595,16 +4729,16 @@
     </row>
     <row r="189" spans="1:12">
       <c r="A189" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B189" s="18">
-        <v>2.4499999999999999E-3</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="D189" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E189" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F189" t="s">
         <v>22</v>
@@ -4615,7 +4749,7 @@
         <v>2</v>
       </c>
       <c r="B191" s="13" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -4623,7 +4757,7 @@
         <v>6</v>
       </c>
       <c r="B192" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
     </row>
     <row r="193" spans="1:12">
@@ -4631,7 +4765,7 @@
         <v>53</v>
       </c>
       <c r="B193" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="194" spans="1:12">
@@ -4647,7 +4781,7 @@
         <v>14</v>
       </c>
       <c r="B195" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="196" spans="1:12">
@@ -4703,7 +4837,7 @@
     </row>
     <row r="199" spans="1:12">
       <c r="A199" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B199" s="18">
         <v>1</v>
@@ -4718,24 +4852,24 @@
         <v>16</v>
       </c>
       <c r="G199" t="s">
+        <v>179</v>
+      </c>
+      <c r="H199" t="s">
         <v>182</v>
-      </c>
-      <c r="H199" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B200" s="18">
-        <v>0.91700000000000004</v>
+        <v>4.4300000000000002E-10</v>
       </c>
       <c r="C200" t="s">
         <v>8</v>
       </c>
       <c r="D200" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F200" t="s">
         <v>17</v>
@@ -4746,65 +4880,233 @@
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>207</v>
+        <v>157</v>
       </c>
       <c r="B201" s="18">
-        <v>0.03</v>
-      </c>
-      <c r="C201" t="s">
-        <v>69</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="D201" t="s">
-        <v>21</v>
+        <v>149</v>
+      </c>
+      <c r="E201" s="15" t="s">
+        <v>158</v>
       </c>
       <c r="F201" t="s">
-        <v>17</v>
-      </c>
-      <c r="G201" t="s">
-        <v>205</v>
-      </c>
-      <c r="H201" t="s">
-        <v>206</v>
+        <v>22</v>
       </c>
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>189</v>
+        <v>156</v>
       </c>
       <c r="B202" s="18">
+        <v>2.4499999999999999E-3</v>
+      </c>
+      <c r="D202" t="s">
+        <v>149</v>
+      </c>
+      <c r="E202" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F202" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="204" spans="1:12">
+      <c r="A204" t="s">
+        <v>2</v>
+      </c>
+      <c r="B204" s="13" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="205" spans="1:12">
+      <c r="A205" t="s">
+        <v>6</v>
+      </c>
+      <c r="B205" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12">
+      <c r="A206" t="s">
+        <v>53</v>
+      </c>
+      <c r="B206" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12">
+      <c r="A207" t="s">
+        <v>7</v>
+      </c>
+      <c r="B207" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="208" spans="1:12">
+      <c r="A208" t="s">
+        <v>14</v>
+      </c>
+      <c r="B208" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12">
+      <c r="A209" t="s">
+        <v>13</v>
+      </c>
+      <c r="B209" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="210" spans="1:12">
+      <c r="A210" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="211" spans="1:12">
+      <c r="A211" t="s">
+        <v>11</v>
+      </c>
+      <c r="B211" t="s">
+        <v>12</v>
+      </c>
+      <c r="C211" t="s">
+        <v>7</v>
+      </c>
+      <c r="D211" t="s">
+        <v>13</v>
+      </c>
+      <c r="E211" t="s">
+        <v>19</v>
+      </c>
+      <c r="F211" t="s">
+        <v>9</v>
+      </c>
+      <c r="G211" t="s">
+        <v>14</v>
+      </c>
+      <c r="H211" t="s">
+        <v>6</v>
+      </c>
+      <c r="I211" t="s">
+        <v>18</v>
+      </c>
+      <c r="J211" t="s">
+        <v>140</v>
+      </c>
+      <c r="K211" t="s">
+        <v>141</v>
+      </c>
+      <c r="L211" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12">
+      <c r="A212" t="s">
+        <v>180</v>
+      </c>
+      <c r="B212" s="18">
+        <v>1</v>
+      </c>
+      <c r="C212" t="s">
+        <v>8</v>
+      </c>
+      <c r="D212" t="s">
+        <v>21</v>
+      </c>
+      <c r="F212" t="s">
+        <v>16</v>
+      </c>
+      <c r="G212" t="s">
+        <v>180</v>
+      </c>
+      <c r="H212" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="213" spans="1:12">
+      <c r="A213" t="s">
+        <v>186</v>
+      </c>
+      <c r="B213" s="18">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="C213" t="s">
+        <v>8</v>
+      </c>
+      <c r="D213" t="s">
+        <v>21</v>
+      </c>
+      <c r="F213" t="s">
+        <v>17</v>
+      </c>
+      <c r="G213" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12">
+      <c r="A214" t="s">
+        <v>205</v>
+      </c>
+      <c r="B214" s="18">
+        <v>0.03</v>
+      </c>
+      <c r="C214" t="s">
+        <v>69</v>
+      </c>
+      <c r="D214" t="s">
+        <v>21</v>
+      </c>
+      <c r="F214" t="s">
+        <v>17</v>
+      </c>
+      <c r="G214" t="s">
+        <v>203</v>
+      </c>
+      <c r="H214" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="215" spans="1:12">
+      <c r="A215" t="s">
+        <v>187</v>
+      </c>
+      <c r="B215" s="18">
         <v>5.2499999999999998E-2</v>
       </c>
-      <c r="C202" t="s">
+      <c r="C215" t="s">
         <v>8</v>
       </c>
-      <c r="D202" t="s">
-        <v>21</v>
-      </c>
-      <c r="F202" t="s">
+      <c r="D215" t="s">
+        <v>21</v>
+      </c>
+      <c r="F215" t="s">
         <v>17</v>
       </c>
-      <c r="G202" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="203" spans="1:12">
-      <c r="A203" t="s">
+      <c r="G215" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12">
+      <c r="A216" t="s">
         <v>146</v>
       </c>
-      <c r="B203" s="18">
+      <c r="B216" s="18">
         <v>1.78</v>
       </c>
-      <c r="C203" t="s">
+      <c r="C216" t="s">
         <v>8</v>
       </c>
-      <c r="D203" t="s">
+      <c r="D216" t="s">
         <v>68</v>
       </c>
-      <c r="F203" t="s">
+      <c r="F216" t="s">
         <v>17</v>
       </c>
-      <c r="G203" t="s">
-        <v>165</v>
+      <c r="G216" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -4895,7 +5197,7 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B6" s="18">
         <v>0.17599999999999999</v>
@@ -4910,7 +5212,7 @@
         <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed malfunction of ndb creation by adapting IAM-variable mapping for h2 FE demands. Excluded TIAM steel sector
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CD9862-F984-4106-B84E-FEC7AE169505}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A5A382-361A-458A-8F35-0EE62D7E213D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -1113,22 +1113,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L216"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="82.6640625" customWidth="1"/>
+    <col min="1" max="1" width="82.7109375" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="85.44140625" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="43.88671875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="85.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="43.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6">
+    <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6">
+    <row r="3" spans="1:9" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6">
+    <row r="10" spans="1:9" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.6">
+    <row r="13" spans="1:9" ht="15.75">
       <c r="A13" s="3" t="s">
         <v>76</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.6">
+    <row r="15" spans="1:9" ht="15.75">
       <c r="A15" s="3" t="s">
         <v>66</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6">
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6">
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6">
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" s="3" t="s">
         <v>76</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.6">
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" s="3" t="s">
         <v>66</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6">
+    <row r="33" spans="1:8" ht="15.75">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
@@ -1664,7 +1664,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="15.75">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="H63" s="5"/>
     </row>
-    <row r="65" spans="1:8" ht="15.6">
+    <row r="65" spans="1:8" ht="15.75">
       <c r="A65" s="4" t="s">
         <v>2</v>
       </c>
@@ -2298,7 +2298,7 @@
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
     </row>
-    <row r="74" spans="1:8" ht="15.6">
+    <row r="74" spans="1:8" ht="15.75">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -2995,7 +2995,7 @@
       <c r="K105" s="15"/>
       <c r="L105" s="15"/>
     </row>
-    <row r="106" spans="1:12" ht="15.6">
+    <row r="106" spans="1:12" ht="15.75">
       <c r="A106" s="3" t="s">
         <v>66</v>
       </c>
@@ -4311,7 +4311,7 @@
       <c r="K164" s="15"/>
       <c r="L164" s="15"/>
     </row>
-    <row r="165" spans="1:12" ht="15.6">
+    <row r="165" spans="1:12" ht="15.75">
       <c r="A165" s="3" t="s">
         <v>66</v>
       </c>
@@ -5118,14 +5118,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
   <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6">
+    <row r="3" spans="1:12" ht="15.75">
       <c r="A3" s="3" t="s">
         <v>66</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6">
+    <row r="4" spans="1:12" ht="15.75">
       <c r="A4" s="3" t="s">
         <v>66</v>
       </c>
@@ -5170,7 +5170,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.6">
+    <row r="5" spans="1:12" ht="15.75">
       <c r="A5" s="3" t="s">
         <v>66</v>
       </c>
@@ -5223,16 +5223,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="7"/>
-    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5546875" style="7"/>
+    <col min="1" max="1" width="11.5703125" style="7"/>
+    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5362,7 +5362,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.4">
+    <row r="9" spans="1:7" ht="15">
       <c r="B9" s="7" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
removed double counted cracking electricity
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A5A382-361A-458A-8F35-0EE62D7E213D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624E6893-72B9-4D74-9A0E-4F056784215D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="218">
   <si>
     <t>Database</t>
   </si>
@@ -591,15 +591,6 @@
     <t>This activity is for ammonia conversion from hydrogen. It is an aiding activity specifically, thus there is no hydrogen itself within this activity.</t>
   </si>
   <si>
-    <t>Wei et al. 2025 Supporting Information, Table S28; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
-  </si>
-  <si>
-    <t>Wei et al. 2025 Supporting Information, Table S21; Data source: Al Ghafri, et al.17 and Wulf and Zapp.18, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
-  </si>
-  <si>
-    <t>Wei et al. 2025 Supporting Information, Table S22; Data source: Al Ghafri, et al.17, https://doi.org/10.1016/j.resconrec.2025.108671.</t>
-  </si>
-  <si>
     <t>Compression of 1 kg hydrogen to 250 bar for transport in lorry</t>
   </si>
   <si>
@@ -621,12 +612,6 @@
     <t>air separation facility</t>
   </si>
   <si>
-    <t>Wei et al. 2025 Supporting Information, Table S29; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671</t>
-  </si>
-  <si>
-    <t>Wei et al. 2025 Supporting Information, Table S30; Data source: D’Angelo, et al.21, https://doi.org/10.1016/j.resconrec.2025.108671</t>
-  </si>
-  <si>
     <t>compensation for losses: Haber-Bosch process, Shipping and cracking (pressure swing adsorption)</t>
   </si>
   <si>
@@ -664,6 +649,33 @@
   </si>
   <si>
     <t>The same compressor type as for pipeline transport is used here. Note, that this might underestimate the actual size of compressor, given the higher pressures required here.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S28; Data source: D’Angelo, et al., https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S29; Data source: D’Angelo, et al., https://doi.org/10.1016/j.resconrec.2025.108671</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S30; Data source: D’Angelo, et al., https://doi.org/10.1016/j.resconrec.2025.108671</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S21; Data source: Al Ghafri, et al. and Wulf and Zapp., https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>Wei et al. 2025 Supporting Information, Table S22; Data source: Al Ghafri, et al., https://doi.org/10.1016/j.resconrec.2025.108671.</t>
+  </si>
+  <si>
+    <t>{"data entry": {"name": "Tobias", "email": "tobias.schliess@ier.uni-stuttgart.de"}</t>
+  </si>
+  <si>
+    <t>{"data entry": {"name": "Tobias", "email": "tobias.schliess@ier.uni-stuttgart.de"}}</t>
+  </si>
+  <si>
+    <t>This activity is for cracking of ammonia to hydrogen. It is an aiding activity specifically, thus there is no hydrogen itself within this activity.</t>
+  </si>
+  <si>
+    <t>3.086 kWh electricity needed for reconversion of 7.67 kg NH3 to 1 kg H2, used to supply the heat required and the pressure swing adsorption. An additional 0.6 kWh is needed for subsequent compression</t>
   </si>
 </sst>
 </file>
@@ -1112,23 +1124,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L216"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:L223"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="82.7109375" customWidth="1"/>
+    <col min="1" max="1" width="82.6640625" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" customWidth="1"/>
-    <col min="7" max="7" width="85.42578125" customWidth="1"/>
-    <col min="8" max="8" width="25.42578125" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
-    <col min="12" max="12" width="43.85546875" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" customWidth="1"/>
-    <col min="14" max="14" width="14.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="85.44140625" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
+    <col min="12" max="12" width="43.88671875" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
+    <row r="1" spans="1:9" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1136,7 +1149,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1177,9 +1190,18 @@
       </c>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>53</v>
-      </c>
+      <c r="A8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
@@ -1189,7 +1211,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1245,7 +1267,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.75">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="3" t="s">
         <v>76</v>
       </c>
@@ -1292,7 +1314,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.75">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="3" t="s">
         <v>66</v>
       </c>
@@ -1337,7 +1359,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75">
+    <row r="18" spans="1:9" ht="15.6">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1378,9 +1400,18 @@
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" t="s">
-        <v>53</v>
-      </c>
+      <c r="A23" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
@@ -1390,7 +1421,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1446,7 +1477,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="3" t="s">
         <v>76</v>
       </c>
@@ -1493,7 +1524,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75">
+    <row r="30" spans="1:9" ht="15.6">
       <c r="A30" s="3" t="s">
         <v>66</v>
       </c>
@@ -1538,7 +1569,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.75">
+    <row r="33" spans="1:8" ht="15.6">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
@@ -1664,7 +1695,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.75">
+    <row r="42" spans="1:8" ht="15.6">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2172,7 +2203,7 @@
       </c>
       <c r="H63" s="5"/>
     </row>
-    <row r="65" spans="1:8" ht="15.75">
+    <row r="65" spans="1:8" ht="15.6">
       <c r="A65" s="4" t="s">
         <v>2</v>
       </c>
@@ -2298,7 +2329,7 @@
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
     </row>
-    <row r="74" spans="1:8" ht="15.75">
+    <row r="74" spans="1:8" ht="15.6">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -2341,7 +2372,7 @@
         <f>B72</f>
         <v>transport, freight, sea, tanker for liquefied ammonia, mgo</v>
       </c>
-      <c r="B76" s="5">
+      <c r="B76" s="14">
         <v>1</v>
       </c>
       <c r="C76" s="5" t="s">
@@ -2364,7 +2395,7 @@
       <c r="A77" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B77" s="5">
+      <c r="B77" s="14">
         <v>0</v>
       </c>
       <c r="C77" s="6" t="s">
@@ -2388,7 +2419,7 @@
       <c r="A78" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B78" s="5">
+      <c r="B78" s="14">
         <v>-1.2999999999999999E-5</v>
       </c>
       <c r="C78" s="12" t="s">
@@ -2412,7 +2443,7 @@
       <c r="A79" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B79" s="5">
+      <c r="B79" s="14">
         <f>(parameters!C7+parameters!C5)/1000</f>
         <v>2.3197999999999999E-3</v>
       </c>
@@ -2437,7 +2468,7 @@
       <c r="A80" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B80" s="5">
+      <c r="B80" s="14">
         <v>1.0593999999999999E-11</v>
       </c>
       <c r="C80" s="5" t="s">
@@ -2457,11 +2488,11 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:12">
       <c r="A81" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B81" s="5">
+      <c r="B81" s="14">
         <v>1.3798099999999999E-16</v>
       </c>
       <c r="C81" s="5" t="s">
@@ -2481,11 +2512,11 @@
         <v>28</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:12">
       <c r="A82" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B82" s="5">
+      <c r="B82" s="14">
         <v>1.0593999999999999E-11</v>
       </c>
       <c r="C82" s="5" t="s">
@@ -2505,11 +2536,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:12">
       <c r="A83" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B83" s="5">
+      <c r="B83" s="14">
         <v>0</v>
       </c>
       <c r="C83" s="12" t="s">
@@ -2527,11 +2558,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:12">
       <c r="A84" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B84" s="5">
+      <c r="B84" s="14">
         <f>(parameters!C10*parameters!C6/1000)*parameters!C9</f>
         <v>6.4616593886462886E-6</v>
       </c>
@@ -2552,37 +2583,37 @@
         <v>51</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
-      <c r="A85" t="s">
-        <v>78</v>
-      </c>
-      <c r="B85">
-        <v>3.0859999999999999</v>
-      </c>
-      <c r="C85" t="s">
-        <v>69</v>
-      </c>
-      <c r="D85" t="s">
-        <v>68</v>
-      </c>
-      <c r="F85" t="s">
-        <v>17</v>
-      </c>
-      <c r="G85" t="s">
-        <v>134</v>
-      </c>
-      <c r="H85" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8">
-      <c r="A86" s="5" t="s">
+    <row r="85" spans="1:12">
+      <c r="A85" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B86" s="5">
+      <c r="B85" s="14">
         <f>((parameters!C15*parameters!C6/1000)*parameters!C9)+((parameters!C16*parameters!C6/1000)*(1-parameters!C9))</f>
         <v>0</v>
       </c>
+      <c r="C85" s="5"/>
+      <c r="D85" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F85" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G85" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H85" s="5"/>
+    </row>
+    <row r="86" spans="1:12">
+      <c r="A86" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B86" s="14">
+        <f>(parameters!C22/1000)*(parameters!C8+parameters!C6)</f>
+        <v>3.1887360000000002E-3</v>
+      </c>
       <c r="C86" s="5"/>
       <c r="D86" s="5" t="s">
         <v>21</v>
@@ -2594,17 +2625,17 @@
         <v>22</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H86" s="5"/>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:12">
       <c r="A87" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B87" s="5">
-        <f>(parameters!C22/1000)*(parameters!C8+parameters!C6)</f>
-        <v>3.1887360000000002E-3</v>
+        <v>32</v>
+      </c>
+      <c r="B87" s="14">
+        <f>(parameters!C24/1000)*(parameters!C8+parameters!C6)</f>
+        <v>2.5600000000000001E-6</v>
       </c>
       <c r="C87" s="5"/>
       <c r="D87" s="5" t="s">
@@ -2621,13 +2652,13 @@
       </c>
       <c r="H87" s="5"/>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:12">
       <c r="A88" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B88" s="5">
-        <f>(parameters!C24/1000)*(parameters!C8+parameters!C6)</f>
-        <v>2.5600000000000001E-6</v>
+        <v>23</v>
+      </c>
+      <c r="B88" s="14">
+        <f>(((parameters!C6+parameters!C8)/1000)*parameters!C23)</f>
+        <v>1.7408000000000001E-7</v>
       </c>
       <c r="C88" s="5"/>
       <c r="D88" s="5" t="s">
@@ -2640,17 +2671,17 @@
         <v>22</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H88" s="5"/>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:12">
       <c r="A89" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B89" s="5">
-        <f>(((parameters!C6+parameters!C8)/1000)*parameters!C23)</f>
-        <v>1.7408000000000001E-7</v>
+        <v>33</v>
+      </c>
+      <c r="B89" s="14">
+        <f>((parameters!C6+parameters!C8)/1000)*parameters!C25</f>
+        <v>1.2800000000000001E-7</v>
       </c>
       <c r="C89" s="5"/>
       <c r="D89" s="5" t="s">
@@ -2662,18 +2693,18 @@
       <c r="F89" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G89" s="6" t="s">
-        <v>85</v>
+      <c r="G89" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="H89" s="5"/>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:12">
       <c r="A90" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B90" s="5">
-        <f>((parameters!C6+parameters!C8)/1000)*parameters!C25</f>
-        <v>1.2800000000000001E-7</v>
+        <v>24</v>
+      </c>
+      <c r="B90" s="14">
+        <f>parameters!C32*(parameters!C8+parameters!C6)/1000</f>
+        <v>1.28E-6</v>
       </c>
       <c r="C90" s="5"/>
       <c r="D90" s="5" t="s">
@@ -2690,13 +2721,13 @@
       </c>
       <c r="H90" s="5"/>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:12">
       <c r="A91" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B91" s="5">
-        <f>parameters!C32*(parameters!C8+parameters!C6)/1000</f>
-        <v>1.28E-6</v>
+        <v>25</v>
+      </c>
+      <c r="B91" s="14">
+        <f>(((parameters!C8+parameters!C6)/1000)*parameters!C27)*(parameters!C9)+(((parameters!C8+parameters!C6)/1000)*parameters!C28)*(1-parameters!C9)</f>
+        <v>1.7079336244541486E-4</v>
       </c>
       <c r="C91" s="5"/>
       <c r="D91" s="5" t="s">
@@ -2708,18 +2739,18 @@
       <c r="F91" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G91" s="5" t="s">
-        <v>56</v>
+      <c r="G91" s="6" t="s">
+        <v>85</v>
       </c>
       <c r="H91" s="5"/>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:12">
       <c r="A92" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B92" s="5">
-        <f>(((parameters!C8+parameters!C6)/1000)*parameters!C27)*(parameters!C9)+(((parameters!C8+parameters!C6)/1000)*parameters!C28)*(1-parameters!C9)</f>
-        <v>1.7079336244541486E-4</v>
+        <v>26</v>
+      </c>
+      <c r="B92" s="14">
+        <f>parameters!C8*parameters!C30/1000</f>
+        <v>4.3399999999999998E-8</v>
       </c>
       <c r="C92" s="5"/>
       <c r="D92" s="5" t="s">
@@ -2731,18 +2762,18 @@
       <c r="F92" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G92" s="6" t="s">
-        <v>85</v>
+      <c r="G92" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="H92" s="5"/>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:12">
       <c r="A93" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B93" s="5">
-        <f>parameters!C8*parameters!C30/1000</f>
-        <v>4.3399999999999998E-8</v>
+        <v>34</v>
+      </c>
+      <c r="B93" s="14">
+        <f>parameters!C31*parameters!C8/1000</f>
+        <v>4.2000000000000004E-9</v>
       </c>
       <c r="C93" s="5"/>
       <c r="D93" s="5" t="s">
@@ -2759,13 +2790,13 @@
       </c>
       <c r="H93" s="5"/>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:12">
       <c r="A94" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B94" s="5">
-        <f>parameters!C31*parameters!C8/1000</f>
-        <v>4.2000000000000004E-9</v>
+        <v>35</v>
+      </c>
+      <c r="B94" s="14">
+        <f>parameters!C8*parameters!C29/1000</f>
+        <v>1.2599999999999999E-7</v>
       </c>
       <c r="C94" s="5"/>
       <c r="D94" s="5" t="s">
@@ -2782,35 +2813,30 @@
       </c>
       <c r="H94" s="5"/>
     </row>
-    <row r="95" spans="1:8">
-      <c r="A95" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B95" s="5">
-        <f>parameters!C8*parameters!C29/1000</f>
-        <v>1.2599999999999999E-7</v>
-      </c>
-      <c r="C95" s="5"/>
-      <c r="D95" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F95" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G95" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="H95" s="5"/>
+    <row r="96" spans="1:12">
+      <c r="A96" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C96" s="15"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="15"/>
+      <c r="G96" s="15"/>
+      <c r="H96" s="15"/>
+      <c r="I96" s="15"/>
+      <c r="J96" s="15"/>
+      <c r="K96" s="15"/>
+      <c r="L96" s="15"/>
     </row>
     <row r="97" spans="1:12">
       <c r="A97" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B97" s="13" t="s">
-        <v>139</v>
+        <v>6</v>
+      </c>
+      <c r="B97" s="15" t="s">
+        <v>190</v>
       </c>
       <c r="C97" s="15"/>
       <c r="D97" s="15"/>
@@ -2825,10 +2851,10 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" s="15" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B98" s="15" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="C98" s="15"/>
       <c r="D98" s="15"/>
@@ -2842,17 +2868,17 @@
       <c r="L98" s="15"/>
     </row>
     <row r="99" spans="1:12">
-      <c r="A99" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B99" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="C99" s="15"/>
-      <c r="D99" s="15"/>
-      <c r="E99" s="15"/>
-      <c r="F99" s="15"/>
-      <c r="G99" s="15"/>
+      <c r="A99" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C99" s="5"/>
+      <c r="D99" s="5"/>
+      <c r="E99" s="5"/>
+      <c r="F99" s="5"/>
+      <c r="G99" s="5"/>
       <c r="H99" s="15"/>
       <c r="I99" s="15"/>
       <c r="J99" s="15"/>
@@ -2995,7 +3021,7 @@
       <c r="K105" s="15"/>
       <c r="L105" s="15"/>
     </row>
-    <row r="106" spans="1:12" ht="15.75">
+    <row r="106" spans="1:12" ht="15.6">
       <c r="A106" s="3" t="s">
         <v>66</v>
       </c>
@@ -3134,7 +3160,7 @@
         <v>6</v>
       </c>
       <c r="B112" s="15" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C112" s="15"/>
       <c r="D112" s="15"/>
@@ -3152,7 +3178,7 @@
         <v>53</v>
       </c>
       <c r="B113" s="15" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="C113" s="15"/>
       <c r="D113" s="15"/>
@@ -3166,11 +3192,11 @@
       <c r="L113" s="15"/>
     </row>
     <row r="114" spans="1:12">
-      <c r="A114" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B114" s="15" t="s">
-        <v>8</v>
+      <c r="A114" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="C114" s="15"/>
       <c r="D114" s="15"/>
@@ -3185,10 +3211,10 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" s="15" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B115" s="15" t="s">
-        <v>144</v>
+        <v>8</v>
       </c>
       <c r="C115" s="15"/>
       <c r="D115" s="15"/>
@@ -3203,10 +3229,10 @@
     </row>
     <row r="116" spans="1:12">
       <c r="A116" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B116" s="15" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
       <c r="C116" s="15"/>
       <c r="D116" s="15"/>
@@ -3221,9 +3247,11 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B117" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B117" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="C117" s="15"/>
       <c r="D117" s="15"/>
       <c r="E117" s="15"/>
@@ -3237,87 +3265,77 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="B118" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C118" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D118" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E118" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F118" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G118" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H118" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I118" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J118" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="K118" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="L118" s="15" t="s">
-        <v>142</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B118" s="15"/>
+      <c r="C118" s="15"/>
+      <c r="D118" s="15"/>
+      <c r="E118" s="15"/>
+      <c r="F118" s="15"/>
+      <c r="G118" s="15"/>
+      <c r="H118" s="15"/>
+      <c r="I118" s="15"/>
+      <c r="J118" s="15"/>
+      <c r="K118" s="15"/>
+      <c r="L118" s="15"/>
     </row>
     <row r="119" spans="1:12">
       <c r="A119" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="B119" s="16">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="B119" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C119" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D119" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E119" s="15"/>
+      <c r="E119" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F119" s="15" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G119" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="H119" s="15"/>
-      <c r="I119" s="15"/>
-      <c r="J119" s="15"/>
-      <c r="K119" s="15"/>
-      <c r="L119" s="15"/>
+        <v>14</v>
+      </c>
+      <c r="H119" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I119" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J119" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K119" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L119" s="15" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="120" spans="1:12">
       <c r="A120" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="B120" s="17">
-        <v>595000</v>
+        <v>144</v>
+      </c>
+      <c r="B120" s="16">
+        <v>1</v>
       </c>
       <c r="C120" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D120" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E120" s="15"/>
       <c r="F120" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G120" s="15" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="H120" s="15"/>
       <c r="I120" s="15"/>
@@ -3327,10 +3345,10 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B121" s="17">
-        <v>380000</v>
+        <v>147</v>
+      </c>
+      <c r="B121" s="16">
+        <v>595000</v>
       </c>
       <c r="C121" s="15" t="s">
         <v>8</v>
@@ -3343,7 +3361,7 @@
         <v>17</v>
       </c>
       <c r="G121" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H121" s="15"/>
       <c r="I121" s="15"/>
@@ -3353,23 +3371,23 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="B122" s="17">
-        <v>20300</v>
+        <v>148</v>
+      </c>
+      <c r="B122" s="16">
+        <v>380000</v>
       </c>
       <c r="C122" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D122" s="15" t="s">
-        <v>149</v>
+        <v>21</v>
       </c>
       <c r="E122" s="15"/>
       <c r="F122" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G122" s="15" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="H122" s="15"/>
       <c r="I122" s="15"/>
@@ -3379,23 +3397,23 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="B123" s="17">
-        <v>150000</v>
+        <v>165</v>
+      </c>
+      <c r="B123" s="16">
+        <v>20300</v>
       </c>
       <c r="C123" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D123" s="15" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="E123" s="15"/>
       <c r="F123" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G123" s="15" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="H123" s="15"/>
       <c r="I123" s="15"/>
@@ -3405,10 +3423,10 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="B124" s="17">
-        <v>140000</v>
+        <v>150</v>
+      </c>
+      <c r="B124" s="16">
+        <v>150000</v>
       </c>
       <c r="C124" s="15" t="s">
         <v>8</v>
@@ -3421,7 +3439,7 @@
         <v>17</v>
       </c>
       <c r="G124" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H124" s="15"/>
       <c r="I124" s="15"/>
@@ -3430,13 +3448,25 @@
       <c r="L124" s="15"/>
     </row>
     <row r="125" spans="1:12">
-      <c r="A125" s="15"/>
-      <c r="B125" s="17"/>
-      <c r="C125" s="15"/>
-      <c r="D125" s="15"/>
+      <c r="A125" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="B125" s="16">
+        <v>140000</v>
+      </c>
+      <c r="C125" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D125" s="15" t="s">
+        <v>21</v>
+      </c>
       <c r="E125" s="15"/>
-      <c r="F125" s="15"/>
-      <c r="G125" s="15"/>
+      <c r="F125" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G125" s="15" t="s">
+        <v>163</v>
+      </c>
       <c r="H125" s="15"/>
       <c r="I125" s="15"/>
       <c r="J125" s="15"/>
@@ -3444,12 +3474,8 @@
       <c r="L125" s="15"/>
     </row>
     <row r="126" spans="1:12">
-      <c r="A126" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B126" s="13" t="s">
-        <v>206</v>
-      </c>
+      <c r="A126" s="15"/>
+      <c r="B126" s="17"/>
       <c r="C126" s="15"/>
       <c r="D126" s="15"/>
       <c r="E126" s="15"/>
@@ -3463,10 +3489,10 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B127" s="15" t="s">
-        <v>207</v>
+        <v>2</v>
+      </c>
+      <c r="B127" s="13" t="s">
+        <v>201</v>
       </c>
       <c r="C127" s="15"/>
       <c r="D127" s="15"/>
@@ -3481,10 +3507,10 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" s="15" t="s">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="B128" s="15" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C128" s="15"/>
       <c r="D128" s="15"/>
@@ -3499,10 +3525,10 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" s="15" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="B129" s="15" t="s">
-        <v>8</v>
+        <v>204</v>
       </c>
       <c r="C129" s="15"/>
       <c r="D129" s="15"/>
@@ -3516,12 +3542,11 @@
       <c r="L129" s="15"/>
     </row>
     <row r="130" spans="1:12">
-      <c r="A130" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B130" s="15" t="str">
-        <f>B126</f>
-        <v>liquid hydrogen regasification</v>
+      <c r="A130" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="C130" s="15"/>
       <c r="D130" s="15"/>
@@ -3536,10 +3561,10 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" s="15" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B131" s="15" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="C131" s="15"/>
       <c r="D131" s="15"/>
@@ -3554,9 +3579,12 @@
     </row>
     <row r="132" spans="1:12">
       <c r="A132" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B132" s="15"/>
+        <v>14</v>
+      </c>
+      <c r="B132" s="15" t="str">
+        <f>B127</f>
+        <v>liquid hydrogen regasification</v>
+      </c>
       <c r="C132" s="15"/>
       <c r="D132" s="15"/>
       <c r="E132" s="15"/>
@@ -3570,64 +3598,32 @@
     </row>
     <row r="133" spans="1:12">
       <c r="A133" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B133" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C133" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D133" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E133" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F133" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G133" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H133" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I133" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J133" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="K133" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="L133" s="15" t="s">
-        <v>142</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="C133" s="15"/>
+      <c r="D133" s="15"/>
+      <c r="E133" s="15"/>
+      <c r="F133" s="15"/>
+      <c r="G133" s="15"/>
+      <c r="H133" s="15"/>
+      <c r="I133" s="15"/>
+      <c r="J133" s="15"/>
+      <c r="K133" s="15"/>
+      <c r="L133" s="15"/>
     </row>
     <row r="134" spans="1:12">
-      <c r="A134" s="15" t="str">
-        <f>B130</f>
-        <v>liquid hydrogen regasification</v>
-      </c>
-      <c r="B134" s="16">
-        <v>1</v>
-      </c>
-      <c r="C134" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D134" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="A134" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B134" s="15"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="15"/>
       <c r="E134" s="15"/>
-      <c r="F134" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G134" s="15" t="str">
-        <f>B130</f>
-        <v>liquid hydrogen regasification</v>
-      </c>
+      <c r="F134" s="15"/>
+      <c r="G134" s="15"/>
       <c r="H134" s="15"/>
       <c r="I134" s="15"/>
       <c r="J134" s="15"/>
@@ -3636,54 +3632,65 @@
     </row>
     <row r="135" spans="1:12">
       <c r="A135" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="B135" s="16">
-        <f>0.88+0.47</f>
-        <v>1.35</v>
+        <v>11</v>
+      </c>
+      <c r="B135" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C135" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D135" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E135" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F135" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G135" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H135" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I135" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J135" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K135" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L135" s="15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12">
+      <c r="A136" s="15" t="str">
+        <f>B132</f>
+        <v>liquid hydrogen regasification</v>
+      </c>
+      <c r="B136" s="16">
+        <v>1</v>
+      </c>
+      <c r="C136" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D135" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E135" s="15"/>
-      <c r="F135" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G135" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="H135" s="15"/>
-      <c r="I135" s="15"/>
-      <c r="J135" s="15"/>
-      <c r="K135" s="15"/>
-      <c r="L135" s="15"/>
-    </row>
-    <row r="136" spans="1:12">
-      <c r="A136" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="B136" s="17">
-        <v>3.4299999999999999E-9</v>
-      </c>
-      <c r="C136" s="15" t="s">
-        <v>69</v>
-      </c>
       <c r="D136" s="15" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E136" s="15"/>
       <c r="F136" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G136" t="s">
-        <v>211</v>
-      </c>
-      <c r="H136" s="15" t="s">
-        <v>212</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G136" s="15" t="str">
+        <f>B132</f>
+        <v>liquid hydrogen regasification</v>
+      </c>
+      <c r="H136" s="15"/>
       <c r="I136" s="15"/>
       <c r="J136" s="15"/>
       <c r="K136" s="15"/>
@@ -3691,39 +3698,54 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" s="15" t="s">
-        <v>71</v>
+        <v>146</v>
       </c>
       <c r="B137" s="16">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="C137" s="15"/>
+        <f>0.88+0.47</f>
+        <v>1.35</v>
+      </c>
+      <c r="C137" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="D137" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E137" s="12" t="s">
-        <v>30</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="E137" s="15"/>
       <c r="F137" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G137" s="15"/>
-      <c r="H137" s="15" t="s">
-        <v>208</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="G137" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H137" s="15"/>
       <c r="I137" s="15"/>
       <c r="J137" s="15"/>
       <c r="K137" s="15"/>
       <c r="L137" s="15"/>
     </row>
     <row r="138" spans="1:12">
-      <c r="A138" s="15"/>
-      <c r="B138" s="12"/>
-      <c r="C138" s="15"/>
-      <c r="D138" s="15"/>
+      <c r="A138" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="B138" s="17">
+        <v>3.4299999999999999E-9</v>
+      </c>
+      <c r="C138" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D138" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="E138" s="15"/>
-      <c r="F138" s="15"/>
-      <c r="G138" s="15"/>
-      <c r="H138" s="15"/>
+      <c r="F138" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G138" t="s">
+        <v>206</v>
+      </c>
+      <c r="H138" s="15" t="s">
+        <v>207</v>
+      </c>
       <c r="I138" s="15"/>
       <c r="J138" s="15"/>
       <c r="K138" s="15"/>
@@ -3731,29 +3753,33 @@
     </row>
     <row r="139" spans="1:12">
       <c r="A139" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B139" s="13" t="s">
-        <v>152</v>
+        <v>71</v>
+      </c>
+      <c r="B139" s="16">
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="C139" s="15"/>
-      <c r="D139" s="15"/>
-      <c r="E139" s="15"/>
-      <c r="F139" s="15"/>
+      <c r="D139" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E139" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F139" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G139" s="15"/>
-      <c r="H139" s="15"/>
+      <c r="H139" s="15" t="s">
+        <v>203</v>
+      </c>
       <c r="I139" s="15"/>
       <c r="J139" s="15"/>
       <c r="K139" s="15"/>
       <c r="L139" s="15"/>
     </row>
     <row r="140" spans="1:12">
-      <c r="A140" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B140" s="15" t="s">
-        <v>192</v>
-      </c>
+      <c r="A140" s="15"/>
+      <c r="B140" s="12"/>
       <c r="C140" s="15"/>
       <c r="D140" s="15"/>
       <c r="E140" s="15"/>
@@ -3767,10 +3793,10 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B141" s="15" t="s">
-        <v>190</v>
+        <v>2</v>
+      </c>
+      <c r="B141" s="13" t="s">
+        <v>152</v>
       </c>
       <c r="C141" s="15"/>
       <c r="D141" s="15"/>
@@ -3785,10 +3811,10 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" s="15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B142" s="15" t="s">
-        <v>8</v>
+        <v>189</v>
       </c>
       <c r="C142" s="15"/>
       <c r="D142" s="15"/>
@@ -3803,10 +3829,10 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" s="15" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="B143" s="15" t="s">
-        <v>152</v>
+        <v>212</v>
       </c>
       <c r="C143" s="15"/>
       <c r="D143" s="15"/>
@@ -3820,11 +3846,11 @@
       <c r="L143" s="15"/>
     </row>
     <row r="144" spans="1:12">
-      <c r="A144" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B144" s="15" t="s">
-        <v>21</v>
+      <c r="A144" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="C144" s="15"/>
       <c r="D144" s="15"/>
@@ -3839,9 +3865,11 @@
     </row>
     <row r="145" spans="1:12">
       <c r="A145" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B145" s="15"/>
+        <v>7</v>
+      </c>
+      <c r="B145" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="C145" s="15"/>
       <c r="D145" s="15"/>
       <c r="E145" s="15"/>
@@ -3855,67 +3883,35 @@
     </row>
     <row r="146" spans="1:12">
       <c r="A146" s="15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B146" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C146" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D146" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="15"/>
+      <c r="F146" s="15"/>
+      <c r="G146" s="15"/>
+      <c r="H146" s="15"/>
+      <c r="I146" s="15"/>
+      <c r="J146" s="15"/>
+      <c r="K146" s="15"/>
+      <c r="L146" s="15"/>
+    </row>
+    <row r="147" spans="1:12">
+      <c r="A147" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E146" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F146" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G146" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H146" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I146" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J146" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="K146" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="L146" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="147" spans="1:12">
-      <c r="A147" s="15" t="str">
-        <f>B143</f>
-        <v>gaseous hydrogen production</v>
-      </c>
-      <c r="B147" s="16">
-        <v>1</v>
-      </c>
-      <c r="C147" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D147" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="B147" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C147" s="15"/>
+      <c r="D147" s="15"/>
       <c r="E147" s="15"/>
-      <c r="F147" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G147" s="15" t="str">
-        <f>B143</f>
-        <v>gaseous hydrogen production</v>
-      </c>
-      <c r="H147" s="15" t="s">
-        <v>143</v>
-      </c>
+      <c r="F147" s="15"/>
+      <c r="G147" s="15"/>
+      <c r="H147" s="15"/>
       <c r="I147" s="15"/>
       <c r="J147" s="15"/>
       <c r="K147" s="15"/>
@@ -3923,78 +3919,82 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="B148">
-        <f>B151</f>
-        <v>3.0000000000000001E-3</v>
-      </c>
-      <c r="C148" t="s">
-        <v>69</v>
-      </c>
-      <c r="D148" t="s">
-        <v>21</v>
-      </c>
-      <c r="F148" t="s">
-        <v>17</v>
-      </c>
-      <c r="G148" t="s">
-        <v>67</v>
-      </c>
-      <c r="H148" t="s">
-        <v>74</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B148" s="15"/>
+      <c r="C148" s="15"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="15"/>
+      <c r="F148" s="15"/>
+      <c r="G148" s="15"/>
+      <c r="H148" s="15"/>
+      <c r="I148" s="15"/>
+      <c r="J148" s="15"/>
+      <c r="K148" s="15"/>
+      <c r="L148" s="15"/>
     </row>
     <row r="149" spans="1:12">
       <c r="A149" s="15" t="s">
-        <v>210</v>
-      </c>
-      <c r="B149" s="17">
-        <v>3.4299999999999999E-9</v>
+        <v>11</v>
+      </c>
+      <c r="B149" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C149" s="15" t="s">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="D149" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E149" s="15"/>
+      <c r="E149" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F149" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G149" t="s">
-        <v>211</v>
+        <v>9</v>
+      </c>
+      <c r="G149" s="15" t="s">
+        <v>14</v>
       </c>
       <c r="H149" s="15" t="s">
-        <v>213</v>
-      </c>
-      <c r="I149" s="15"/>
-      <c r="J149" s="15"/>
-      <c r="K149" s="15"/>
-      <c r="L149" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="I149" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J149" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K149" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L149" s="15" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="150" spans="1:12">
-      <c r="A150" s="15" t="s">
-        <v>146</v>
+      <c r="A150" s="15" t="str">
+        <f>B146</f>
+        <v>gaseous hydrogen production</v>
       </c>
       <c r="B150" s="16">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="C150" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="E150" s="15"/>
       <c r="F150" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G150" s="15" t="s">
-        <v>164</v>
+        <v>16</v>
+      </c>
+      <c r="G150" s="15" t="str">
+        <f>B146</f>
+        <v>gaseous hydrogen production</v>
       </c>
       <c r="H150" s="15" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="I150" s="15"/>
       <c r="J150" s="15"/>
@@ -4003,50 +4003,50 @@
     </row>
     <row r="151" spans="1:12">
       <c r="A151" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="B151" s="16">
+        <v>66</v>
+      </c>
+      <c r="B151">
+        <f>B154</f>
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="C151" s="15"/>
-      <c r="D151" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E151" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F151" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G151" s="15"/>
-      <c r="H151" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="I151" s="15"/>
-      <c r="J151" s="15"/>
-      <c r="K151" s="15"/>
-      <c r="L151" s="15"/>
+      <c r="C151" t="s">
+        <v>69</v>
+      </c>
+      <c r="D151" t="s">
+        <v>21</v>
+      </c>
+      <c r="F151" t="s">
+        <v>17</v>
+      </c>
+      <c r="G151" t="s">
+        <v>67</v>
+      </c>
+      <c r="H151" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="152" spans="1:12">
       <c r="A152" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="B152" s="12">
-        <v>3.8000000000000002E-4</v>
-      </c>
-      <c r="C152" s="15"/>
+        <v>205</v>
+      </c>
+      <c r="B152" s="17">
+        <v>3.4299999999999999E-9</v>
+      </c>
+      <c r="C152" s="15" t="s">
+        <v>69</v>
+      </c>
       <c r="D152" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="E152" s="15" t="s">
-        <v>154</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E152" s="15"/>
       <c r="F152" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G152" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="G152" t="s">
+        <v>206</v>
+      </c>
       <c r="H152" s="15" t="s">
-        <v>153</v>
+        <v>208</v>
       </c>
       <c r="I152" s="15"/>
       <c r="J152" s="15"/>
@@ -4055,22 +4055,24 @@
     </row>
     <row r="153" spans="1:12">
       <c r="A153" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="B153" s="15">
-        <v>9.4600000000000004E-2</v>
-      </c>
-      <c r="C153" s="15"/>
+        <v>146</v>
+      </c>
+      <c r="B153" s="16">
+        <v>1.25</v>
+      </c>
+      <c r="C153" s="15" t="s">
+        <v>8</v>
+      </c>
       <c r="D153" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="E153" s="15" t="s">
-        <v>155</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="E153" s="15"/>
       <c r="F153" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="G153" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="G153" s="15" t="s">
+        <v>164</v>
+      </c>
       <c r="H153" s="15" t="s">
         <v>153</v>
       </c>
@@ -4081,17 +4083,17 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="B154" s="15">
-        <v>9.5000000000000001E-2</v>
+        <v>71</v>
+      </c>
+      <c r="B154" s="16">
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="C154" s="15"/>
       <c r="D154" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="E154" s="15" t="s">
-        <v>158</v>
+        <v>21</v>
+      </c>
+      <c r="E154" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F154" s="15" t="s">
         <v>22</v>
@@ -4106,14 +4108,26 @@
       <c r="L154" s="15"/>
     </row>
     <row r="155" spans="1:12">
-      <c r="A155" s="15"/>
-      <c r="B155" s="15"/>
+      <c r="A155" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B155" s="12">
+        <v>3.8000000000000002E-4</v>
+      </c>
       <c r="C155" s="15"/>
-      <c r="D155" s="15"/>
-      <c r="E155" s="15"/>
-      <c r="F155" s="15"/>
+      <c r="D155" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E155" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="F155" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G155" s="15"/>
-      <c r="H155" s="15"/>
+      <c r="H155" s="15" t="s">
+        <v>153</v>
+      </c>
       <c r="I155" s="15"/>
       <c r="J155" s="15"/>
       <c r="K155" s="15"/>
@@ -4121,17 +4135,25 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B156" s="13" t="s">
-        <v>167</v>
+        <v>156</v>
+      </c>
+      <c r="B156" s="15">
+        <v>9.4600000000000004E-2</v>
       </c>
       <c r="C156" s="15"/>
-      <c r="D156" s="15"/>
-      <c r="E156" s="15"/>
-      <c r="F156" s="15"/>
+      <c r="D156" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E156" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F156" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G156" s="15"/>
-      <c r="H156" s="15"/>
+      <c r="H156" s="15" t="s">
+        <v>153</v>
+      </c>
       <c r="I156" s="15"/>
       <c r="J156" s="15"/>
       <c r="K156" s="15"/>
@@ -4139,29 +4161,33 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="B157" s="15" t="s">
-        <v>174</v>
+        <v>157</v>
+      </c>
+      <c r="B157" s="15">
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="C157" s="15"/>
-      <c r="D157" s="15"/>
-      <c r="E157" s="15"/>
-      <c r="F157" s="15"/>
+      <c r="D157" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="E157" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="F157" s="15" t="s">
+        <v>22</v>
+      </c>
       <c r="G157" s="15"/>
-      <c r="H157" s="15"/>
+      <c r="H157" s="15" t="s">
+        <v>153</v>
+      </c>
       <c r="I157" s="15"/>
       <c r="J157" s="15"/>
       <c r="K157" s="15"/>
       <c r="L157" s="15"/>
     </row>
     <row r="158" spans="1:12">
-      <c r="A158" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B158" s="15" t="s">
-        <v>190</v>
-      </c>
+      <c r="A158" s="15"/>
+      <c r="B158" s="15"/>
       <c r="C158" s="15"/>
       <c r="D158" s="15"/>
       <c r="E158" s="15"/>
@@ -4175,10 +4201,10 @@
     </row>
     <row r="159" spans="1:12">
       <c r="A159" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B159" s="15" t="s">
-        <v>8</v>
+        <v>2</v>
+      </c>
+      <c r="B159" s="13" t="s">
+        <v>167</v>
       </c>
       <c r="C159" s="15"/>
       <c r="D159" s="15"/>
@@ -4193,10 +4219,10 @@
     </row>
     <row r="160" spans="1:12">
       <c r="A160" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B160" s="15" t="s">
-        <v>167</v>
+        <v>6</v>
+      </c>
+      <c r="B160" t="s">
+        <v>216</v>
       </c>
       <c r="C160" s="15"/>
       <c r="D160" s="15"/>
@@ -4211,10 +4237,10 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" s="15" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="B161" s="15" t="s">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="C161" s="15"/>
       <c r="D161" s="15"/>
@@ -4228,10 +4254,12 @@
       <c r="L161" s="15"/>
     </row>
     <row r="162" spans="1:12">
-      <c r="A162" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B162" s="15"/>
+      <c r="A162" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B162" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="C162" s="15"/>
       <c r="D162" s="15"/>
       <c r="E162" s="15"/>
@@ -4245,119 +4273,69 @@
     </row>
     <row r="163" spans="1:12">
       <c r="A163" s="15" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B163" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C163" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="D163" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E163" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F163" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G163" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C163" s="15"/>
+      <c r="D163" s="15"/>
+      <c r="E163" s="15"/>
+      <c r="F163" s="15"/>
+      <c r="G163" s="15"/>
+      <c r="H163" s="15"/>
+      <c r="I163" s="15"/>
+      <c r="J163" s="15"/>
+      <c r="K163" s="15"/>
+      <c r="L163" s="15"/>
+    </row>
+    <row r="164" spans="1:12">
+      <c r="A164" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="H163" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I163" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J163" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="K163" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="L163" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="164" spans="1:12">
-      <c r="A164" s="15" t="str">
-        <f>B160</f>
-        <v>ammonia cracking</v>
-      </c>
-      <c r="B164" s="16">
-        <v>1</v>
-      </c>
-      <c r="C164" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D164" s="15" t="s">
-        <v>21</v>
-      </c>
+      <c r="B164" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="C164" s="15"/>
+      <c r="D164" s="15"/>
       <c r="E164" s="15"/>
-      <c r="F164" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="G164" s="15" t="str">
-        <f>B160</f>
-        <v>ammonia cracking</v>
-      </c>
-      <c r="H164" s="15" t="s">
-        <v>143</v>
-      </c>
+      <c r="F164" s="15"/>
+      <c r="G164" s="15"/>
+      <c r="H164" s="15"/>
       <c r="I164" s="15"/>
       <c r="J164" s="15"/>
       <c r="K164" s="15"/>
       <c r="L164" s="15"/>
     </row>
-    <row r="165" spans="1:12" ht="15.75">
-      <c r="A165" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B165">
-        <v>0.35</v>
-      </c>
-      <c r="C165" t="s">
-        <v>69</v>
-      </c>
-      <c r="D165" t="s">
-        <v>21</v>
-      </c>
-      <c r="F165" t="s">
-        <v>17</v>
-      </c>
-      <c r="G165" t="s">
-        <v>67</v>
-      </c>
-      <c r="H165" t="s">
-        <v>201</v>
-      </c>
+    <row r="165" spans="1:12">
+      <c r="A165" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B165" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C165" s="15"/>
+      <c r="D165" s="15"/>
+      <c r="E165" s="15"/>
+      <c r="F165" s="15"/>
+      <c r="G165" s="15"/>
+      <c r="H165" s="15"/>
+      <c r="I165" s="15"/>
+      <c r="J165" s="15"/>
+      <c r="K165" s="15"/>
+      <c r="L165" s="15"/>
     </row>
     <row r="166" spans="1:12">
       <c r="A166" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="B166" s="17">
-        <f>1/(28*1000*300*50)</f>
-        <v>2.380952380952381E-9</v>
-      </c>
-      <c r="C166" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D166" s="15" t="s">
-        <v>13</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="B166" s="15"/>
+      <c r="C166" s="15"/>
+      <c r="D166" s="15"/>
       <c r="E166" s="15"/>
-      <c r="F166" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G166" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="H166" s="15" t="s">
-        <v>173</v>
-      </c>
+      <c r="F166" s="15"/>
+      <c r="G166" s="15"/>
+      <c r="H166" s="15"/>
       <c r="I166" s="15"/>
       <c r="J166" s="15"/>
       <c r="K166" s="15"/>
@@ -4365,747 +4343,887 @@
     </row>
     <row r="167" spans="1:12">
       <c r="A167" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="B167" s="17">
-        <f>1/(28*1000*300*50)</f>
-        <v>2.380952380952381E-9</v>
+        <v>11</v>
+      </c>
+      <c r="B167" s="15" t="s">
+        <v>12</v>
       </c>
       <c r="C167" s="15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D167" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E167" s="15"/>
+      <c r="E167" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="F167" s="15" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G167" s="15" t="s">
-        <v>171</v>
+        <v>14</v>
       </c>
       <c r="H167" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="I167" s="15"/>
-      <c r="J167" s="15"/>
-      <c r="K167" s="15"/>
-      <c r="L167" s="15"/>
+        <v>6</v>
+      </c>
+      <c r="I167" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J167" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K167" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L167" s="15" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="168" spans="1:12">
-      <c r="A168" s="15" t="s">
-        <v>146</v>
+      <c r="A168" s="15" t="str">
+        <f>B164</f>
+        <v>ammonia cracking</v>
       </c>
       <c r="B168" s="16">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="C168" s="15" t="s">
         <v>8</v>
       </c>
       <c r="D168" s="15" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="E168" s="15"/>
       <c r="F168" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G168" s="15" t="s">
-        <v>164</v>
+        <v>16</v>
+      </c>
+      <c r="G168" s="15" t="str">
+        <f>B164</f>
+        <v>ammonia cracking</v>
       </c>
       <c r="H168" s="15" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="I168" s="15"/>
       <c r="J168" s="15"/>
       <c r="K168" s="15"/>
       <c r="L168" s="15"/>
     </row>
+    <row r="169" spans="1:12" ht="15.6">
+      <c r="A169" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B169">
+        <v>0.35</v>
+      </c>
+      <c r="C169" t="s">
+        <v>69</v>
+      </c>
+      <c r="D169" t="s">
+        <v>21</v>
+      </c>
+      <c r="F169" t="s">
+        <v>17</v>
+      </c>
+      <c r="G169" t="s">
+        <v>67</v>
+      </c>
+      <c r="H169" t="s">
+        <v>196</v>
+      </c>
+    </row>
     <row r="170" spans="1:12">
-      <c r="A170" t="s">
-        <v>2</v>
-      </c>
-      <c r="B170" s="13" t="s">
-        <v>175</v>
-      </c>
+      <c r="A170" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B170" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C170" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D170" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E170" s="15"/>
+      <c r="F170" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G170" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="H170" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="I170" s="15"/>
+      <c r="J170" s="15"/>
+      <c r="K170" s="15"/>
+      <c r="L170" s="15"/>
     </row>
     <row r="171" spans="1:12">
-      <c r="A171" t="s">
-        <v>6</v>
-      </c>
-      <c r="B171" t="s">
-        <v>188</v>
-      </c>
+      <c r="A171" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B171" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C171" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D171" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E171" s="15"/>
+      <c r="F171" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G171" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="H171" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="I171" s="15"/>
+      <c r="J171" s="15"/>
+      <c r="K171" s="15"/>
+      <c r="L171" s="15"/>
     </row>
     <row r="172" spans="1:12">
       <c r="A172" t="s">
-        <v>53</v>
-      </c>
-      <c r="B172" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="173" spans="1:12">
-      <c r="A173" t="s">
-        <v>7</v>
-      </c>
-      <c r="B173" t="s">
-        <v>8</v>
+        <v>78</v>
+      </c>
+      <c r="B172" s="18">
+        <f>3.086+0.6</f>
+        <v>3.6859999999999999</v>
+      </c>
+      <c r="C172" t="s">
+        <v>69</v>
+      </c>
+      <c r="D172" t="s">
+        <v>68</v>
+      </c>
+      <c r="F172" t="s">
+        <v>17</v>
+      </c>
+      <c r="G172" t="s">
+        <v>64</v>
+      </c>
+      <c r="H172" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>14</v>
-      </c>
-      <c r="B174" t="str">
-        <f>B170</f>
-        <v>liquid ammonia production</v>
+        <v>2</v>
+      </c>
+      <c r="B174" s="13" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B175" t="s">
-        <v>21</v>
+        <v>188</v>
       </c>
     </row>
     <row r="176" spans="1:12">
       <c r="A176" t="s">
-        <v>10</v>
+        <v>53</v>
+      </c>
+      <c r="B176" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="177" spans="1:12">
-      <c r="A177" t="s">
-        <v>11</v>
-      </c>
-      <c r="B177" t="s">
-        <v>12</v>
-      </c>
-      <c r="C177" t="s">
+      <c r="A177" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12">
+      <c r="A178" t="s">
         <v>7</v>
       </c>
-      <c r="D177" t="s">
-        <v>13</v>
-      </c>
-      <c r="E177" t="s">
-        <v>19</v>
-      </c>
-      <c r="F177" t="s">
-        <v>9</v>
-      </c>
-      <c r="G177" t="s">
+      <c r="B178" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12">
+      <c r="A179" t="s">
         <v>14</v>
       </c>
-      <c r="H177" t="s">
-        <v>6</v>
-      </c>
-      <c r="I177" t="s">
-        <v>18</v>
-      </c>
-      <c r="J177" t="s">
-        <v>140</v>
-      </c>
-      <c r="K177" t="s">
-        <v>141</v>
-      </c>
-      <c r="L177" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="178" spans="1:12">
-      <c r="A178" t="str">
+      <c r="B179" t="str">
         <f>B174</f>
         <v>liquid ammonia production</v>
       </c>
-      <c r="B178" s="18">
-        <v>1</v>
-      </c>
-      <c r="C178" t="s">
-        <v>8</v>
-      </c>
-      <c r="D178" t="s">
-        <v>21</v>
-      </c>
-      <c r="F178" t="s">
-        <v>16</v>
-      </c>
-      <c r="G178" t="s">
-        <v>176</v>
-      </c>
-      <c r="H178" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="179" spans="1:12">
-      <c r="A179" t="s">
-        <v>179</v>
-      </c>
-      <c r="B179" s="18">
-        <v>0.81499999999999995</v>
-      </c>
-      <c r="C179" t="s">
-        <v>8</v>
-      </c>
-      <c r="D179" t="s">
-        <v>21</v>
-      </c>
-      <c r="F179" t="s">
-        <v>17</v>
-      </c>
-      <c r="G179" t="s">
-        <v>179</v>
-      </c>
-      <c r="H179" t="s">
-        <v>145</v>
-      </c>
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
-        <v>180</v>
-      </c>
-      <c r="B180" s="18">
-        <v>5.1499999999999998E-5</v>
-      </c>
-      <c r="C180" t="s">
-        <v>8</v>
-      </c>
-      <c r="D180" t="s">
-        <v>21</v>
-      </c>
-      <c r="F180" t="s">
-        <v>17</v>
-      </c>
-      <c r="G180" t="s">
-        <v>180</v>
-      </c>
-      <c r="H180" t="s">
-        <v>145</v>
+        <v>13</v>
+      </c>
+      <c r="B180" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>170</v>
-      </c>
-      <c r="B181" s="18">
-        <v>3.29E-10</v>
-      </c>
-      <c r="C181" t="s">
-        <v>8</v>
-      </c>
-      <c r="D181" t="s">
-        <v>13</v>
-      </c>
-      <c r="F181" t="s">
-        <v>17</v>
-      </c>
-      <c r="G181" t="s">
-        <v>171</v>
+        <v>10</v>
       </c>
     </row>
     <row r="182" spans="1:12">
       <c r="A182" t="s">
-        <v>146</v>
-      </c>
-      <c r="B182" s="18">
-        <v>1.44</v>
+        <v>11</v>
+      </c>
+      <c r="B182" t="s">
+        <v>12</v>
       </c>
       <c r="C182" t="s">
+        <v>7</v>
+      </c>
+      <c r="D182" t="s">
+        <v>13</v>
+      </c>
+      <c r="E182" t="s">
+        <v>19</v>
+      </c>
+      <c r="F182" t="s">
+        <v>9</v>
+      </c>
+      <c r="G182" t="s">
+        <v>14</v>
+      </c>
+      <c r="H182" t="s">
+        <v>6</v>
+      </c>
+      <c r="I182" t="s">
+        <v>18</v>
+      </c>
+      <c r="J182" t="s">
+        <v>140</v>
+      </c>
+      <c r="K182" t="s">
+        <v>141</v>
+      </c>
+      <c r="L182" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12">
+      <c r="A183" t="str">
+        <f>B179</f>
+        <v>liquid ammonia production</v>
+      </c>
+      <c r="B183" s="18">
+        <v>1</v>
+      </c>
+      <c r="C183" t="s">
         <v>8</v>
       </c>
-      <c r="D182" t="s">
-        <v>68</v>
-      </c>
-      <c r="F182" t="s">
-        <v>17</v>
-      </c>
-      <c r="G182" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="183" spans="1:12">
-      <c r="A183" t="s">
-        <v>181</v>
-      </c>
-      <c r="B183" s="18">
-        <v>5.1499999999999998E-5</v>
-      </c>
-      <c r="C183" t="s">
-        <v>138</v>
-      </c>
       <c r="D183" t="s">
         <v>21</v>
       </c>
       <c r="F183" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G183" t="s">
-        <v>202</v>
+        <v>176</v>
+      </c>
+      <c r="H183" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="B184" s="18">
-        <v>0.14899999999999999</v>
+        <v>0.81499999999999995</v>
+      </c>
+      <c r="C184" t="s">
+        <v>8</v>
       </c>
       <c r="D184" t="s">
-        <v>149</v>
-      </c>
-      <c r="E184" s="15" t="s">
-        <v>158</v>
+        <v>21</v>
       </c>
       <c r="F184" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G184" t="s">
+        <v>179</v>
+      </c>
+      <c r="H184" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>71</v>
+        <v>180</v>
       </c>
       <c r="B185" s="18">
-        <v>7.67E-4</v>
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C185" t="s">
+        <v>8</v>
       </c>
       <c r="D185" t="s">
         <v>21</v>
       </c>
-      <c r="E185" s="12" t="s">
-        <v>30</v>
-      </c>
       <c r="F185" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G185" t="s">
+        <v>180</v>
+      </c>
+      <c r="H185" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>20</v>
+        <v>170</v>
       </c>
       <c r="B186" s="18">
-        <v>1.6299999999999999E-3</v>
+        <v>3.29E-10</v>
+      </c>
+      <c r="C186" t="s">
+        <v>8</v>
       </c>
       <c r="D186" t="s">
-        <v>21</v>
-      </c>
-      <c r="E186" s="12" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F186" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G186" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="187" spans="1:12">
       <c r="A187" t="s">
-        <v>25</v>
+        <v>146</v>
       </c>
       <c r="B187" s="18">
-        <v>1E-3</v>
+        <v>1.44</v>
+      </c>
+      <c r="C187" t="s">
+        <v>8</v>
       </c>
       <c r="D187" t="s">
-        <v>21</v>
-      </c>
-      <c r="E187" s="12" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="F187" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G187" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="188" spans="1:12">
       <c r="A188" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="B188" s="18">
-        <v>4.7600000000000003E-2</v>
+        <v>5.1499999999999998E-5</v>
+      </c>
+      <c r="C188" t="s">
+        <v>138</v>
       </c>
       <c r="D188" t="s">
-        <v>149</v>
-      </c>
-      <c r="E188" s="12" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F188" t="s">
-        <v>22</v>
+        <v>17</v>
+      </c>
+      <c r="G188" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="189" spans="1:12">
       <c r="A189" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B189" s="18">
-        <v>0.10100000000000001</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="D189" t="s">
         <v>149</v>
       </c>
       <c r="E189" s="15" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F189" t="s">
         <v>22</v>
       </c>
     </row>
+    <row r="190" spans="1:12">
+      <c r="A190" t="s">
+        <v>71</v>
+      </c>
+      <c r="B190" s="18">
+        <v>7.67E-4</v>
+      </c>
+      <c r="D190" t="s">
+        <v>21</v>
+      </c>
+      <c r="E190" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F190" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="191" spans="1:12">
       <c r="A191" t="s">
-        <v>2</v>
-      </c>
-      <c r="B191" s="13" t="s">
-        <v>179</v>
+        <v>20</v>
+      </c>
+      <c r="B191" s="18">
+        <v>1.6299999999999999E-3</v>
+      </c>
+      <c r="D191" t="s">
+        <v>21</v>
+      </c>
+      <c r="E191" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F191" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="192" spans="1:12">
       <c r="A192" t="s">
-        <v>6</v>
-      </c>
-      <c r="B192" t="s">
-        <v>195</v>
+        <v>25</v>
+      </c>
+      <c r="B192" s="18">
+        <v>1E-3</v>
+      </c>
+      <c r="D192" t="s">
+        <v>21</v>
+      </c>
+      <c r="E192" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F192" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="193" spans="1:12">
       <c r="A193" t="s">
-        <v>53</v>
-      </c>
-      <c r="B193" t="s">
-        <v>199</v>
+        <v>156</v>
+      </c>
+      <c r="B193" s="18">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="D193" t="s">
+        <v>149</v>
+      </c>
+      <c r="E193" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F193" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="194" spans="1:12">
       <c r="A194" t="s">
-        <v>7</v>
-      </c>
-      <c r="B194" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="195" spans="1:12">
-      <c r="A195" t="s">
-        <v>14</v>
-      </c>
-      <c r="B195" t="s">
-        <v>179</v>
+        <v>156</v>
+      </c>
+      <c r="B194" s="18">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="D194" t="s">
+        <v>149</v>
+      </c>
+      <c r="E194" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F194" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="196" spans="1:12">
       <c r="A196" t="s">
-        <v>13</v>
-      </c>
-      <c r="B196" t="s">
-        <v>21</v>
+        <v>2</v>
+      </c>
+      <c r="B196" s="13" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="197" spans="1:12">
       <c r="A197" t="s">
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="B197" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="198" spans="1:12">
       <c r="A198" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="B198" t="s">
-        <v>12</v>
-      </c>
-      <c r="C198" t="s">
-        <v>7</v>
-      </c>
-      <c r="D198" t="s">
-        <v>13</v>
-      </c>
-      <c r="E198" t="s">
-        <v>19</v>
-      </c>
-      <c r="F198" t="s">
-        <v>9</v>
-      </c>
-      <c r="G198" t="s">
-        <v>14</v>
-      </c>
-      <c r="H198" t="s">
-        <v>6</v>
-      </c>
-      <c r="I198" t="s">
-        <v>18</v>
-      </c>
-      <c r="J198" t="s">
-        <v>140</v>
-      </c>
-      <c r="K198" t="s">
-        <v>141</v>
-      </c>
-      <c r="L198" t="s">
-        <v>142</v>
+        <v>210</v>
       </c>
     </row>
     <row r="199" spans="1:12">
-      <c r="A199" t="s">
-        <v>179</v>
-      </c>
-      <c r="B199" s="18">
-        <v>1</v>
-      </c>
-      <c r="C199" t="s">
-        <v>8</v>
-      </c>
-      <c r="D199" t="s">
-        <v>21</v>
-      </c>
-      <c r="F199" t="s">
-        <v>16</v>
-      </c>
-      <c r="G199" t="s">
-        <v>179</v>
-      </c>
-      <c r="H199" t="s">
-        <v>182</v>
+      <c r="A199" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B199" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>183</v>
-      </c>
-      <c r="B200" s="18">
-        <v>4.4300000000000002E-10</v>
-      </c>
-      <c r="C200" t="s">
+        <v>7</v>
+      </c>
+      <c r="B200" t="s">
         <v>8</v>
-      </c>
-      <c r="D200" t="s">
-        <v>13</v>
-      </c>
-      <c r="F200" t="s">
-        <v>17</v>
-      </c>
-      <c r="G200" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>157</v>
-      </c>
-      <c r="B201" s="18">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="D201" t="s">
-        <v>149</v>
-      </c>
-      <c r="E201" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="F201" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="B201" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>156</v>
-      </c>
-      <c r="B202" s="18">
-        <v>2.4499999999999999E-3</v>
-      </c>
-      <c r="D202" t="s">
-        <v>149</v>
-      </c>
-      <c r="E202" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="F202" t="s">
-        <v>22</v>
+        <v>13</v>
+      </c>
+      <c r="B202" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12">
+      <c r="A203" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="204" spans="1:12">
       <c r="A204" t="s">
-        <v>2</v>
-      </c>
-      <c r="B204" s="13" t="s">
-        <v>180</v>
+        <v>11</v>
+      </c>
+      <c r="B204" t="s">
+        <v>12</v>
+      </c>
+      <c r="C204" t="s">
+        <v>7</v>
+      </c>
+      <c r="D204" t="s">
+        <v>13</v>
+      </c>
+      <c r="E204" t="s">
+        <v>19</v>
+      </c>
+      <c r="F204" t="s">
+        <v>9</v>
+      </c>
+      <c r="G204" t="s">
+        <v>14</v>
+      </c>
+      <c r="H204" t="s">
+        <v>6</v>
+      </c>
+      <c r="I204" t="s">
+        <v>18</v>
+      </c>
+      <c r="J204" t="s">
+        <v>140</v>
+      </c>
+      <c r="K204" t="s">
+        <v>141</v>
+      </c>
+      <c r="L204" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>6</v>
-      </c>
-      <c r="B205" t="s">
-        <v>184</v>
+        <v>179</v>
+      </c>
+      <c r="B205" s="18">
+        <v>1</v>
+      </c>
+      <c r="C205" t="s">
+        <v>8</v>
+      </c>
+      <c r="D205" t="s">
+        <v>21</v>
+      </c>
+      <c r="F205" t="s">
+        <v>16</v>
+      </c>
+      <c r="G205" t="s">
+        <v>179</v>
+      </c>
+      <c r="H205" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="206" spans="1:12">
       <c r="A206" t="s">
-        <v>53</v>
-      </c>
-      <c r="B206" t="s">
-        <v>200</v>
+        <v>183</v>
+      </c>
+      <c r="B206" s="18">
+        <v>4.4300000000000002E-10</v>
+      </c>
+      <c r="C206" t="s">
+        <v>8</v>
+      </c>
+      <c r="D206" t="s">
+        <v>13</v>
+      </c>
+      <c r="F206" t="s">
+        <v>17</v>
+      </c>
+      <c r="G206" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>7</v>
-      </c>
-      <c r="B207" t="s">
-        <v>8</v>
+        <v>157</v>
+      </c>
+      <c r="B207" s="18">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="D207" t="s">
+        <v>149</v>
+      </c>
+      <c r="E207" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="F207" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>14</v>
-      </c>
-      <c r="B208" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="209" spans="1:12">
-      <c r="A209" t="s">
-        <v>13</v>
-      </c>
-      <c r="B209" t="s">
-        <v>21</v>
+        <v>156</v>
+      </c>
+      <c r="B208" s="18">
+        <v>2.4499999999999999E-3</v>
+      </c>
+      <c r="D208" t="s">
+        <v>149</v>
+      </c>
+      <c r="E208" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="F208" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>10</v>
+        <v>2</v>
+      </c>
+      <c r="B210" s="13" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="211" spans="1:12">
       <c r="A211" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B211" t="s">
-        <v>12</v>
-      </c>
-      <c r="C211" t="s">
-        <v>7</v>
-      </c>
-      <c r="D211" t="s">
-        <v>13</v>
-      </c>
-      <c r="E211" t="s">
-        <v>19</v>
-      </c>
-      <c r="F211" t="s">
-        <v>9</v>
-      </c>
-      <c r="G211" t="s">
-        <v>14</v>
-      </c>
-      <c r="H211" t="s">
-        <v>6</v>
-      </c>
-      <c r="I211" t="s">
-        <v>18</v>
-      </c>
-      <c r="J211" t="s">
-        <v>140</v>
-      </c>
-      <c r="K211" t="s">
-        <v>141</v>
-      </c>
-      <c r="L211" t="s">
-        <v>142</v>
+        <v>184</v>
       </c>
     </row>
     <row r="212" spans="1:12">
       <c r="A212" t="s">
-        <v>180</v>
-      </c>
-      <c r="B212" s="18">
-        <v>1</v>
-      </c>
-      <c r="C212" t="s">
-        <v>8</v>
-      </c>
-      <c r="D212" t="s">
-        <v>21</v>
-      </c>
-      <c r="F212" t="s">
-        <v>16</v>
-      </c>
-      <c r="G212" t="s">
-        <v>180</v>
-      </c>
-      <c r="H212" t="s">
-        <v>185</v>
+        <v>53</v>
+      </c>
+      <c r="B212" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="213" spans="1:12">
-      <c r="A213" t="s">
-        <v>186</v>
-      </c>
-      <c r="B213" s="18">
-        <v>0.91700000000000004</v>
-      </c>
-      <c r="C213" t="s">
-        <v>8</v>
-      </c>
-      <c r="D213" t="s">
-        <v>21</v>
-      </c>
-      <c r="F213" t="s">
-        <v>17</v>
-      </c>
-      <c r="G213" t="s">
-        <v>196</v>
+      <c r="A213" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B213" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>205</v>
-      </c>
-      <c r="B214" s="18">
-        <v>0.03</v>
-      </c>
-      <c r="C214" t="s">
-        <v>69</v>
-      </c>
-      <c r="D214" t="s">
-        <v>21</v>
-      </c>
-      <c r="F214" t="s">
-        <v>17</v>
-      </c>
-      <c r="G214" t="s">
-        <v>203</v>
-      </c>
-      <c r="H214" t="s">
-        <v>204</v>
+        <v>7</v>
+      </c>
+      <c r="B214" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>187</v>
-      </c>
-      <c r="B215" s="18">
-        <v>5.2499999999999998E-2</v>
-      </c>
-      <c r="C215" t="s">
-        <v>8</v>
-      </c>
-      <c r="D215" t="s">
-        <v>21</v>
-      </c>
-      <c r="F215" t="s">
-        <v>17</v>
-      </c>
-      <c r="G215" t="s">
-        <v>197</v>
+        <v>14</v>
+      </c>
+      <c r="B215" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
+        <v>13</v>
+      </c>
+      <c r="B216" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="217" spans="1:12">
+      <c r="A217" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12">
+      <c r="A218" t="s">
+        <v>11</v>
+      </c>
+      <c r="B218" t="s">
+        <v>12</v>
+      </c>
+      <c r="C218" t="s">
+        <v>7</v>
+      </c>
+      <c r="D218" t="s">
+        <v>13</v>
+      </c>
+      <c r="E218" t="s">
+        <v>19</v>
+      </c>
+      <c r="F218" t="s">
+        <v>9</v>
+      </c>
+      <c r="G218" t="s">
+        <v>14</v>
+      </c>
+      <c r="H218" t="s">
+        <v>6</v>
+      </c>
+      <c r="I218" t="s">
+        <v>18</v>
+      </c>
+      <c r="J218" t="s">
+        <v>140</v>
+      </c>
+      <c r="K218" t="s">
+        <v>141</v>
+      </c>
+      <c r="L218" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="219" spans="1:12">
+      <c r="A219" t="s">
+        <v>180</v>
+      </c>
+      <c r="B219" s="18">
+        <v>1</v>
+      </c>
+      <c r="C219" t="s">
+        <v>8</v>
+      </c>
+      <c r="D219" t="s">
+        <v>21</v>
+      </c>
+      <c r="F219" t="s">
+        <v>16</v>
+      </c>
+      <c r="G219" t="s">
+        <v>180</v>
+      </c>
+      <c r="H219" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12">
+      <c r="A220" t="s">
+        <v>186</v>
+      </c>
+      <c r="B220" s="18">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="C220" t="s">
+        <v>8</v>
+      </c>
+      <c r="D220" t="s">
+        <v>21</v>
+      </c>
+      <c r="F220" t="s">
+        <v>17</v>
+      </c>
+      <c r="G220" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="221" spans="1:12">
+      <c r="A221" t="s">
+        <v>200</v>
+      </c>
+      <c r="B221" s="18">
+        <v>0.03</v>
+      </c>
+      <c r="C221" t="s">
+        <v>69</v>
+      </c>
+      <c r="D221" t="s">
+        <v>21</v>
+      </c>
+      <c r="F221" t="s">
+        <v>17</v>
+      </c>
+      <c r="G221" t="s">
+        <v>198</v>
+      </c>
+      <c r="H221" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="222" spans="1:12">
+      <c r="A222" t="s">
+        <v>187</v>
+      </c>
+      <c r="B222" s="18">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="C222" t="s">
+        <v>8</v>
+      </c>
+      <c r="D222" t="s">
+        <v>21</v>
+      </c>
+      <c r="F222" t="s">
+        <v>17</v>
+      </c>
+      <c r="G222" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12">
+      <c r="A223" t="s">
         <v>146</v>
       </c>
-      <c r="B216" s="18">
+      <c r="B223" s="18">
         <v>1.78</v>
       </c>
-      <c r="C216" t="s">
+      <c r="C223" t="s">
         <v>8</v>
       </c>
-      <c r="D216" t="s">
+      <c r="D223" t="s">
         <v>68</v>
       </c>
-      <c r="F216" t="s">
+      <c r="F223" t="s">
         <v>17</v>
       </c>
-      <c r="G216" t="s">
+      <c r="G223" t="s">
         <v>164</v>
       </c>
     </row>
@@ -5117,15 +5235,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
-  <dimension ref="A1:L6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75">
+    <row r="3" spans="1:12" ht="15.6">
       <c r="A3" s="3" t="s">
         <v>66</v>
       </c>
@@ -5145,7 +5263,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75">
+    <row r="4" spans="1:12" ht="15.6">
       <c r="A4" s="3" t="s">
         <v>66</v>
       </c>
@@ -5170,7 +5288,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.75">
+    <row r="5" spans="1:12" ht="15.6">
       <c r="A5" s="3" t="s">
         <v>66</v>
       </c>
@@ -5214,6 +5332,34 @@
       <c r="G6" t="s">
         <v>178</v>
       </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" s="16">
+        <v>0.6</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -5223,16 +5369,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="7"/>
-    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5703125" style="7"/>
+    <col min="1" max="1" width="11.5546875" style="7"/>
+    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5546875" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5362,7 +5508,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15">
+    <row r="9" spans="1:7" ht="14.4">
       <c r="B9" s="7" t="s">
         <v>99</v>
       </c>

</xml_diff>

<commit_message>
change units of transport services to -unit-
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624E6893-72B9-4D74-9A0E-4F056784215D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B907B229-9E3C-45C0-8AFA-2B7C3D702C51}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2926,7 +2926,7 @@
         <v>13</v>
       </c>
       <c r="B102" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C102" s="15"/>
       <c r="D102" s="15"/>
@@ -3004,7 +3004,7 @@
         <v>8</v>
       </c>
       <c r="D105" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E105" s="15"/>
       <c r="F105" s="15" t="s">
@@ -3601,7 +3601,7 @@
         <v>13</v>
       </c>
       <c r="B133" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C133" s="15"/>
       <c r="D133" s="15"/>
@@ -3680,7 +3680,7 @@
         <v>8</v>
       </c>
       <c r="D136" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E136" s="15"/>
       <c r="F136" s="15" t="s">
@@ -3904,7 +3904,7 @@
         <v>13</v>
       </c>
       <c r="B147" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C147" s="15"/>
       <c r="D147" s="15"/>
@@ -3983,7 +3983,7 @@
         <v>8</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E150" s="15"/>
       <c r="F150" s="15" t="s">
@@ -4312,7 +4312,7 @@
         <v>13</v>
       </c>
       <c r="B165" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C165" s="15"/>
       <c r="D165" s="15"/>
@@ -4391,7 +4391,7 @@
         <v>8</v>
       </c>
       <c r="D168" s="15" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E168" s="15"/>
       <c r="F168" s="15" t="s">
@@ -4568,7 +4568,7 @@
         <v>13</v>
       </c>
       <c r="B180" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="181" spans="1:12">
@@ -4626,7 +4626,7 @@
         <v>8</v>
       </c>
       <c r="D183" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F183" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
took out hydrogen exchange from NH3 cracking - avoiding double counting losses
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
+++ b/premise/data/additional_inventories/lci-hydrogen-transport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac145674\coding_projects\premise_h2-distribution\premise\data\additional_inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B907B229-9E3C-45C0-8AFA-2B7C3D702C51}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D88F829-590D-49A3-8E89-27E5FAEABD66}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="hydrogen-transport" sheetId="1" r:id="rId1"/>
@@ -1124,24 +1124,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L223"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <dimension ref="A1:L222"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="82.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="82.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.109375" customWidth="1"/>
-    <col min="7" max="7" width="85.44140625" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" customWidth="1"/>
-    <col min="11" max="11" width="13.33203125" customWidth="1"/>
-    <col min="12" max="12" width="43.88671875" customWidth="1"/>
-    <col min="13" max="13" width="13.33203125" customWidth="1"/>
-    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="85.42578125" customWidth="1"/>
+    <col min="8" max="8" width="25.42578125" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="12" max="12" width="43.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6">
+    <row r="1" spans="1:9" ht="15.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1149,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6">
+    <row r="3" spans="1:9" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6">
+    <row r="10" spans="1:9" ht="15.75">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="15.6">
+    <row r="13" spans="1:9" ht="15.75">
       <c r="A13" s="3" t="s">
         <v>76</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15.6">
+    <row r="15" spans="1:9" ht="15.75">
       <c r="A15" s="3" t="s">
         <v>66</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.6">
+    <row r="18" spans="1:9" ht="15.75">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.6">
+    <row r="25" spans="1:9" ht="15.75">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6">
+    <row r="28" spans="1:9" ht="15.75">
       <c r="A28" s="3" t="s">
         <v>76</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.6">
+    <row r="30" spans="1:9" ht="15.75">
       <c r="A30" s="3" t="s">
         <v>66</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6">
+    <row r="33" spans="1:8" ht="15.75">
       <c r="A33" s="4" t="s">
         <v>2</v>
       </c>
@@ -1695,7 +1695,7 @@
       <c r="G41" s="5"/>
       <c r="H41" s="5"/>
     </row>
-    <row r="42" spans="1:8" ht="15.6">
+    <row r="42" spans="1:8" ht="15.75">
       <c r="A42" s="4" t="s">
         <v>10</v>
       </c>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="H63" s="5"/>
     </row>
-    <row r="65" spans="1:8" ht="15.6">
+    <row r="65" spans="1:8" ht="15.75">
       <c r="A65" s="4" t="s">
         <v>2</v>
       </c>
@@ -2329,7 +2329,7 @@
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
     </row>
-    <row r="74" spans="1:8" ht="15.6">
+    <row r="74" spans="1:8" ht="15.75">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -3021,7 +3021,7 @@
       <c r="K105" s="15"/>
       <c r="L105" s="15"/>
     </row>
-    <row r="106" spans="1:12" ht="15.6">
+    <row r="106" spans="1:12" ht="15.75">
       <c r="A106" s="3" t="s">
         <v>66</v>
       </c>
@@ -4409,32 +4409,38 @@
       <c r="K168" s="15"/>
       <c r="L168" s="15"/>
     </row>
-    <row r="169" spans="1:12" ht="15.6">
-      <c r="A169" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B169">
-        <v>0.35</v>
-      </c>
-      <c r="C169" t="s">
-        <v>69</v>
-      </c>
-      <c r="D169" t="s">
-        <v>21</v>
-      </c>
-      <c r="F169" t="s">
+    <row r="169" spans="1:12">
+      <c r="A169" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B169" s="17">
+        <f>1/(28*1000*300*50)</f>
+        <v>2.380952380952381E-9</v>
+      </c>
+      <c r="C169" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D169" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E169" s="15"/>
+      <c r="F169" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="G169" t="s">
-        <v>67</v>
-      </c>
-      <c r="H169" t="s">
-        <v>196</v>
-      </c>
+      <c r="G169" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="H169" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="I169" s="15"/>
+      <c r="J169" s="15"/>
+      <c r="K169" s="15"/>
+      <c r="L169" s="15"/>
     </row>
     <row r="170" spans="1:12">
       <c r="A170" s="15" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B170" s="17">
         <f>1/(28*1000*300*50)</f>
@@ -4451,10 +4457,10 @@
         <v>17</v>
       </c>
       <c r="G170" s="15" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H170" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I170" s="15"/>
       <c r="J170" s="15"/>
@@ -4462,188 +4468,182 @@
       <c r="L170" s="15"/>
     </row>
     <row r="171" spans="1:12">
-      <c r="A171" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="B171" s="17">
-        <f>1/(28*1000*300*50)</f>
-        <v>2.380952380952381E-9</v>
-      </c>
-      <c r="C171" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D171" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E171" s="15"/>
-      <c r="F171" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G171" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="H171" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="I171" s="15"/>
-      <c r="J171" s="15"/>
-      <c r="K171" s="15"/>
-      <c r="L171" s="15"/>
-    </row>
-    <row r="172" spans="1:12">
-      <c r="A172" t="s">
+      <c r="A171" t="s">
         <v>78</v>
       </c>
-      <c r="B172" s="18">
+      <c r="B171" s="18">
         <f>3.086+0.6</f>
         <v>3.6859999999999999</v>
       </c>
-      <c r="C172" t="s">
+      <c r="C171" t="s">
         <v>69</v>
       </c>
-      <c r="D172" t="s">
+      <c r="D171" t="s">
         <v>68</v>
       </c>
-      <c r="F172" t="s">
+      <c r="F171" t="s">
         <v>17</v>
       </c>
-      <c r="G172" t="s">
+      <c r="G171" t="s">
         <v>64</v>
       </c>
-      <c r="H172" t="s">
+      <c r="H171" t="s">
         <v>217</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12">
+      <c r="A173" t="s">
+        <v>2</v>
+      </c>
+      <c r="B173" s="13" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>2</v>
-      </c>
-      <c r="B174" s="13" t="s">
-        <v>175</v>
+        <v>6</v>
+      </c>
+      <c r="B174" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B175" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
     </row>
     <row r="176" spans="1:12">
-      <c r="A176" t="s">
-        <v>53</v>
-      </c>
-      <c r="B176" t="s">
-        <v>209</v>
+      <c r="A176" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B176" s="12" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="177" spans="1:12">
-      <c r="A177" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B177" s="12" t="s">
-        <v>215</v>
+      <c r="A177" t="s">
+        <v>7</v>
+      </c>
+      <c r="B177" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>7</v>
-      </c>
-      <c r="B178" t="s">
-        <v>8</v>
+        <v>14</v>
+      </c>
+      <c r="B178" t="str">
+        <f>B173</f>
+        <v>liquid ammonia production</v>
       </c>
     </row>
     <row r="179" spans="1:12">
       <c r="A179" t="s">
-        <v>14</v>
-      </c>
-      <c r="B179" t="str">
-        <f>B174</f>
-        <v>liquid ammonia production</v>
+        <v>13</v>
+      </c>
+      <c r="B179" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
-        <v>13</v>
-      </c>
-      <c r="B180" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B181" t="s">
+        <v>12</v>
+      </c>
+      <c r="C181" t="s">
+        <v>7</v>
+      </c>
+      <c r="D181" t="s">
+        <v>13</v>
+      </c>
+      <c r="E181" t="s">
+        <v>19</v>
+      </c>
+      <c r="F181" t="s">
+        <v>9</v>
+      </c>
+      <c r="G181" t="s">
+        <v>14</v>
+      </c>
+      <c r="H181" t="s">
+        <v>6</v>
+      </c>
+      <c r="I181" t="s">
+        <v>18</v>
+      </c>
+      <c r="J181" t="s">
+        <v>140</v>
+      </c>
+      <c r="K181" t="s">
+        <v>141</v>
+      </c>
+      <c r="L181" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="182" spans="1:12">
-      <c r="A182" t="s">
-        <v>11</v>
-      </c>
-      <c r="B182" t="s">
-        <v>12</v>
+      <c r="A182" t="str">
+        <f>B178</f>
+        <v>liquid ammonia production</v>
+      </c>
+      <c r="B182" s="18">
+        <v>1</v>
       </c>
       <c r="C182" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D182" t="s">
         <v>13</v>
       </c>
-      <c r="E182" t="s">
-        <v>19</v>
-      </c>
       <c r="F182" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G182" t="s">
-        <v>14</v>
+        <v>176</v>
       </c>
       <c r="H182" t="s">
-        <v>6</v>
-      </c>
-      <c r="I182" t="s">
-        <v>18</v>
-      </c>
-      <c r="J182" t="s">
-        <v>140</v>
-      </c>
-      <c r="K182" t="s">
-        <v>141</v>
-      </c>
-      <c r="L182" t="s">
-        <v>142</v>
+        <v>177</v>
       </c>
     </row>
     <row r="183" spans="1:12">
-      <c r="A183" t="str">
-        <f>B179</f>
-        <v>liquid ammonia production</v>
+      <c r="A183" t="s">
+        <v>179</v>
       </c>
       <c r="B183" s="18">
-        <v>1</v>
+        <v>0.81499999999999995</v>
       </c>
       <c r="C183" t="s">
         <v>8</v>
       </c>
       <c r="D183" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F183" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G183" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H183" t="s">
-        <v>177</v>
+        <v>145</v>
       </c>
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B184" s="18">
-        <v>0.81499999999999995</v>
+        <v>5.1499999999999998E-5</v>
       </c>
       <c r="C184" t="s">
         <v>8</v>
@@ -4655,7 +4655,7 @@
         <v>17</v>
       </c>
       <c r="G184" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H184" t="s">
         <v>145</v>
@@ -4663,99 +4663,93 @@
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B185" s="18">
-        <v>5.1499999999999998E-5</v>
+        <v>3.29E-10</v>
       </c>
       <c r="C185" t="s">
         <v>8</v>
       </c>
       <c r="D185" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F185" t="s">
         <v>17</v>
       </c>
       <c r="G185" t="s">
-        <v>180</v>
-      </c>
-      <c r="H185" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="B186" s="18">
-        <v>3.29E-10</v>
+        <v>1.44</v>
       </c>
       <c r="C186" t="s">
         <v>8</v>
       </c>
       <c r="D186" t="s">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="F186" t="s">
         <v>17</v>
       </c>
       <c r="G186" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="187" spans="1:12">
       <c r="A187" t="s">
-        <v>146</v>
+        <v>181</v>
       </c>
       <c r="B187" s="18">
-        <v>1.44</v>
+        <v>5.1499999999999998E-5</v>
       </c>
       <c r="C187" t="s">
-        <v>8</v>
+        <v>138</v>
       </c>
       <c r="D187" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="F187" t="s">
         <v>17</v>
       </c>
       <c r="G187" t="s">
-        <v>164</v>
+        <v>197</v>
       </c>
     </row>
     <row r="188" spans="1:12">
       <c r="A188" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
       <c r="B188" s="18">
-        <v>5.1499999999999998E-5</v>
-      </c>
-      <c r="C188" t="s">
-        <v>138</v>
+        <v>0.14899999999999999</v>
       </c>
       <c r="D188" t="s">
-        <v>21</v>
+        <v>149</v>
+      </c>
+      <c r="E188" s="15" t="s">
+        <v>158</v>
       </c>
       <c r="F188" t="s">
-        <v>17</v>
-      </c>
-      <c r="G188" t="s">
-        <v>197</v>
+        <v>22</v>
       </c>
     </row>
     <row r="189" spans="1:12">
       <c r="A189" t="s">
-        <v>157</v>
+        <v>71</v>
       </c>
       <c r="B189" s="18">
-        <v>0.14899999999999999</v>
+        <v>7.67E-4</v>
       </c>
       <c r="D189" t="s">
-        <v>149</v>
-      </c>
-      <c r="E189" s="15" t="s">
-        <v>158</v>
+        <v>21</v>
+      </c>
+      <c r="E189" s="12" t="s">
+        <v>30</v>
       </c>
       <c r="F189" t="s">
         <v>22</v>
@@ -4763,10 +4757,10 @@
     </row>
     <row r="190" spans="1:12">
       <c r="A190" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="B190" s="18">
-        <v>7.67E-4</v>
+        <v>1.6299999999999999E-3</v>
       </c>
       <c r="D190" t="s">
         <v>21</v>
@@ -4780,10 +4774,10 @@
     </row>
     <row r="191" spans="1:12">
       <c r="A191" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B191" s="18">
-        <v>1.6299999999999999E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="D191" t="s">
         <v>21</v>
@@ -4797,13 +4791,13 @@
     </row>
     <row r="192" spans="1:12">
       <c r="A192" t="s">
-        <v>25</v>
+        <v>156</v>
       </c>
       <c r="B192" s="18">
-        <v>1E-3</v>
+        <v>4.7600000000000003E-2</v>
       </c>
       <c r="D192" t="s">
-        <v>21</v>
+        <v>149</v>
       </c>
       <c r="E192" s="12" t="s">
         <v>30</v>
@@ -4817,316 +4811,322 @@
         <v>156</v>
       </c>
       <c r="B193" s="18">
-        <v>4.7600000000000003E-2</v>
+        <v>0.10100000000000001</v>
       </c>
       <c r="D193" t="s">
         <v>149</v>
       </c>
-      <c r="E193" s="12" t="s">
-        <v>30</v>
+      <c r="E193" s="15" t="s">
+        <v>155</v>
       </c>
       <c r="F193" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="194" spans="1:12">
-      <c r="A194" t="s">
-        <v>156</v>
-      </c>
-      <c r="B194" s="18">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="D194" t="s">
-        <v>149</v>
-      </c>
-      <c r="E194" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="F194" t="s">
-        <v>22</v>
+    <row r="195" spans="1:12">
+      <c r="A195" t="s">
+        <v>2</v>
+      </c>
+      <c r="B195" s="13" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="196" spans="1:12">
       <c r="A196" t="s">
-        <v>2</v>
-      </c>
-      <c r="B196" s="13" t="s">
-        <v>179</v>
+        <v>6</v>
+      </c>
+      <c r="B196" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="197" spans="1:12">
       <c r="A197" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B197" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
     </row>
     <row r="198" spans="1:12">
-      <c r="A198" t="s">
-        <v>53</v>
-      </c>
-      <c r="B198" t="s">
-        <v>210</v>
+      <c r="A198" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B198" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="199" spans="1:12">
-      <c r="A199" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B199" s="12" t="s">
-        <v>214</v>
+      <c r="A199" t="s">
+        <v>7</v>
+      </c>
+      <c r="B199" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="200" spans="1:12">
       <c r="A200" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B200" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B201" t="s">
-        <v>179</v>
+        <v>21</v>
       </c>
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>13</v>
-      </c>
-      <c r="B202" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="203" spans="1:12">
       <c r="A203" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B203" t="s">
+        <v>12</v>
+      </c>
+      <c r="C203" t="s">
+        <v>7</v>
+      </c>
+      <c r="D203" t="s">
+        <v>13</v>
+      </c>
+      <c r="E203" t="s">
+        <v>19</v>
+      </c>
+      <c r="F203" t="s">
+        <v>9</v>
+      </c>
+      <c r="G203" t="s">
+        <v>14</v>
+      </c>
+      <c r="H203" t="s">
+        <v>6</v>
+      </c>
+      <c r="I203" t="s">
+        <v>18</v>
+      </c>
+      <c r="J203" t="s">
+        <v>140</v>
+      </c>
+      <c r="K203" t="s">
+        <v>141</v>
+      </c>
+      <c r="L203" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="204" spans="1:12">
       <c r="A204" t="s">
-        <v>11</v>
-      </c>
-      <c r="B204" t="s">
-        <v>12</v>
+        <v>179</v>
+      </c>
+      <c r="B204" s="18">
+        <v>1</v>
       </c>
       <c r="C204" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D204" t="s">
-        <v>13</v>
-      </c>
-      <c r="E204" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F204" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G204" t="s">
-        <v>14</v>
+        <v>179</v>
       </c>
       <c r="H204" t="s">
-        <v>6</v>
-      </c>
-      <c r="I204" t="s">
-        <v>18</v>
-      </c>
-      <c r="J204" t="s">
-        <v>140</v>
-      </c>
-      <c r="K204" t="s">
-        <v>141</v>
-      </c>
-      <c r="L204" t="s">
-        <v>142</v>
+        <v>182</v>
       </c>
     </row>
     <row r="205" spans="1:12">
       <c r="A205" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B205" s="18">
-        <v>1</v>
+        <v>4.4300000000000002E-10</v>
       </c>
       <c r="C205" t="s">
         <v>8</v>
       </c>
       <c r="D205" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F205" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G205" t="s">
-        <v>179</v>
-      </c>
-      <c r="H205" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
     </row>
     <row r="206" spans="1:12">
       <c r="A206" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="B206" s="18">
-        <v>4.4300000000000002E-10</v>
-      </c>
-      <c r="C206" t="s">
-        <v>8</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="D206" t="s">
-        <v>13</v>
+        <v>149</v>
+      </c>
+      <c r="E206" s="15" t="s">
+        <v>158</v>
       </c>
       <c r="F206" t="s">
-        <v>17</v>
-      </c>
-      <c r="G206" t="s">
-        <v>195</v>
+        <v>22</v>
       </c>
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B207" s="18">
-        <v>4.0000000000000001E-3</v>
+        <v>2.4499999999999999E-3</v>
       </c>
       <c r="D207" t="s">
         <v>149</v>
       </c>
       <c r="E207" s="15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F207" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="208" spans="1:12">
-      <c r="A208" t="s">
-        <v>156</v>
-      </c>
-      <c r="B208" s="18">
-        <v>2.4499999999999999E-3</v>
-      </c>
-      <c r="D208" t="s">
-        <v>149</v>
-      </c>
-      <c r="E208" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="F208" t="s">
-        <v>22</v>
+    <row r="209" spans="1:12">
+      <c r="A209" t="s">
+        <v>2</v>
+      </c>
+      <c r="B209" s="13" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>2</v>
-      </c>
-      <c r="B210" s="13" t="s">
-        <v>180</v>
+        <v>6</v>
+      </c>
+      <c r="B210" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="211" spans="1:12">
       <c r="A211" t="s">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="B211" t="s">
-        <v>184</v>
+        <v>211</v>
       </c>
     </row>
     <row r="212" spans="1:12">
-      <c r="A212" t="s">
-        <v>53</v>
-      </c>
-      <c r="B212" t="s">
-        <v>211</v>
+      <c r="A212" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B212" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="213" spans="1:12">
-      <c r="A213" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B213" s="12" t="s">
-        <v>214</v>
+      <c r="A213" t="s">
+        <v>7</v>
+      </c>
+      <c r="B213" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B214" t="s">
-        <v>8</v>
+        <v>180</v>
       </c>
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B215" t="s">
-        <v>180</v>
+        <v>21</v>
       </c>
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>13</v>
-      </c>
-      <c r="B216" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="217" spans="1:12">
       <c r="A217" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B217" t="s">
+        <v>12</v>
+      </c>
+      <c r="C217" t="s">
+        <v>7</v>
+      </c>
+      <c r="D217" t="s">
+        <v>13</v>
+      </c>
+      <c r="E217" t="s">
+        <v>19</v>
+      </c>
+      <c r="F217" t="s">
+        <v>9</v>
+      </c>
+      <c r="G217" t="s">
+        <v>14</v>
+      </c>
+      <c r="H217" t="s">
+        <v>6</v>
+      </c>
+      <c r="I217" t="s">
+        <v>18</v>
+      </c>
+      <c r="J217" t="s">
+        <v>140</v>
+      </c>
+      <c r="K217" t="s">
+        <v>141</v>
+      </c>
+      <c r="L217" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="218" spans="1:12">
       <c r="A218" t="s">
-        <v>11</v>
-      </c>
-      <c r="B218" t="s">
-        <v>12</v>
+        <v>180</v>
+      </c>
+      <c r="B218" s="18">
+        <v>1</v>
       </c>
       <c r="C218" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D218" t="s">
-        <v>13</v>
-      </c>
-      <c r="E218" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F218" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G218" t="s">
-        <v>14</v>
+        <v>180</v>
       </c>
       <c r="H218" t="s">
-        <v>6</v>
-      </c>
-      <c r="I218" t="s">
-        <v>18</v>
-      </c>
-      <c r="J218" t="s">
-        <v>140</v>
-      </c>
-      <c r="K218" t="s">
-        <v>141</v>
-      </c>
-      <c r="L218" t="s">
-        <v>142</v>
+        <v>185</v>
       </c>
     </row>
     <row r="219" spans="1:12">
       <c r="A219" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B219" s="18">
-        <v>1</v>
+        <v>0.91700000000000004</v>
       </c>
       <c r="C219" t="s">
         <v>8</v>
@@ -5135,24 +5135,21 @@
         <v>21</v>
       </c>
       <c r="F219" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G219" t="s">
-        <v>180</v>
-      </c>
-      <c r="H219" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>186</v>
+        <v>200</v>
       </c>
       <c r="B220" s="18">
-        <v>0.91700000000000004</v>
+        <v>0.03</v>
       </c>
       <c r="C220" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D220" t="s">
         <v>21</v>
@@ -5161,18 +5158,21 @@
         <v>17</v>
       </c>
       <c r="G220" t="s">
-        <v>193</v>
+        <v>198</v>
+      </c>
+      <c r="H220" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="221" spans="1:12">
       <c r="A221" t="s">
-        <v>200</v>
+        <v>187</v>
       </c>
       <c r="B221" s="18">
-        <v>0.03</v>
+        <v>5.2499999999999998E-2</v>
       </c>
       <c r="C221" t="s">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="D221" t="s">
         <v>21</v>
@@ -5181,49 +5181,26 @@
         <v>17</v>
       </c>
       <c r="G221" t="s">
-        <v>198</v>
-      </c>
-      <c r="H221" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="222" spans="1:12">
       <c r="A222" t="s">
-        <v>187</v>
+        <v>146</v>
       </c>
       <c r="B222" s="18">
-        <v>5.2499999999999998E-2</v>
+        <v>1.78</v>
       </c>
       <c r="C222" t="s">
         <v>8</v>
       </c>
       <c r="D222" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="F222" t="s">
         <v>17</v>
       </c>
       <c r="G222" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="223" spans="1:12">
-      <c r="A223" t="s">
-        <v>146</v>
-      </c>
-      <c r="B223" s="18">
-        <v>1.78</v>
-      </c>
-      <c r="C223" t="s">
-        <v>8</v>
-      </c>
-      <c r="D223" t="s">
-        <v>68</v>
-      </c>
-      <c r="F223" t="s">
-        <v>17</v>
-      </c>
-      <c r="G223" t="s">
         <v>164</v>
       </c>
     </row>
@@ -5235,15 +5212,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFFD7E1F-62C4-4B55-9EF4-FABFBE79AE8D}">
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.6">
+    <row r="3" spans="1:12" ht="15.75">
       <c r="A3" s="3" t="s">
         <v>66</v>
       </c>
@@ -5263,7 +5240,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6">
+    <row r="4" spans="1:12" ht="15.75">
       <c r="A4" s="3" t="s">
         <v>66</v>
       </c>
@@ -5288,7 +5265,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="15.6">
+    <row r="5" spans="1:12" ht="15.75">
       <c r="A5" s="3" t="s">
         <v>66</v>
       </c>
@@ -5360,6 +5337,29 @@
       <c r="J7" s="15"/>
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
+    </row>
+    <row r="8" spans="1:12" ht="15.75">
+      <c r="A8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8">
+        <v>0.35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" t="s">
+        <v>196</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -5369,16 +5369,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A8E48C-ECCC-42B7-B70A-16D5D4E493BD}">
   <dimension ref="A1:G34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="7"/>
-    <col min="2" max="2" width="22.44140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.5546875" style="7"/>
+    <col min="1" max="1" width="11.5703125" style="7"/>
+    <col min="2" max="2" width="22.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.5703125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5508,7 +5508,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.4">
+    <row r="9" spans="1:7" ht="15">
       <c r="B9" s="7" t="s">
         <v>99</v>
       </c>

</xml_diff>